<commit_message>
feat: deteccao de alteracoes + envio de email + workflow Actions
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,24 +430,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
@@ -452,50 +462,60 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Próxima ação do proponente</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Alterações detectadas</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Objetivo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Público-alvo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor total</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Valor por proposta</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Contato</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Próxima ação do proponente</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Ações do proponente (todas)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>PDF (URL)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Arquivo local</t>
         </is>
@@ -512,37 +532,43 @@
           <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -557,17 +583,17 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
@@ -584,37 +610,43 @@
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -629,17 +661,17 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
@@ -656,37 +688,43 @@
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>R$ 10.000,00</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
 2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
@@ -703,17 +741,17 @@
 2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
         </is>
@@ -730,37 +768,43 @@
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -774,17 +818,17 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
@@ -801,37 +845,43 @@
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -845,17 +895,17 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições.pdf</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
@@ -872,37 +922,43 @@
           <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02 a 2026-10-27: Segunda Chamada - Período de submissão das propostas (Até 17h59)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento desses TCCs por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC). As propostas devem apresentar soluções inovadoras e empreendedoras, alinhadas aos ODS da ONU e ao Plano ES 500 Anos, com potencial de impacto econômico, social e/ou ambiental no Espírito Santo.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Professores orientadores (proponentes) com vínculo estatutário ou celetista por tempo indeterminado em Instituições de Ensino Superior (IES) públicas ou privadas, reconhecidas pelo MEC e localizadas no Espírito Santo, que orientem estudantes de graduação regularmente matriculados em fase de conclusão de curso.</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02 a 2026-10-27: Segunda Chamada - Período de submissão das propostas (Até 17h59)</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes do fim do período de submissão da Primeira Chamada)
 2026-02-02 a 2026-03-30: Primeira Chamada - Período de submissão das propostas (Até 17h59)
@@ -916,17 +972,17 @@
 ?: Terceira Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O edital aceita todos os formatos de TCC definidos pelas DCNs. As propostas serão avaliadas por microrregião, com um limite de 20 projetos na primeira chamada e 10 nas subsequentes. Recursos remanescentes serão destinados por ampla concorrência. O proponente pode indicar de 3 a 5 alunos orientados por proposta. O valor da bolsa BTCC e do auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. O orientador receberá até dois auxílios para orientação. Contatos adicionais para dúvidas: suporte@fapes.es.gov.br (cadastro e validação no Acesso Cidadão), sucon@fapes.es.gov.br (assinatura de documentos no E-docs/Acesso Cidadão), contacorrente@fapes.es.gov.br (pagamento de recursos financeiros).</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
@@ -943,37 +999,43 @@
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-21: Início da contratação e submissão de documentos (A partir desta data. Inclui submissão do projeto completo no SIGFAPES, documentos para contratação, assinatura eletrônica do Termo de Outorga e Projeto Aprovado via E-Docs, e envio do e-Flow (Formulário nº 26).)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Este edital visa fomentar projetos inovadores, por meio de subvenção econômica, para fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, possuam no mínimo 3 empregados CLT na unidade capixaba (até 3 meses antes da submissão) e infraestrutura instalada. Não podem ter sido contratadas nos Editais nº 07/2024 – Programa Tecnova III e n° 10/2025 – Nova Economia Capixaba.</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 600.000,00</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, gabinete@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-21: Início da contratação e submissão de documentos (A partir desta data. Inclui submissão do projeto completo no SIGFAPES, documentos para contratação, assinatura eletrônica do Termo de Outorga e Projeto Aprovado via E-Docs, e envio do e-Flow (Formulário nº 26).)</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-04-06: Período de submissão das propostas (Até às 17h59)
 ?: Prazo para submissão de recursos administrativos (habilitação) (5 dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -982,17 +1044,17 @@
 ?: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As propostas contratadas terão prazo de execução e vigência de 24 meses, prorrogáveis por até 12 meses. As empresas classificadas e selecionadas deverão depositar 5% do valor da subvenção econômica como contrapartida financeira. O resultado da proposta, ao final da execução, deverá estar em condição de ingressar em etapas de certificação, produção e/ou comercialização. Cada proponente ou empresa poderá submeter apenas uma única proposta.</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
@@ -1009,33 +1071,39 @@
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1049,17 +1117,17 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
@@ -1076,45 +1144,51 @@
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>As diretrizes da FAPES visam apoiar a participação de pesquisadores do estado do Espírito Santo em propostas colaborativas submetidas ao programa Horizonte Europa. O objetivo é fomentar a pesquisa e inovação, permitindo que entidades brasileiras se unam a parceiros europeus e internacionais para desenvolver projetos, contribuindo para o desenvolvimento científico e tecnológico do estado.</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores (co-PIs) do estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>€ 50.000</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta. A consulta deve ser enviada para parcerias@fapes.es.gov.br.)
 ?: Submissão de propostas à FAPES (Propostas associadas às chamadas do Horizonte Europa são recebidas a qualquer momento, respeitando os prazos do Horizonte Europa. A proposta só será aceita para avaliação se a FAPES tiver sido previamente consultada.)</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Os projetos selecionados terão prazo de vigência de até 36 meses, não podendo ultrapassar a vigência do Arranjo Administrativo Horizon Europe 2021-2027. O financiamento pela FAPES está condicionado à aprovação da proposta pelo Horizonte Europa e à submissão do Acordo de Subvenção. Os recursos financeiros são oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado.</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
@@ -1131,49 +1205,55 @@
           <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>€ 40.000,00</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>€ 40.000,00</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2025-11-13: Prazo para envio de pré-propostas
 2026-04-13: Prazo para envio de propostas completas convidadas</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
@@ -1190,33 +1270,39 @@
           <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1225,17 +1311,17 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
@@ -1252,44 +1338,50 @@
           <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-30: Prazo final para registro</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-04-30: Prazo final para registro</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
@@ -1306,48 +1398,54 @@
           <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>R$ 150.000,00</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
         </is>
@@ -1364,48 +1462,54 @@
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Novo - aguardando envio</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-04-25 19:38
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1400,7 +1400,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Novo - aguardando envio</t>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: detec\u00e7\u00e3o de altera\u00e7\u00f5es por PDF separado + e-mail s\u00f3 com submiss\u00e3o e diff
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -929,18 +929,30 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 a 2026-10-27: Segunda Chamada - Período de submissão das propostas (Até 17h59)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento desses TCCs por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC). As propostas devem apresentar soluções inovadoras e empreendedoras, alinhadas aos ODS da ONU e ao Plano ES 500 Anos, com potencial de impacto econômico, social e/ou ambiental no Espírito Santo." → "Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC)."
+Público-alvo: "Professores orientadores (proponentes) com vínculo estatutário ou celetista por tempo indeterminado em Instituições de Ensino Superior (IES) públicas ou privadas, reconhecidas pelo MEC e localizadas no Espírito Santo, que orientem estudantes de graduação regularmente matriculados em fase de conclusão de curso." → "Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes."
+Contato: "editais.extensao@fapes.es.gov.br" → "editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
+Submissão (nova): Submissão de propostas (Primeira Chamada) — 2026-02-02 a 2026-03-30
+Submissão (nova): Submissão de propostas (Segunda Chamada) — 2026-09-02 a 2026-10-27
+Submissão (nova): Submissão de propostas (Terceira Chamada) — 2027-02-02 a 2027-03-30
+Submissão (removida): Primeira Chamada - Período de submissão das propostas — 2026-02-02 a 2026-03-30
+Submissão (removida): Segunda Chamada - Período de submissão das propostas — 2026-09-02 a 2026-10-27
+Submissão (removida): Terceira Chamada - Período de submissão das propostas — 2027-02-02 a 2027-03-30</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento desses TCCs por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC). As propostas devem apresentar soluções inovadoras e empreendedoras, alinhadas aos ODS da ONU e ao Plano ES 500 Anos, com potencial de impacto econômico, social e/ou ambiental no Espírito Santo.</t>
+          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Professores orientadores (proponentes) com vínculo estatutário ou celetista por tempo indeterminado em Instituições de Ensino Superior (IES) públicas ou privadas, reconhecidas pelo MEC e localizadas no Espírito Santo, que orientem estudantes de graduação regularmente matriculados em fase de conclusão de curso.</t>
+          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -955,26 +967,28 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>?: Impugnação do edital (Até 5 dias úteis antes do fim do período de submissão da Primeira Chamada)
-2026-02-02 a 2026-03-30: Primeira Chamada - Período de submissão das propostas (Até 17h59)
-?: Primeira Chamada - Prazo para interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado de seleção)
-?: Primeira Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)
-2026-09-02 a 2026-10-27: Segunda Chamada - Período de submissão das propostas (Até 17h59)
-?: Segunda Chamada - Prazo para interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado de seleção)
-?: Segunda Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)
-2027-02-02 a 2027-03-30: Terceira Chamada - Período de submissão das propostas (Até 17h59)
-?: Terceira Chamada - Prazo para interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado de seleção)
-?: Terceira Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
+          <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
+2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
+2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2026-06-23 a 2026-06-27: Prazo de contratação (Primeira Chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2026-10-20: Impugnação do Edital (Segunda Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da segunda chamada)
+2026-09-02 a 2026-10-27: Submissão de propostas (Segunda Chamada) (Até 17h59)
+2026-12-23 a 2026-12-29: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2027-01-28 a 2027-02-03: Prazo de contratação (Segunda Chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2027-03-23: Impugnação do Edital (Terceira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da terceira chamada)
+2027-02-02 a 2027-03-30: Submissão de propostas (Terceira Chamada) (Até 17h59)
+2027-05-25 a 2027-05-31: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>O edital aceita todos os formatos de TCC definidos pelas DCNs. As propostas serão avaliadas por microrregião, com um limite de 20 projetos na primeira chamada e 10 nas subsequentes. Recursos remanescentes serão destinados por ampla concorrência. O proponente pode indicar de 3 a 5 alunos orientados por proposta. O valor da bolsa BTCC e do auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. O orientador receberá até dois auxílios para orientação. Contatos adicionais para dúvidas: suporte@fapes.es.gov.br (cadastro e validação no Acesso Cidadão), sucon@fapes.es.gov.br (assinatura de documentos no E-docs/Acesso Cidadão), contacorrente@fapes.es.gov.br (pagamento de recursos financeiros).</t>
+          <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1006,18 +1020,26 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21: Início da contratação e submissão de documentos (A partir desta data. Inclui submissão do projeto completo no SIGFAPES, documentos para contratação, assinatura eletrônica do Termo de Outorga e Projeto Aprovado via E-Docs, e envio do e-Flow (Formulário nº 26).)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Este edital visa fomentar projetos inovadores, por meio de subvenção econômica, para fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado." → "O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado."
+Público-alvo: "Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, possuam no mínimo 3 empregados CLT na unidade capixaba (até 3 meses antes da submissão) e infraestrutura instalada. Não podem ter sido contratadas nos Editais nº 07/2024 – Programa Tecnova III e n° 10/2025 – Nova Economia Capixaba." → "Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes."
+Contato: "duvidas.inovacao@fapes.es.gov.br, gabinete@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br"
+Submissão (nova): Período de submissão das propostas — 2026-02-20 a 2026-05-06
+Submissão (removida): Período de submissão das propostas — 2026-02-20 a 2026-04-06</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa fomentar projetos inovadores, por meio de subvenção econômica, para fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
+          <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, possuam no mínimo 3 empregados CLT na unidade capixaba (até 3 meses antes da submissão) e infraestrutura instalada. Não podem ter sido contratadas nos Editais nº 07/2024 – Programa Tecnova III e n° 10/2025 – Nova Economia Capixaba.</t>
+          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1032,21 +1054,20 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, gabinete@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-02-20 a 2026-04-06: Período de submissão das propostas (Até às 17h59)
-?: Prazo para submissão de recursos administrativos (habilitação) (5 dias úteis a partir da publicação do resultado de habilitação das propostas)
-?: Prazo para submissão de recursos administrativos (avaliação de mérito) (5 dias úteis a partir da publicação do resultado preliminar de avaliação de mérito)
-2026-07-21: Início da contratação e submissão de documentos (A partir desta data. Inclui submissão do projeto completo no SIGFAPES, documentos para contratação, assinatura eletrônica do Termo de Outorga e Projeto Aprovado via E-Docs, e envio do e-Flow (Formulário nº 26).)
-?: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga)</t>
+          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
+2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
+2026-07-25 a 2026-07-31: Prazo para submissão de recursos administrativos (mérito) (5 (cinco) dias úteis a partir da publicação do resultado preliminar de avaliação de mérito)
+2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>As propostas contratadas terão prazo de execução e vigência de 24 meses, prorrogáveis por até 12 meses. As empresas classificadas e selecionadas deverão depositar 5% do valor da subvenção econômica como contrapartida financeira. O resultado da proposta, ao final da execução, deverá estar em condição de ingressar em etapas de certificação, produção e/ou comercialização. Cada proponente ou empresa poderá submeter apenas uma única proposta.</t>
+          <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1150,21 +1171,29 @@
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "As diretrizes da FAPES visam apoiar a participação de pesquisadores do estado do Espírito Santo em propostas colaborativas submetidas ao programa Horizonte Europa. O objetivo é fomentar a pesquisa e inovação, permitindo que entidades brasileiras se unam a parceiros europeus e internacionais para desenvolver projetos, contribuindo para o desenvolvimento científico e tecnológico do estado." → "Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais."
+Público-alvo: "Pesquisadores (co-PIs) do estado do Espírito Santo." → "Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa."
+Valor por proposta: "€ 50.000" → "€ 25.000,00 por ano de projeto"
+Submissão (nova): Submissão da Proposta à FAPES — ? a ?
+Submissão (removida): Submissão de propostas à FAPES — ? a ?</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>As diretrizes da FAPES visam apoiar a participação de pesquisadores do estado do Espírito Santo em propostas colaborativas submetidas ao programa Horizonte Europa. O objetivo é fomentar a pesquisa e inovação, permitindo que entidades brasileiras se unam a parceiros europeus e internacionais para desenvolver projetos, contribuindo para o desenvolvimento científico e tecnológico do estado.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores (co-PIs) do estado do Espírito Santo.</t>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>€ 50.000</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1174,13 +1203,14 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>?: Consulta de Elegibilidade (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta. A consulta deve ser enviada para parcerias@fapes.es.gov.br.)
-?: Submissão de propostas à FAPES (Propostas associadas às chamadas do Horizonte Europa são recebidas a qualquer momento, respeitando os prazos do Horizonte Europa. A proposta só será aceita para avaliação se a FAPES tiver sido previamente consultada.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Os projetos selecionados terão prazo de vigência de até 36 meses, não podendo ultrapassar a vigência do Arranjo Administrativo Horizon Europe 2021-2027. O financiamento pela FAPES está condicionado à aprovação da proposta pelo Horizonte Europa e à submissão do Acordo de Subvenção. Os recursos financeiros são oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-04-25 20:33
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,9 +524,9 @@
           <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -610,9 +602,9 @@
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -688,9 +680,9 @@
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -768,9 +760,9 @@
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -845,9 +837,9 @@
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -922,25 +914,25 @@
           <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 a 2026-10-27: Segunda Chamada - Período de submissão das propostas (Até 17h59)</t>
+          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento desses TCCs por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC). As propostas devem apresentar soluções inovadoras e empreendedoras, alinhadas aos ODS da ONU e ao Plano ES 500 Anos, com potencial de impacto econômico, social e/ou ambiental no Espírito Santo.</t>
+          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Professores orientadores (proponentes) com vínculo estatutário ou celetista por tempo indeterminado em Instituições de Ensino Superior (IES) públicas ou privadas, reconhecidas pelo MEC e localizadas no Espírito Santo, que orientem estudantes de graduação regularmente matriculados em fase de conclusão de curso.</t>
+          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -955,26 +947,28 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>?: Impugnação do edital (Até 5 dias úteis antes do fim do período de submissão da Primeira Chamada)
-2026-02-02 a 2026-03-30: Primeira Chamada - Período de submissão das propostas (Até 17h59)
-?: Primeira Chamada - Prazo para interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado de seleção)
-?: Primeira Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)
-2026-09-02 a 2026-10-27: Segunda Chamada - Período de submissão das propostas (Até 17h59)
-?: Segunda Chamada - Prazo para interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado de seleção)
-?: Segunda Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)
-2027-02-02 a 2027-03-30: Terceira Chamada - Período de submissão das propostas (Até 17h59)
-?: Terceira Chamada - Prazo para interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado de seleção)
-?: Terceira Chamada - Prazo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
+          <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
+2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
+2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2026-06-23 a 2026-06-27: Prazo de contratação (Primeira Chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2026-10-20: Impugnação do Edital (Segunda Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da segunda chamada)
+2026-09-02 a 2026-10-27: Submissão de propostas (Segunda Chamada) (Até 17h59)
+2026-12-23 a 2026-12-29: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2027-01-28 a 2027-02-03: Prazo de contratação (Segunda Chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2027-03-23: Impugnação do Edital (Terceira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da terceira chamada)
+2027-02-02 a 2027-03-30: Submissão de propostas (Terceira Chamada) (Até 17h59)
+2027-05-25 a 2027-05-31: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>O edital aceita todos os formatos de TCC definidos pelas DCNs. As propostas serão avaliadas por microrregião, com um limite de 20 projetos na primeira chamada e 10 nas subsequentes. Recursos remanescentes serão destinados por ampla concorrência. O proponente pode indicar de 3 a 5 alunos orientados por proposta. O valor da bolsa BTCC e do auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. O orientador receberá até dois auxílios para orientação. Contatos adicionais para dúvidas: suporte@fapes.es.gov.br (cadastro e validação no Acesso Cidadão), sucon@fapes.es.gov.br (assinatura de documentos no E-docs/Acesso Cidadão), contacorrente@fapes.es.gov.br (pagamento de recursos financeiros).</t>
+          <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -999,25 +993,25 @@
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21: Início da contratação e submissão de documentos (A partir desta data. Inclui submissão do projeto completo no SIGFAPES, documentos para contratação, assinatura eletrônica do Termo de Outorga e Projeto Aprovado via E-Docs, e envio do e-Flow (Formulário nº 26).)</t>
+          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa fomentar projetos inovadores, por meio de subvenção econômica, para fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
+          <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, possuam no mínimo 3 empregados CLT na unidade capixaba (até 3 meses antes da submissão) e infraestrutura instalada. Não podem ter sido contratadas nos Editais nº 07/2024 – Programa Tecnova III e n° 10/2025 – Nova Economia Capixaba.</t>
+          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1032,21 +1026,20 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, gabinete@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-02-20 a 2026-04-06: Período de submissão das propostas (Até às 17h59)
-?: Prazo para submissão de recursos administrativos (habilitação) (5 dias úteis a partir da publicação do resultado de habilitação das propostas)
-?: Prazo para submissão de recursos administrativos (avaliação de mérito) (5 dias úteis a partir da publicação do resultado preliminar de avaliação de mérito)
-2026-07-21: Início da contratação e submissão de documentos (A partir desta data. Inclui submissão do projeto completo no SIGFAPES, documentos para contratação, assinatura eletrônica do Termo de Outorga e Projeto Aprovado via E-Docs, e envio do e-Flow (Formulário nº 26).)
-?: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga)</t>
+          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
+2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
+2026-07-25 a 2026-07-31: Prazo para submissão de recursos administrativos (mérito) (5 (cinco) dias úteis a partir da publicação do resultado preliminar de avaliação de mérito)
+2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>As propostas contratadas terão prazo de execução e vigência de 24 meses, prorrogáveis por até 12 meses. As empresas classificadas e selecionadas deverão depositar 5% do valor da subvenção econômica como contrapartida financeira. O resultado da proposta, ao final da execução, deverá estar em condição de ingressar em etapas de certificação, produção e/ou comercialização. Cada proponente ou empresa poderá submeter apenas uma única proposta.</t>
+          <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1071,9 +1064,9 @@
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1144,27 +1137,27 @@
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>As diretrizes da FAPES visam apoiar a participação de pesquisadores do estado do Espírito Santo em propostas colaborativas submetidas ao programa Horizonte Europa. O objetivo é fomentar a pesquisa e inovação, permitindo que entidades brasileiras se unam a parceiros europeus e internacionais para desenvolver projetos, contribuindo para o desenvolvimento científico e tecnológico do estado.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores (co-PIs) do estado do Espírito Santo.</t>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>€ 50.000</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1174,13 +1167,14 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>?: Consulta de Elegibilidade (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta. A consulta deve ser enviada para parcerias@fapes.es.gov.br.)
-?: Submissão de propostas à FAPES (Propostas associadas às chamadas do Horizonte Europa são recebidas a qualquer momento, respeitando os prazos do Horizonte Europa. A proposta só será aceita para avaliação se a FAPES tiver sido previamente consultada.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Os projetos selecionados terão prazo de vigência de até 36 meses, não podendo ultrapassar a vigência do Arranjo Administrativo Horizon Europe 2021-2027. O financiamento pela FAPES está condicionado à aprovação da proposta pelo Horizonte Europa e à submissão do Acordo de Subvenção. Os recursos financeiros são oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1205,9 +1199,9 @@
           <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1270,9 +1264,9 @@
           <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1338,9 +1332,9 @@
           <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1398,9 +1392,9 @@
           <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1462,9 +1456,9 @@
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-04-25 21:01
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -524,9 +532,9 @@
           <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -602,9 +610,9 @@
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -680,9 +688,9 @@
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -760,9 +768,9 @@
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -837,9 +845,9 @@
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -914,9 +922,9 @@
           <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -993,9 +1001,9 @@
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1064,9 +1072,9 @@
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1137,9 +1145,9 @@
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1199,9 +1207,9 @@
           <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1264,9 +1272,9 @@
           <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1332,9 +1340,9 @@
           <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1392,9 +1400,9 @@
           <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1456,9 +1464,9 @@
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 25/04/2026</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-04-26 08:19
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,9 +524,9 @@
           <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -610,9 +602,9 @@
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -688,9 +680,9 @@
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -768,9 +760,9 @@
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -845,9 +837,9 @@
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -922,9 +914,9 @@
           <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1001,9 +993,9 @@
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1072,9 +1064,9 @@
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
@@ -1145,9 +1137,9 @@
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
@@ -1207,9 +1199,9 @@
           <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
@@ -1272,9 +1264,9 @@
           <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1340,9 +1332,9 @@
           <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1400,9 +1392,9 @@
           <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1464,9 +1456,9 @@
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 25/04/2026</t>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-04-29 08:38
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -516,51 +524,120 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 09/2026 - BOLSAS DE ESTÁGIO DOUTORADO SANDUÍCHE</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 29/04/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)</t>
+          <t>2026-04-28 a 2026-06-29: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas.)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Apoiar alunos de doutorado regularmente matriculados em programas de pós-graduação do Espírito Santo para a realização de estágio de pesquisa no exterior. O objetivo é proporcionar aprofundamento teórico, coleta e/ou tratamento de dados, ou desenvolvimento parcial da tese, visando ao intercâmbio científico e ao aprimoramento da qualificação acadêmica, com a concessão de bolsa na modalidade Doutorado Sanduíche.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Alunos de doutorado regularmente matriculados em Programas de Pós-graduação stricto sensu, recomendados pela CAPES e vinculados a instituições de ensino superior e/ou pesquisa (IES/P) públicas ou privadas no Espírito Santo. Os proponentes devem ser brasileiros ou estrangeiros com autorização de residência, residentes no Espírito Santo, sem título de doutor, com currículo Lattes atualizado, cursando entre o 13º e o 42º mês do doutorado (com pelo menos seis meses restantes para a conclusão após o estágio no exterior), com proficiência na língua da instituição de destino, e com anuência do orientador, supervisor no exterior, e coordenador do PPG. Não devem ter realizado mobilidade acadêmica no exterior com auxílio da Fapes nos últimos 12 meses, nem ter sido contemplados com bolsa de Doutorado Sanduíche da Fapes, Capes ou CNPq anteriormente, e devem estar adimplentes junto à Fapes.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28 a 2026-06-29: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas.)
+2026-04-28 a 2026-07-02: Prazo para dúvidas e informações (Até 2 dias úteis antecedentes ao término da submissão das propostas.)
+2026-07-06: Submissão das propostas (Até as 17h59.)
+2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)
+2026-10-09 a 2026-10-16: Prazo para recurso (classificação) (Até 5 dias úteis após a divulgação do resultado preliminar de classificação.)
+2026-11-01: Contratação dos projetos (Inclui a assinatura eletrônica do Termo de Outorga e o envio de documentos pessoais, com datas a serem divulgadas no resultado homologado.)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>A duração do estágio de doutorado sanduíche é de, no mínimo, 6 e, no máximo, 12 meses. Os valores das bolsas mensais variam de US$ 1.100,00 a US$ 1.800,00, dependendo do país de destino. O auxílio instalação é equivalente a uma mensalidade da bolsa. O auxílio seguro-saúde é limitado a US$ 90,00 por mês de bolsa, e o auxílio deslocamento é limitado a R$ 12.000,00. A conversão da moeda estrangeira (dólar) ocorre pelo câmbio oficial na data de aprovação do Resultado de Classificação. Taxas administrativas, acadêmicas (tuition &amp; fees), de bancada (bench fees) e adicional dependente não são cobertas. Não é permitida a alteração da instituição de destino ou do supervisor após a submissão da proposta. O prazo de vigência do instrumento de contratação é de 16 meses, improrrogáveis, e o proponente deve realizar o deslocamento dentro desse período. As atividades devem ser realizadas presencialmente na instituição de destino. Para o pagamento integral da mensalidade, o bolsista deve ter executado as atividades por no mínimo 16 dias no mês. O beneficiário tem 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. A existência de inadimplência do proponente com a Fapes ou com as Fazendas Federal, Estadual e Municipal e a Justiça Trabalhista constitui fator impeditivo para contratação. Para a assinatura eletrônica do Termo de Outorga, o proponente e o gestor institucional da IES/P devem ter cadastro ativo no portal 'Acesso Cidadão'.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL%20FAPES%20N°%2009.2026%20-%20BDS.pdf</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_No_09_2026_-_BOLSAS_DE_ESTÁGIO_DOUTORADO_SANDUÍCHE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -575,70 +652,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -653,70 +730,70 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 10.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
 2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
@@ -733,70 +810,70 @@
 2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -810,70 +887,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -887,70 +964,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
 2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
@@ -966,70 +1043,70 @@
 2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 600.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
 2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -1037,66 +1114,66 @@
 2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1110,146 +1187,81 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1273,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1269,34 +1281,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1305,79 +1382,19 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1406,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
+          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1399,49 +1416,45 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+          <t>2026-04-30: Prazo final para registro</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
+          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
+          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>global@fapes.es.gov.br</t>
+          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+          <t>2026-04-30: Prazo final para registro</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
+          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
+          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1466,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1463,47 +1476,111 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-04-30 08:37
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -532,9 +532,9 @@
           <t>EDITAL FAPES Nº 09/2026 - BOLSAS DE ESTÁGIO DOUTORADO SANDUÍCHE</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 29/04/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1062,51 +1062,122 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Extensão</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 30/04/2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)</t>
+          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 60.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
+?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
+?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
+?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 600.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
 2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -1114,66 +1185,66 @@
 2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1187,146 +1258,81 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1344,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1346,34 +1352,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1382,79 +1453,19 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1477,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
+          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1476,49 +1487,45 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+          <t>2026-04-30: Prazo final para registro</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
+          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
+          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>global@fapes.es.gov.br</t>
+          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+          <t>2026-04-30: Prazo final para registro</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
+          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
+          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1537,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1540,47 +1547,111 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-01 08:30
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)</t>
+          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -1070,9 +1070,9 @@
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 30/04/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1277,127 +1277,139 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+          <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 01/05/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30: Prazo para impugnação do edital (1ª chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada.)</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores, com o objetivo de transformar ideias inovadoras em empreendimentos sustentáveis e fortalecer micro e pequenas empresas de base tecnológica no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>R$ 10.662.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>R$ 355.400,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília).)
+2026-06-30: Prazo para impugnação do edital (1ª chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada.)
+?: Prazo para recursos administrativos de habilitação (1ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar de habilitação.)
+?: Prazo para recursos administrativos de mérito (1ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar da avaliação de mérito e apresentação oral.)
+2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h (horário de Brasília).)
+2026-10-27 a 2026-11-03: Processo de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado, incluindo constituição de empresa, atualização documental, assinatura do Termo de Outorga e envio do e-Flow de registro de documentação.)
+?: Prazo para recursos administrativos de habilitação (2ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar de habilitação.)
+?: Prazo para recursos administrativos de mérito (2ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar da avaliação de mérito e apresentação oral.)
+2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado, incluindo constituição de empresa, atualização documental, assinatura do Termo de Outorga e envio do e-Flow de registro de documentação.)
+?: Contratação de propostas suplentes (Período a ser definido, se aplicável.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações publicadas no site da FAPES. O prazo de execução dos projetos será de 24 meses, podendo ser prorrogado por no máximo 12 meses. O edital poderá ser suspenso, revogado ou anulado, no todo ou em parte, por motivo de interesse público ou exigência legal, sem que isso implique direito a indenização ou reclamação de qualquer natureza. Os casos omissos serão resolvidos pela Diretoria Executiva da FAPES.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_10-2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1421,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1417,34 +1429,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1453,79 +1530,19 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-30: Prazo final para registro</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1554,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
+          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1545,51 +1562,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
+          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
+          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+      <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>global@fapes.es.gov.br</t>
+          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+          <t>2026-04-30: Prazo final para registro</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
+          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
+          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1610,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1609,49 +1618,109 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
         </is>
       </c>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-02 08:20
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1285,9 +1277,9 @@
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 01/05/2026</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-05 08:33
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA OCEAN 2 CRA - BELMONT FORUM</t>
+          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1554,165 +1554,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Este edital, parte da iniciativa OCEAN 2 CRA do Belmont Forum, visa apoiar pesquisas transdisciplinares que abordem desafios globais do oceano e contribuam para a Década da Ciência Oceânica para o Desenvolvimento Sustentável. Serão financiados projetos com duração de 36 meses, focados em conservação da biodiversidade, soluções baseadas na natureza, integração oceano-biodiversidade-clima, e governança oceânica e ética para a sustentabilidade, visando o bem-estar da natureza e humano. As propostas devem focar em pelo menos uma das três áreas-chave especificadas.</t>
+          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores vinculados a instituições de pesquisa do estado do Espírito Santo, Brasil, que participem de consórcios de pesquisa transdisciplinares e internacionais, conforme as diretrizes do Belmont Forum e as regras das agências de fomento participantes.</t>
+          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>USD 20.000,00</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>larisse.faroni@belmontforum.org, info@belmontforum.org</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30: Prazo final para registro</t>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Os projetos aprovados terão duração esperada de 36 meses e deverão envolver consórcios de pesquisa com participantes de múltiplos países e disciplinas, incluindo parceiros sociais. As propostas devem focar em pelo menos uma das seguintes áreas-chave: Conservação da Biodiversidade e Soluções Baseadas na Natureza; Integração Oceano-Biodiversidade-Clima; Futuros da Natureza, Governança Oceânica e Ética para a Sustentabilidade. Organizações de financiamento de diversos países e algumas organizações não governamentais concordaram provisoriamente em apoiar esta chamada. Para se manter atualizado, é recomendado juntar-se à lista de e-mails ou visitar o site e redes sociais do Belmont Forum. Os documentos da chamada incluem: Chamada para Propostas (disponível em inglês, francês, português e espanhol), Formulário de Registro e Instruções, e Ferramenta de Comparação de Anexos. As candidaturas são aceitas em vários idiomas através da plataforma BFgo.org. O Secretariado do Belmont Forum é hospedado pelo Inter-American Institute for Global Change Research (IAI) no Panamá.</t>
+          <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ocean%202%20–%20Towards%20the%20Ocean%20We%20Want_%20Biodiversity%20and%20Ecosystem%20Sustainability%20for%20Nature%20and%20Human%20Well-being%20-%20Belmont%20Forum.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_OCEAN_2_CRA_-_BELMONT_FORUM.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONJUNTA CONICET 2026 - RESISTÊNCIA ANTIMICROBIANA (RAM)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>O programa visa planejar e implementar projetos de pesquisa e transferência de conhecimento relacionados à Resistência Antimicrobiana (RAM), no contexto da produção intensiva de animais para consumo humano na Argentina, Brasil, Paraguai e Uruguai. Os projetos devem abordar diversos aspectos da RAM, promovendo a integração e o fortalecimento das capacidades regionais, além de incentivar a participação intersetorial entre cientistas, produtores e órgãos reguladores.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores vinculados a Instituições de Ensino Superior e Pesquisa (públicas ou privadas sem fins lucrativos) sediadas no estado do Espírito Santo, que atendam aos critérios de elegibilidade da modalidade Auxílio à Pesquisa Regular (Instrução de Serviços № 082/2025). Cada pesquisador pode participar de, no máximo, 2 propostas e ser Pesquisador Responsável/Coordenador em apenas uma delas.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>global@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-01 a 2026-04-30: Submissão de propostas (Para a FAPES via SIGFAPES (www.sigfapes.es.gov.br), até as 23:59h GMT-3. Propostas devem estar em português ou inglês.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>A Chamada é uma iniciativa conjunta da FAPES, FAPESP, ANII, CONACYT e CONICET, com apoio do Centro de Pesquisas para o Desenvolvimento (IDRC). O foco é a Resistência Antimicrobiana (RAM) na produção intensiva de animais para consumo humano. As propostas devem incluir grupos de pesquisa de instituições localizadas em pelo menos dois dos territórios de abrangência das agências participantes (Argentina, Brasil - Espírito Santo e São Paulo, Paraguai e Uruguai). Serão financiados até 5 projetos no total, sendo que a FAPES financiará até 2 projetos. As propostas devem abordar um ou mais dos eixos temáticos listados no Anexo 1. Há possibilidade de financiamento adicional (USD 10.000) para colaborações com grupos de países da América Latina e Caribe receptores de Ajuda Oficial ao Desenvolvimento não contemplados pelas agências participantes.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada%20de%20Propostas%20Conjuntas%20-%20FAPES-FAPESP-ANII%20CONACYT%20CONICET.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONJUNTA_CONICET_2026_-_RESISTÊNCIA_ANTIMICROBIANA_(RAM).pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>USD 20.000,00</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-08 09:11
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1277,25 +1285,33 @@
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 08/05/2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Prazo para impugnação do edital (1ª chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores, com o objetivo de transformar ideias inovadoras em empreendimentos sustentáveis e fortalecer micro e pequenas empresas de base tecnológica no Espírito Santo." → "Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica."
+Público-alvo: "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras." → "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba."
+Contato: "duvidas.inovacao@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
+Submissão (nova): Abertura de empresa e atualização documental (1ª chamada) — 2026-10-27 a 2026-11-03
+Submissão (nova): Abertura de empresa e atualização documental (2ª chamada) — 2027-04-27 a 2027-05-03</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores, com o objetivo de transformar ideias inovadoras em empreendimentos sustentáveis e fortalecer micro e pequenas empresas de base tecnológica no Espírito Santo.</t>
+          <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras.</t>
+          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1310,31 +1326,40 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília).)
-2026-06-30: Prazo para impugnação do edital (1ª chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada.)
-?: Prazo para recursos administrativos de habilitação (1ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar de habilitação.)
-?: Prazo para recursos administrativos de mérito (1ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar da avaliação de mérito e apresentação oral.)
-2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h (horário de Brasília).)
-2026-10-27 a 2026-11-03: Processo de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado, incluindo constituição de empresa, atualização documental, assinatura do Termo de Outorga e envio do e-Flow de registro de documentação.)
-?: Prazo para recursos administrativos de habilitação (2ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar de habilitação.)
-?: Prazo para recursos administrativos de mérito (2ª chamada) (Prazo de 5 dias úteis a partir da publicação do resultado preliminar da avaliação de mérito e apresentação oral.)
-2027-04-27 a 2027-05-03: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado, incluindo constituição de empresa, atualização documental, assinatura do Termo de Outorga e envio do e-Flow de registro de documentação.)
-?: Contratação de propostas suplentes (Período a ser definido, se aplicável.)</t>
+          <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
+2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
+2026-07-31 a 2026-08-06: Prazo para recursos administrativos da habilitação (1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+2026-10-02 a 2026-10-08: Prazo para recursos administrativos da avaliação de mérito (1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
+2026-10-27 a 2026-11-03: Período de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2026-10-27 a 2026-11-03: Abertura de empresa e atualização documental (1ª chamada) (Para propostas aprovadas sem empresas constituídas, até as 17h00min)
+2026-10-27 a 2026-11-03: Atualização documental no SIGFAPES (1ª chamada) (Envio de documentos pessoais, até as 17h00min)
+2026-10-27 a 2026-11-03: Assinatura do Termo de Outorga e Projeto Aprovado (1ª chamada) (Eletronicamente via E-docs, até as 17h00min)
+2026-11-03: Envio do e-Flow (Formulário nº 25) e disponibilização de documentos no SIGFAPES (1ª chamada) (Até as 17h00min)
+2026-11-04: Período de contratação de suplentes (1ª chamada) (Se aplicável, até as 17h00min)
+2027-01-08 a 2027-01-14: Prazo para recursos administrativos da habilitação (2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+2027-03-19 a 2027-03-25: Prazo para recursos administrativos da avaliação de mérito (2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+2027-04-27 a 2027-05-03: Período de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2027-04-27 a 2027-05-03: Abertura de empresa e atualização documental (2ª chamada) (Para propostas aprovadas sem empresas constituídas, até as 17h00min)
+2027-04-27 a 2027-05-03: Atualização documental no SIGFAPES (2ª chamada) (Envio de documentos pessoais, até as 17h00min)
+2027-04-27 a 2027-05-03: Assinatura do Termo de Outorga e Projeto Aprovado (2ª chamada) (Eletronicamente via E-docs, até as 17h00min)
+2027-05-03: Envio do e-Flow (Formulário nº 25) e disponibilização de documentos no SIGFAPES (2ª chamada) (Até as 17h00min)
+2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações publicadas no site da FAPES. O prazo de execução dos projetos será de 24 meses, podendo ser prorrogado por no máximo 12 meses. O edital poderá ser suspenso, revogado ou anulado, no todo ou em parte, por motivo de interesse público ou exigência legal, sem que isso implique direito a indenização ou reclamação de qualquer natureza. Os casos omissos serão resolvidos pela Diretoria Executiva da FAPES.</t>
+          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_10-2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-12 08:43
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -598,38 +598,38 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 12/05/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)</t>
+          <t>2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
+          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.500.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>US$ 2.700,00</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -639,44 +639,48 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
-2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
-2026-02-06 a 2026-03-09: Período de submissão (1ª Chamada) (eventos com início entre 01/05/2026 a 31/07/2026, até as 17h59)
-2026-03-07: Prazo para envio de dúvidas (1ª Chamada) (até 2 dias antes do prazo final de submissão da 1ª Chamada)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 1ª Chamada)
-2026-03-17 a 2026-04-24: Período de submissão (2ª Chamada) (eventos com início entre 01/08/2026 a 31/12/2026)
-2026-04-22: Prazo para envio de dúvidas (2ª Chamada) (até 2 dias antes do prazo final de submissão da 2ª Chamada)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)
-2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)
-2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
+          <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
+2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
+?: Interposição de recursos - 1ª Chamada (5 dias úteis após a publicação do resultado preliminar)
+2026-04-30: Contratação / Assinatura do TO e envio de documentos - 1ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
+2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)
+?: Interposição de recursos - 2ª Chamada (5 dias úteis após a publicação do resultado preliminar)
+2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
+2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)
+?: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar)
+2026-10-30: Contratação / Assinatura do TO e envio de documentos - 3ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
+2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59)
+?: Interposição de recursos - 4ª Chamada (5 dias úteis após a publicação do resultado preliminar)
+2026-12-30: Contratação / Assinatura do TO e envio de documentos - 4ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
+?: Informar dados da conta bancária (Até 30 dias a partir do início da vigência do TO (publicação no DIO-ES).)
+?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
+          <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Extensão</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -686,348 +690,36 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
+          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
+          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
+          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.500.000,00</t>
+          <t>R$ 1.600.000,00</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
+          <t>R$ 11.000,00</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
-2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
-2026-03-07: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 1ª chamada)
-2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Eventos com início entre 01/08/2026 a 31/12/2026)
-2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 2ª chamada)
-2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)
-2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)
-2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>R$ 10.000,00</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
-2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada) (Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-04-22: Prazo final para envio de dúvidas (2ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada) (Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-08-13: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas da última chamada.)
-2026-08-18: Prazo final para envio de dúvidas (3ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>US$ 2.600,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
-2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
-2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-03-17 a 2026-04-24: Submissão de propostas (2ª Chamada) (Para visitas com início entre 01/08/2026 a 31/12/2026.)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
-2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
-2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)
-2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
-2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
-2026-03-04 a 2026-04-09: Submissão de propostas (Até as 17:59h. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
-2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
-?: Contratação e assinatura do Termo de Outorga (Até 30 dias após a publicação do resultado final homologado. Período específico de assinatura será definido após a homologação.)
-?: Prazo para informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga)
-?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Extensão</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 1.600.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 11.000,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
 2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
@@ -1043,70 +735,70 @@
 2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1114,70 +806,70 @@
 ?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 600.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
 2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -1185,66 +877,66 @@
 2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1258,78 +950,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 11/05/2026</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Fomentar o empreendedorismo inovador por meio de projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou de processos inovadores, com o objetivo de transformar ideias inovadoras em empreendimentos sustentáveis e fortalecer micro e pequenas empresas de base tecnológica no Espírito Santo." → "Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica."
-Público-alvo: "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras." → "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba."
-Contato: "duvidas.inovacao@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
-Submissão (nova): Abertura de empresa e atualização documental (1ª chamada) — 2026-10-27 a 2026-11-03
-Submissão (nova): Abertura de empresa e atualização documental (2ª chamada) — 2027-04-27 a 2027-05-03</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1352,193 +1036,193 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>€ 40.000,00</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>€ 40.000,00</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2025-11-13: Prazo para envio de pré-propostas
 2026-04-13: Prazo para envio de propostas completas convidadas</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1547,81 +1231,81 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-13 08:46
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -601,9 +593,9 @@
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 12/05/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-14 08:39
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1052,122 +1060,117 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 14/05/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1182,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1187,34 +1190,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1223,81 +1291,81 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-15 08:41
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1063,9 +1055,9 @@
           <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 14/05/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-16 08:26
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -585,51 +593,119 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 13/2026  - PROGRAMA INSTITUCIONAL DE BOLSAS DE INICIAÇÃO CIENTÍFICA, TECNOLÓGICA E DE INOVAÇÃO DO ESPÍRITO SANTO (PIBICES 2026/2027)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 16/05/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)</t>
+          <t>2026-06-16: Impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>O Programa Institucional de Bolsas de Iniciação Científica, Tecnológica e de Inovação do Estado do Espírito Santo (PIBICES) visa fomentar a participação de estudantes de graduação em atividades sistemáticas de pesquisa científica, desenvolvimento tecnológico e inovação. O edital busca fortalecer o sistema capixaba de pesquisa e a formação de recursos humanos qualificados, contribuindo para a ampliação da cultura científica e a produção de conhecimento alinhada às demandas da sociedade. Serão concedidas cotas institucionais de bolsas para Programas Institucionais de Bolsas de Iniciação Científica, Tecnológica e de Inovação (PIBICTI) em Instituições de Ensino Superior e/ou Pesquisa.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Coordenadores Institucionais de Programas de Bolsas de Iniciação Científica, Tecnológica e de Inovação (PIBICTI) vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo, que sejam pesquisadores/docentes com título de mestre ou doutor e vínculo empregatício indeterminado com a IES/P.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>R$ 8.640.000,00</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16: Impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
+2026-06-23: Submissão das propostas (até as 17h59 (horário de Brasília))
+?: Interposição de recursos (habilitação) (até 5 dias úteis após a divulgação do resultado preliminar)
+2026-08-03: Contratação dos projetos
+?: Indicação dos bolsistas (a partir do início de vigência do Termo de Outorga)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Serão disponibilizadas 800 bolsas de Iniciação Científica e Tecnológica (ICT). Cada bolsa terá duração mínima de 4 e máxima de 12 meses, com valor mensal atual de R$ 900,00. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações de atividades, utilizando a citação padrão fornecida no edital. A Fapes pode alterar datas e prazos do cronograma ou reabrir prazos em casos de força maior ou falhas comprovadas nos sistemas.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20PIBICES%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_No_13_2026_-_PROGRAMA_INSTITUCIONAL_DE_BOLSAS_DE_INICIAÇÃO_CIENTÍFICA,_TECNOLÓGICA_E_DE_INOVAÇÃO_DO_ESPÍRITO_SANTO_(PIBICES_2026_2027).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -648,70 +724,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
 2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
@@ -727,70 +803,70 @@
 2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -798,70 +874,70 @@
 ?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 600.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
 2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -869,66 +945,66 @@
 2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -942,70 +1018,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1028,79 +1104,19 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1112,7 +1128,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1120,114 +1136,109 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1250,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1247,34 +1258,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1283,81 +1359,81 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-17 08:29
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -601,9 +593,9 @@
           <t>EDITAL FAPES Nº 13/2026  - PROGRAMA INSTITUCIONAL DE BOLSAS DE INICIAÇÃO CIENTÍFICA, TECNOLÓGICA E DE INOVAÇÃO DO ESPÍRITO SANTO (PIBICES 2026/2027)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 16/05/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-21 09:08
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -735,12 +735,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
+          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -750,186 +750,36 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
+          <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
+          <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
+          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>R$ 1.600.000,00</t>
+          <t>R$ 12.000.000,00</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>R$ 11.000,00</t>
+          <t>R$ 600.000,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
-2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
-2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
-2026-06-23 a 2026-06-27: Prazo de contratação (Primeira Chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2026-10-20: Impugnação do Edital (Segunda Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da segunda chamada)
-2026-09-02 a 2026-10-27: Submissão de propostas (Segunda Chamada) (Até 17h59)
-2026-12-23 a 2026-12-29: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
-2027-01-28 a 2027-02-03: Prazo de contratação (Segunda Chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2027-03-23: Impugnação do Edital (Terceira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da terceira chamada)
-2027-02-02 a 2027-03-30: Submissão de propostas (Terceira Chamada) (Até 17h59)
-2027-05-25 a 2027-05-31: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
-2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Extensão</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 60.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
-?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
-?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
-?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 12.000.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 600.000,00</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
 2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -937,66 +787,66 @@
 2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1010,70 +860,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1096,19 +946,141 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>€ 25.000,00 por ano de projeto</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1092,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1128,47 +1100,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1157,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1188,161 +1165,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
+          <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>32.045.000 Euro</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>32.045.000 Euro</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1351,81 +1201,81 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-22 08:59
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -735,51 +743,201 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Extensão</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
+          <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
+          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
+          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.600.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 11.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
+2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
+2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2026-06-23 a 2026-06-27: Prazo de contratação (Primeira Chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2026-10-20: Impugnação do Edital (Segunda Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da segunda chamada)
+2026-09-02 a 2026-10-27: Submissão de propostas (Segunda Chamada) (Até 17h59)
+2026-12-23 a 2026-12-29: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2027-01-28 a 2027-02-03: Prazo de contratação (Segunda Chamada) (Até 5 dias úteis da publicação do resultado homologado)
+2027-03-23: Impugnação do Edital (Terceira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da terceira chamada)
+2027-02-02 a 2027-03-30: Submissão de propostas (Terceira Chamada) (Até 17h59)
+2027-05-25 a 2027-05-31: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
+2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Extensão</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 60.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
+?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
+?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
+?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 600.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
 2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
@@ -787,66 +945,66 @@
 2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -860,70 +1018,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -946,253 +1104,326 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 22/05/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.500.000,00</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>R$ 30.000,00</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
+?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
+2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)
+2026-09-21 a 2026-09-30: Apresentação do pitch (A partir de 21/09/2026)
+?: Prazo para recurso administrativo (Fase 2) (Até 5 dias úteis após divulgação do resultado preliminar)
+?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>€ 40.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 40.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2025-11-13: Prazo para envio de pré-propostas
 2026-04-13: Prazo para envio de propostas completas convidadas</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1201,81 +1432,81 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-23 08:30
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1131,9 +1123,9 @@
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 22/05/2026</t>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-28 09:15
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -653,51 +661,192 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES/SEGER Nº 14/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL SERVIDORES PÚBLICOS 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 28/05/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)</t>
+          <t>2026-05-25 a 2026-06-23: Submissão de candidaturas (O prazo de submissão vence às 17h59min do dia 23/06/2026. O Governo do Estado do Espírito Santo e o Instituto Trajetórias fornecem suporte e informações aos candidatos de 08h até às 18h. É considerado o horário oficial de Brasília/DF.)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>Este edital visa selecionar até 10 servidores públicos efetivos, estáveis e ativos do Poder Executivo do Estado do Espírito Santo para realizar cursos presenciais de mestrado em universidades estrangeiras de excelência. O programa busca fortalecer a capacidade institucional do Estado, apoiar projetos de pesquisa e desenvolver lideranças transformadoras no setor público, contribuindo para a geração de conhecimento, inovação e desenvolvimento.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Servidores públicos estaduais efetivos, estáveis e ativos do Poder Executivo do Estado do Espírito Santo integrantes da administração pública direta, autárquica ou fundacional.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>US$ 500.000,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Bolsa de estudo de mestrado internacional (BMI-TG) de US$ 5.000,00 por parcela trimestral (vigência de 12 a 24 meses) e Auxílio-Instalação (AI-TG) de US$ 10.000,00 em parcela única.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>?: Impugnação ao Edital (Até 5 (cinco) dias úteis anteriores ao encerramento do prazo de submissão das propostas.)
+2026-05-25 a 2026-06-23: Submissão de candidaturas (O prazo de submissão vence às 17h59min do dia 23/06/2026. O Governo do Estado do Espírito Santo e o Instituto Trajetórias fornecem suporte e informações aos candidatos de 08h até às 18h. É considerado o horário oficial de Brasília/DF.)
+?: Interposição de recurso administrativo do resultado preliminar de habilitação e de avaliação de mérito (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar.)
+?: Atualização documental para contratação (O cronograma do procedimento será informado oportunamente, após a publicação do resultado final. O candidato deve acessar o sistema Sigfapes e inserir os documentos pessoais listados no Anexo VII.)
+?: Assinatura do Termo de Concessão de Bolsa (O cronograma do procedimento será informado oportunamente, após a publicação do resultado final. A assinatura é eletrônica via E-Docs/Acesso Cidadão.)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>As bolsas e o auxílio-instalação serão pagas em reais (BRL) conforme conversão a ser realizada através do Conversor de Moedas do Banco Central do Brasil. Todo o custeio do curso, incluindo anuidades e taxas de matrícula, moradia, passagens, visto, transporte, acomodação, realização da pesquisa e outras despesas, é de responsabilidade exclusiva do beneficiário. Os aprovados podem ser elegíveis a se candidatar a descontos de 15% a 100% nas anuidades e taxas de matrícula de universidades conveniadas, e financiamento para custeio do curso no exterior, oferecidos pelo Instituto Trajetórias. A aprovação no processo seletivo não garante autorização automática de afastamento remunerado, que é um ato discricionário e condicionado a processo próprio e autorização do Governador. O curso de mestrado deve se enquadrar em áreas como transformação digital, políticas de inovação, sustentabilidade, desenvolvimento econômico regional, saúde pública, educação pública ou planejamento governamental. As universidades de excelência são aquelas entre os 100 primeiros colocados nos rankings QS World University Rankings ou Times Higher Education World University Rankings (edições de 2026). Há vedações específicas para participação, incluindo servidores em cargo em comissão, com licenças sem vencimentos nos últimos 2 anos, ou que não concluíram cursos anteriores. O beneficiário deve retornar ao Brasil e permanecer a serviço do Estado do Espírito Santo pelo prazo correspondente ao período de licenciamento, aplicando o conhecimento adquirido. O reconhecimento (revalidação) do título de mestrado obtido no exterior é de competência exclusiva do beneficiário e deve ocorrer em até 1 (um) ano após a conclusão do curso.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_SERVIDORES_ES_22.05.2026.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_SEGER_No_14_2026_-_PROGRAMA_TALENTOS_GLOBAIS_ESPÍRITO_SANTO_-_MESTRADO_INTERNACIONAL_SERVIDORES_PÚBLICOS_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Formação Científica</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES/SECTI Nº 15/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL PÚBLICO GERAL 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25 a 2026-06-23: Submissão de candidatura (Prazo de submissão vence às 17h59min do dia 23/06/2026. Suporte e informações aos candidatos de 08h até às 18h (horário oficial de Brasília/DF).)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>O edital visa selecionar até 10 candidatos para cursos presenciais de mestrado stricto sensu em instituições estrangeiras de excelência, no âmbito do Programa Talentos Globais Espírito Santo – Mestrado Internacional. O programa busca estimular a mobilidade acadêmica internacional, apoiar a formação de recursos humanos altamente qualificados para o desenvolvimento do Estado e promover o retorno e aplicação do conhecimento adquirido no Brasil.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Candidatos brasileiros, com graduação completa e diploma reconhecido no Brasil, residentes no Estado do Espírito Santo, que tenham iniciado processo de candidatura ou possuam carta de aceite/admissão em programa presencial de mestrado em universidade estrangeira de excelência nas áreas do conhecimento destacadas no edital.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>US$ 500.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>US$ 30.000,00 a US$ 50.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-25 a 2026-06-23: Submissão de candidatura (Prazo de submissão vence às 17h59min do dia 23/06/2026. Suporte e informações aos candidatos de 08h até às 18h (horário oficial de Brasília/DF).)
+2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>O edital prevê duas etapas de seleção: Habilitação e Análise de Mérito, conduzidas por um Comitê de Avaliação. As universidades estrangeiras de excelência são aquelas entre as 100 primeiras colocadas nos rankings QS World University Rankings ou Times Higher Education World University Rankings (edições de 2026). O custeio total do curso, incluindo anuidades, taxas, moradia, passagens e visto, é de responsabilidade exclusiva do beneficiário. Os aprovados podem ser elegíveis a descontos de 15% a 100% nas anuidades/taxas de universidades conveniadas e financiamento para custeio do curso, oferecidos pelo Instituto Trajetórias. O cronograma para a assinatura do Termo de Concessão de Bolsa será informado após a publicação do resultado final. O beneficiário se compromete a residir e atuar no Brasil pelo mesmo período de vigência da bolsa, aplicando o conhecimento adquirido em atividades de ensino, pesquisa, inovação, extensão, gestão pública ou iniciativas de impacto social e econômico no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Talentos_Globais_Secti_22.05.2026.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_SECTI_No_15_2026_-_PROGRAMA_TALENTOS_GLOBAIS_ESPÍRITO_SANTO_-_MESTRADO_INTERNACIONAL_PÚBLICO_GERAL_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -716,149 +865,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 01/2026 - TCC EMPREENDEDOR INOVADOR</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Chamada pública para seleção de Trabalhos de Conclusão de Curso (TCCs) previstos nos Projetos Pedagógicos dos cursos de graduação, com ênfase em inovação, aplicação prática, geração de valor e/ou impacto socioambiental. O edital visa incentivar o desenvolvimento de TCCs com foco em inovação, empreendedorismo e aplicabilidade prática, por meio da concessão de Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC).</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Estudantes de graduação em fase de conclusão de curso, regularmente matriculados em Instituições de Ensino Superior (IES) públicas ou privadas, sediadas no Estado do Espírito Santo, e seus orientadores. O proponente (professor orientador) deve ter vínculo estatutário ou celetista por tempo indeterminado com IES reconhecida pelo MEC no Espírito Santo, não estar afastado da IES, estar adimplente junto à FAPES, residir no Espírito Santo ou municípios limítrofes, ter currículo Lattes atualizado (menos de 6 meses), e comprovar matrícula dos alunos aprovados. Se o proponente indicar alunos de outra IES, deve apresentar declaração de autorização de ambas as IES. O aluno orientado deve ser estudante regular de graduação na IES de vínculo do proponente localizada no Espírito Santo, ter coeficiente de rendimento igual ou superior a 7,0, estar adimplente com a FAPES, ter professor orientador durante todo o período da bolsa, residir no Espírito Santo ou municípios limítrofes, e ser cadastrado no Sigfapes.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>R$ 1.600.000,00</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>R$ 11.000,00</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-21: Impugnação do Edital (Primeira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada)
-2026-02-02 a 2026-03-30: Submissão de propostas (Primeira Chamada) (Até 17h59)
-2026-05-27 a 2026-06-02: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
-2026-06-23 a 2026-06-27: Prazo de contratação (Primeira Chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2026-10-20: Impugnação do Edital (Segunda Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da segunda chamada)
-2026-09-02 a 2026-10-27: Submissão de propostas (Segunda Chamada) (Até 17h59)
-2026-12-23 a 2026-12-29: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
-2027-01-28 a 2027-02-03: Prazo de contratação (Segunda Chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2027-03-23: Impugnação do Edital (Terceira Chamada) (Até 5 dias úteis antes do encerramento do prazo de submissão da terceira chamada)
-2027-02-02 a 2027-03-30: Submissão de propostas (Terceira Chamada) (Até 17h59)
-2027-05-25 a 2027-05-31: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 dias úteis a partir da publicação do resultado de seleção)
-2027-06-23 a 2027-06-29: Prazo de contratação (Terceira Chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses para apresentação da Declaração ou Ata de Defesa do TCC. As propostas concorrerão com as demais de suas respectivas microrregiões, sendo apoiados, na primeira chamada, no máximo 20 projetos de TCC por microrregião e, na segunda e terceira chamadas, até 10 projetos de TCC por microrregião. Recursos financeiros remanescentes serão destinados aos demais projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. O proponente pode indicar no mínimo 3 e no máximo 5 alunos orientados por proposta. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis. Além das bolsas BTCC para os alunos, o orientador receberá até dois auxílios para orientação de TCC. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Não será permitido o acúmulo de bolsas Fapes pelo aluno orientado, exceto com bolsas do Programa Nossa Bolsa, do Programa Universidade para Todos (Prouni) e com Bolsas de Extensão (Ext-E e Ext-F) da Fapes.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_01_2026_-_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Extensão</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
 ?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -866,137 +936,138 @@
 ?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 06/2026 - APOIO AOS CLUSTERS DE INOVAÇÃO CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>O edital tem como objetivo fomentar projetos inovadores que visam fortalecer, modernizar e aumentar a competitividade dos setores de Comércio e da Indústria de Alimentos e Bebidas no Espírito Santo. A iniciativa busca incentivar a transformação digital, a melhoria da eficiência operacional e a adoção de práticas sustentáveis pelas empresas, contribuindo para o desenvolvimento econômico, social e ambiental do Estado.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no território do Espírito Santo, que comprovem faturamento local, tenham no mínimo 3 empregados CLT na unidade capixaba e infraestrutura instalada, e que estejam regularizadas junto às Fazendas Públicas e adimplentes com a Fapes. Podem contar com apoio de ICTs ou IES/P reconhecidas pela Fapes.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 12.000.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 600.000,00</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-20 a 2026-05-06: Período de submissão das propostas (Até às 17h59)
-2026-05-30 a 2026-06-05: Prazo para submissão de recursos administrativos (habilitação) (5 (cinco) dias úteis a partir da publicação do resultado de habilitação das propostas)
-2026-07-25 a 2026-07-31: Prazo para submissão de recursos administrativos (mérito) (5 (cinco) dias úteis a partir da publicação do resultado preliminar de avaliação de mérito)
-2026-08-24 a 2026-10-23: Início da contratação (Período de até 60 dias após a publicação do resultado final homologado para submissão de documentos e assinatura do Termo de Outorga e Projeto Aprovado, via SIGFAPES e E-Docs, até às 17h00min.)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Cada proponente ou empresa poderá submeter apenas uma única proposta. As propostas contratadas terão prazo de 24 meses para execução, prorrogáveis por até 12 meses. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. As empresas selecionadas devem depositar 5% do valor da subvenção como contrapartida financeira. Pelo menos um membro da equipe deve realizar o curso 'uso da propriedade intelectual em negócios de base tecnológica' do INPI.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Clusters_Inovadores_-_2ª_Edição_-_Lançamento.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_No_06_2026_-_APOIO_AOS_CLUSTERS_DE_INOVAÇÃO_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Extensão</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 28/05/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
+          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 5.000.000,00</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 80.000,00</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
+2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
+2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
+2026-10-05 a 2026-10-09: Prazo para submissão de recursos administrativos (Análise de Mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
+2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1010,70 +1081,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1096,70 +1167,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1169,79 +1240,19 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1264,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1261,114 +1272,109 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1386,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1388,34 +1394,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1424,81 +1495,77 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>USD 20.000,00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>USD 20.000,00</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-05-29 09:07
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -669,9 +661,9 @@
           <t>EDITAL FAPES/SEGER Nº 14/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL SERVIDORES PÚBLICOS 2026</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 28/05/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -741,9 +733,9 @@
           <t>EDITAL FAPES/SECTI Nº 15/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL PÚBLICO GERAL 2026</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 28/05/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -963,9 +955,9 @@
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 28/05/2026</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-10 09:11
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -881,38 +881,38 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
+          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)</t>
+          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado.</t>
+          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes.</t>
+          <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
+          <t>R$ 5.000.000,00</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 80.000,00</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -921,77 +921,6 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-09: Data limite para submissão das propostas (até 17h59, via Sigfapes)
-?: Prazo para submissão de recursos administrativos (habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação)
-?: Prazo para submissão de recursos administrativos (mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar do mérito)
-?: Início da contratação / Assinatura do Termo de Outorga (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Serão apoiados 4 projetos oriundos das IES/P/T para cada microrregião e 10 projetos na ampla concorrência. Recursos remanescentes da não contratação de projetos em uma microrregião serão redistribuídos para os projetos mais bem classificados da ampla concorrência. O orçamento do projeto poderá ser aprovado na íntegra ou parcialmente. Cada proponente poderá ser coordenador(a) de somente uma proposta; em caso de mais de uma submissão, a última será considerada para análise. Não será permitida a participação de Empresário Individual, Microempreendedor individual (MEI) ou Empresa Júnior como empresa parceira do projeto.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Extensão</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 5.000.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 80.000,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
 2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
@@ -1000,66 +929,66 @@
 2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1073,70 +1002,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1159,70 +1088,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1232,19 +1161,79 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1245,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1264,47 +1253,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 25.000,00 por ano de projeto</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1307,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1328,45 +1319,48 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>€ 25.000,00 por ano de projeto</t>
+          <t>€ 40.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1372,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1386,99 +1380,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+          <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+          <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
+          <t>32.045.000 Euro</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+          <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>32.045.000 Euro</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1487,77 +1416,77 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>USD 20.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
+        </is>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
+          <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>USD 20.000,00</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-11 09:25
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -881,46 +889,125 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 11/06/2026</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado."
+Público-alvo: "Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes." → "Coordenadores de projetos vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, com graduação e experiência em projetos de extensão (mínimo 3 anos) ou titulação mínima de mestre, currículo Lattes atualizado, adimplentes com a Fapes, brasileiros/estrangeiros com visto permanente e residentes no ES ou municípios limítrofes."
+Contato: "editais.extensao@fapes.es.gov.br" → "editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br"
+Submissão (nova): Data limite para submissão das propostas — ? a 2026-06-30
+Submissão (removida): Data limite para submissão das propostas — ? a 2026-06-09</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Coordenadores de projetos vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, com graduação e experiência em projetos de extensão (mínimo 3 anos) ou titulação mínima de mestre, currículo Lattes atualizado, adimplentes com a Fapes, brasileiros/estrangeiros com visto permanente e residentes no ES ou municípios limítrofes.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>R$ 60.000,00</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))
+2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)
+?: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
+?: Prazo para submissão de recursos administrativos (Avaliação de Mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
+?: Assinatura do Termo de Outorga e do Projeto Aprovado (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)
+2026-10-01: Início da vigência dos projetos contratados (No 1º dia útil do mês subsequente à data de assinatura do Termo de Outorga)
+?: Contratação de suplentes (se aplicável) (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)
+?: Envio do Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Suplentes) (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Extensão</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
 2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
@@ -929,66 +1016,66 @@
 2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1002,70 +1089,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1088,70 +1175,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1161,79 +1248,19 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1272,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1253,114 +1280,109 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1394,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1380,34 +1402,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1416,77 +1503,77 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-12 09:08
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -892,9 +884,9 @@
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 11/06/2026</t>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -902,15 +894,7 @@
           <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) localizadas no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado."
-Público-alvo: "Profissionais vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T), públicas e privadas, com atividades de extensão regulamentadas, localizadas no estado do Espírito Santo. O proponente deve ser coordenador do projeto, possuir vínculo empregatício (ou termo de adesão a trabalho voluntário se aposentado), ter graduação concluída com 3 anos de experiência em projetos de extensão ou titulação mínima de mestre, currículo Lattes atualizado há menos de 6 meses, não integrar outra equipe executora neste edital, estar adimplente com a Fapes, ser brasileiro ou estrangeiro com visto permanente e residir no Espírito Santo ou municípios limítrofes." → "Coordenadores de projetos vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, com graduação e experiência em projetos de extensão (mínimo 3 anos) ou titulação mínima de mestre, currículo Lattes atualizado, adimplentes com a Fapes, brasileiros/estrangeiros com visto permanente e residentes no ES ou municípios limítrofes."
-Contato: "editais.extensao@fapes.es.gov.br" → "editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br"
-Submissão (nova): Data limite para submissão das propostas — ? a 2026-06-30
-Submissão (removida): Data limite para submissão das propostas — ? a 2026-06-09</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-18 09:12
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1256,28 +1264,28 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 18/06/2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
@@ -1289,22 +1297,22 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1324,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1324,114 +1332,109 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1446,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1451,34 +1454,99 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>€ 40.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2025-11-13: Prazo para envio de pré-propostas
+2026-04-13: Prazo para envio de propostas completas convidadas</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>32.045.000 Euro</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
 2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
@@ -1487,77 +1555,77 @@
 ?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>USD 20.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-19 09:24
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1267,9 +1259,9 @@
           <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 18/06/2026</t>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-23 09:05
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -799,46 +807,116 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 23/06/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -857,70 +935,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Coordenadores de projetos vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, com graduação e experiência em projetos de extensão (mínimo 3 anos) ou titulação mínima de mestre, currículo Lattes atualizado, adimplentes com a Fapes, brasileiros/estrangeiros com visto permanente e residentes no ES ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))
 2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)
@@ -932,66 +1010,66 @@
 ?: Envio do Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Suplentes) (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
 2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
@@ -1000,66 +1078,66 @@
 2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1073,70 +1151,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1159,70 +1237,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1232,139 +1310,93 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 18/2026 PARCERIAS ENTRE STARTUPS</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 23/06/2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-07-21: Prazo final para solicitar atendimento especializado (Até 10 dias úteis antes do prazo final para submissão das propostas.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>Selecionar e apoiar startups capixabas, através de subvenção econômica (recursos não reembolsáveis), para celebrar parcerias estratégicas com outras startups (locais, nacionais ou internacionais) visando a expansão de mercado, inovação, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+          <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e que atendam aos requisitos do edital.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 9.800.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 250.000,00</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-07-21: Prazo final para solicitar atendimento especializado (Até 10 dias úteis antes do prazo final para submissão das propostas.)
+2026-07-27: Prazo final para impugnação do edital (Até 5 dias úteis antes da data final para submissão das propostas.)
+2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES.)
+2026-10-03 a 2026-10-09: Prazo para submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
+?: Para constituir Empresa e atualização documental no SIGFAPES (Período a ser definido na fase de contratação.)
+?: Assinatura do Termo de Outorga e do Projeto Aprovado (Período a ser definido na fase de contratação.)
+2026-12-01 a 2026-12-30: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. Cada proponente pode submeter até 2 propostas em modalidades diferentes e com parceiros distintos. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. O prazo de execução das propostas contratadas é de 24 meses, prorrogável por até 12 meses. Para critérios de contratação, algumas empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_PARCERIAS_ENTRE_STARTUPS.pdf</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1408,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1384,242 +1416,169 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WATER4ALL</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES visa apoiar projetos colaborativos de pesquisa e inovação no âmbito da Chamada Confap &amp; Water4All – Water and Health 2025. O edital busca financiar propostas que abordem os principais desafios relacionados à interconexão entre água e saúde humana. Isso inclui temas como qualidade da água, contaminantes e tecnologias de tratamento, visando identificar soluções e estratégias para a área.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projeto com titulação mínima de doutor, brasileiros ou estrangeiros com visto permanente, vinculados a Instituições de Ensino Superior, Pesquisa e/ou Tecnológica e/ou de Inovação (públicas ou privadas) no estado do Espírito Santo, com vínculo empregatício por prazo indeterminado (se ativos) ou termo de adesão ao serviço voluntário (se aposentados), residentes no Espírito Santo e adimplentes junto à FAPES. Devem também atender aos critérios de elegibilidade da Chamada CONFAP-Water4All 2025 e normas da Resolução CCAF № 357/2025 e Instrução de Serviço № 082/2025.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>€ 40.000,00</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, parcerias@fapes.es.gov.br, parcerias1@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-13: Prazo para envio de pré-propostas
-2026-04-13: Prazo para envio de propostas completas convidadas</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>A FAPES apoiará 01 (um) projeto com recursos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo (FUNCITEC). Os temas abordados incluem contaminantes transmitidos pela água e riscos à saúde, ferramentas e tecnologias inovadoras de monitoramento, tratamento de água e redução de exposição, e governança, inovação socioeconômica e integração de políticas. O projeto selecionado terá prazo de vigência de até 36 meses, e o apoio financeiro da FAPES cobrirá despesas de custeio e capital, exceto bolsas. As propostas devem ser submetidas na plataforma internacional da chamada, e a FAPES fará o controle de elegibilidade nas fases de pré-propostas e propostas completas. A contratação seguirá a ordem de classificação da Comissão Europeia.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada_Water4All_2025%20-%20Water4ALL.pdf</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WATER4ALL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>3ª CHAMADA TRANSACIONAL CONJUNTA - PARCERIA ECONOMIA AZUL SUSTENTÁVEL</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa impulsionar a digitalização e a inovação para ecossistemas marinhos, negócios e comunidades resilientes, fortalecendo a competitividade da Economia Azul da União Europeia. Serão financiados projetos de pesquisa e inovação que contribuam para a transição para uma economia azul sustentável, resiliente e neutra em carbono, com foco em áreas como Gêmeos Digitais do Oceano, transição de setores da economia azul, planejamento climático inteligente, bio-recursos azuis e comunidades costeiras resilientes. O objetivo é gerar conhecimento acionável e soluções para um oceano saudável e uma economia azul produtiva.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Consórcios compostos por parceiros elegíveis de pelo menos três países diferentes participantes da chamada, solicitando apoio financeiro de pelo menos três Organizações Financiadoras Participantes (PFOs) distintas. Adicionalmente, os projetos devem envolver pelo menos duas entidades legais independentes de dois Estados Membros da UE ou Países Associados ao Horizon Europe elegíveis para financiamento da UE. O Investigador Principal (PI) do coordenador do consórcio deve ser empregado por uma organização elegível em um dos países participantes da chamada.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>32.045.000 Euro</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>sbep.call-secretariat@uefiscdi.ro, epss.sbep@g.etag.ee</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2025-11-17: Prazo final para submissão de pré-propostas (Até as 15:00 CET)
-2026-03-15 a 2026-04-01: Período para procedimento de recurso (Etapa 1)
-2026-06-17: Prazo final para submissão de propostas completas (Até as 15:00 CET)
-2026-11-01 a 2026-11-15: Período para procedimento de recurso (Etapa 2)
-?: Negociações de subvenções nacionais/regionais para os projetos recomendados para financiamento</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>A chamada é co-patrocinada pela Década das Nações Unidas da Ciência Oceânica para o Desenvolvimento Sustentável. Os projetos devem ser orientados para o impacto, seguindo uma abordagem de via de impacto. É exigido o envolvimento de múltiplos stakeholders (quádrupla hélice), incluindo pelo menos um parceiro da indústria, governo, institutos de pesquisa ou público. Atividades de participação cidadã e literacia oceânica são encorajadas. As propostas são fortemente recomendadas a cobrir um mínimo de duas bacias marítimas da UE (Oceano Atlântico, Mar Báltico, Mar Negro, Mar Mediterrâneo, Mar do Norte). Todas as propostas devem estar alinhadas com a Taxonomia da UE e cumprir os princípios éticos. Um processo de submissão em duas etapas é obrigatório (pré-proposta e, em seguida, proposta completa mediante convite). As informações fornecidas nas pré-propostas são vinculativas para as propostas completas; nenhuma alteração importante no conteúdo é permitida. O coordenador do consórcio pode ser Investigador Principal (PI) em apenas uma proposta. Parceiros do mesmo país não podem solicitar mais de 60% do financiamento total. A duração do projeto é de 36 meses. Os beneficiários do financiamento devem reconhecer o financiamento da SBEP e do Horizon Europe e aderir à Política de Ciência Aberta da CE para publicações.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/SBEP%20Call%20text%202025.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/3a_CHAMADA_TRANSACIONAL_CONJUNTA_-_PARCERIA_ECONOMIA_AZUL_SUSTENTÁVEL.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP BRASIL–ILLINOIS 2026</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>O programa visa promover e fortalecer a colaboração científica por meio de projetos de pesquisa conjuntos entre pesquisadores e instituições afiliadas às Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras e à University of Illinois System. O objetivo é fomentar a cooperação internacional e abordar áreas de pesquisa prioritárias.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores/coordenadores que desenvolvam atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros, sediados em estados cujas FAPs confirmaram participação na chamada.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>USD 20.000,00</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-26: Submissão de propostas (Até 23:59 (BRT) para PIs do lado brasileiro e 23:59 (GMT-5) para PIs do lado da University of Illinois System. Submissão via https://sistema.confap.org.br, podendo ser exigida submissão adicional nas plataformas das FAPs participantes.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Serão apoiados até 20 projetos de pesquisa conjuntos. As propostas devem ser elaboradas em inglês (máximo 10 páginas) e incluir uma descrição clara da colaboração planejada, valor agregado e complementaridade das equipes. As áreas de pesquisa prioritárias são: Clima, Sustentabilidade, Agricultura; Saúde Pública e Medicina; e Democracia e Inclusão. Cada PI pode submeter apenas uma proposta. O apoio financeiro para o lado brasileiro (FAPs) destina-se a cobrir custos gerais, viagens internacionais, diárias, fundos semente para custos diretos de pesquisa e workshops. É exigido seguro médico para visitantes.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Cooperative%20Program%20-U%20of%20I%20and%20Confap%20v%205%2024-03.docx.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_BRASIL–ILLINOIS_2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-24 08:59
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23: Submissão das propostas (até as 17h59 (horário de Brasília))</t>
+          <t>2026-08-03: Contratação dos projetos</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -674,11 +674,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25 a 2026-06-23: Submissão de candidaturas (O prazo de submissão vence às 17h59min do dia 23/06/2026. O Governo do Estado do Espírito Santo e o Instituto Trajetórias fornecem suporte e informações aos candidatos de 08h até às 18h. É considerado o horário oficial de Brasília/DF.)</t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -748,7 +744,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-25 a 2026-06-23: Submissão de candidatura (Prazo de submissão vence às 17h59min do dia 23/06/2026. Suporte e informações aos candidatos de 08h até às 18h (horário oficial de Brasília/DF).)</t>
+          <t>2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -810,9 +806,9 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 23/06/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -969,7 +965,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))</t>
+          <t>2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
@@ -1040,7 +1036,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)</t>
+          <t>2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1334,28 +1330,28 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 18/2026 PARCERIAS ENTRE STARTUPS</t>
+          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Novo - e-mail enviado em 23/06/2026</t>
+          <t>Novo - e-mail enviado em 24/06/2026</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21: Prazo final para solicitar atendimento especializado (Até 10 dias úteis antes do prazo final para submissão das propostas.)</t>
+          <t>2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Selecionar e apoiar startups capixabas, através de subvenção econômica (recursos não reembolsáveis), para celebrar parcerias estratégicas com outras startups (locais, nacionais ou internacionais) visando a expansão de mercado, inovação, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca, acesso a financiamento e impacto socioambiental sustentável.</t>
+          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Startups (pessoas jurídicas) sediadas no Espírito Santo, com faturamento bruto anual de até R$ 16.000.000,00 e que atendam aos requisitos do edital.</t>
+          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1375,18 +1371,19 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21: Prazo final para solicitar atendimento especializado (Até 10 dias úteis antes do prazo final para submissão das propostas.)
-2026-07-27: Prazo final para impugnação do edital (Até 5 dias úteis antes da data final para submissão das propostas.)
-2026-06-22 a 2026-08-04: Submissão de propostas (Via SIGFAPES.)
-2026-10-03 a 2026-10-09: Prazo para submissão de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar da habilitação.)
-?: Para constituir Empresa e atualização documental no SIGFAPES (Período a ser definido na fase de contratação.)
-?: Assinatura do Termo de Outorga e do Projeto Aprovado (Período a ser definido na fase de contratação.)
-2026-12-01 a 2026-12-30: Prazo para informar dados da conta bancária (30 dias a partir do início da vigência do Termo de Outorga.)</t>
+          <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
+2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
+2026-10-02 a 2026-10-09: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)
+?: Constituição de empresa e atualização documental no SIGFAPES (Proponentes aprovados) (Para proponentes aprovados sem empresa constituída. Período a ser definido pela FAPES após homologação do resultado.)
+?: Assinatura do Termo de Outorga e Projeto Aprovado (Proponentes aprovados) (Até às 17h. Período a ser definido pela FAPES após homologação do resultado.)
+?: Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Até às 17h. Período a ser definido pela FAPES após homologação do resultado. Envio via e-Flow Formulário nº 26.)
+2026-12-01 a 2026-12-31: Informar dados da conta bancária aberta (Prazo de 30 dias a partir do início da vigência do Termo de Outorga.)
+?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. Cada proponente pode submeter até 2 propostas em modalidades diferentes e com parceiros distintos. É vedada a submissão de propostas com as mesmas startups alternando funções de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. O prazo de execução das propostas contratadas é de 24 meses, prorrogável por até 12 meses. Para critérios de contratação, algumas empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo.</t>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1396,7 +1393,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-25 08:55
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -430,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -593,12 +585,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Formação Científica</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 13/2026  - PROGRAMA INSTITUCIONAL DE BOLSAS DE INICIAÇÃO CIENTÍFICA, TECNOLÓGICA E DE INOVAÇÃO DO ESPÍRITO SANTO (PIBICES 2026/2027)</t>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -608,65 +600,67 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03: Contratação dos projetos</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>O Programa Institucional de Bolsas de Iniciação Científica, Tecnológica e de Inovação do Estado do Espírito Santo (PIBICES) visa fomentar a participação de estudantes de graduação em atividades sistemáticas de pesquisa científica, desenvolvimento tecnológico e inovação. O edital busca fortalecer o sistema capixaba de pesquisa e a formação de recursos humanos qualificados, contribuindo para a ampliação da cultura científica e a produção de conhecimento alinhada às demandas da sociedade. Serão concedidas cotas institucionais de bolsas para Programas Institucionais de Bolsas de Iniciação Científica, Tecnológica e de Inovação (PIBICTI) em Instituições de Ensino Superior e/ou Pesquisa.</t>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Coordenadores Institucionais de Programas de Bolsas de Iniciação Científica, Tecnológica e de Inovação (PIBICTI) vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo, que sejam pesquisadores/docentes com título de mestre ou doutor e vínculo empregatício indeterminado com a IES/P.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>R$ 8.640.000,00</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n"/>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>bolsas.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16: Impugnação do edital (até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
-2026-06-23: Submissão das propostas (até as 17h59 (horário de Brasília))
-?: Interposição de recursos (habilitação) (até 5 dias úteis após a divulgação do resultado preliminar)
-2026-08-03: Contratação dos projetos
-?: Indicação dos bolsistas (a partir do início de vigência do Termo de Outorga)</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Serão disponibilizadas 800 bolsas de Iniciação Científica e Tecnológica (ICT). Cada bolsa terá duração mínima de 4 e máxima de 12 meses, com valor mensal atual de R$ 900,00. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações de atividades, utilizando a citação padrão fornecida no edital. A Fapes pode alterar datas e prazos do cronograma ou reabrir prazos em casos de força maior ou falhas comprovadas nos sistemas.</t>
+          <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20PIBICES%20-%20Assinado.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>formacao_cientifica/EDITAL_FAPES_No_13_2026_-_PROGRAMA_INSTITUCIONAL_DE_BOLSAS_DE_INICIAÇÃO_CIENTÍFICA,_TECNOLÓGICA_E_DE_INOVAÇÃO_DO_ESPÍRITO_SANTO_(PIBICES_2026_2027).pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Formação Científica</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES/SEGER Nº 14/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL SERVIDORES PÚBLICOS 2026</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -674,245 +668,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa selecionar até 10 servidores públicos efetivos, estáveis e ativos do Poder Executivo do Estado do Espírito Santo para realizar cursos presenciais de mestrado em universidades estrangeiras de excelência. O programa busca fortalecer a capacidade institucional do Estado, apoiar projetos de pesquisa e desenvolver lideranças transformadoras no setor público, contribuindo para a geração de conhecimento, inovação e desenvolvimento.</t>
+          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Servidores públicos estaduais efetivos, estáveis e ativos do Poder Executivo do Estado do Espírito Santo integrantes da administração pública direta, autárquica ou fundacional.</t>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>US$ 500.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Bolsa de estudo de mestrado internacional (BMI-TG) de US$ 5.000,00 por parcela trimestral (vigência de 12 a 24 meses) e Auxílio-Instalação (AI-TG) de US$ 10.000,00 em parcela única.</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>?: Impugnação ao Edital (Até 5 (cinco) dias úteis anteriores ao encerramento do prazo de submissão das propostas.)
-2026-05-25 a 2026-06-23: Submissão de candidaturas (O prazo de submissão vence às 17h59min do dia 23/06/2026. O Governo do Estado do Espírito Santo e o Instituto Trajetórias fornecem suporte e informações aos candidatos de 08h até às 18h. É considerado o horário oficial de Brasília/DF.)
-?: Interposição de recurso administrativo do resultado preliminar de habilitação e de avaliação de mérito (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar.)
-?: Atualização documental para contratação (O cronograma do procedimento será informado oportunamente, após a publicação do resultado final. O candidato deve acessar o sistema Sigfapes e inserir os documentos pessoais listados no Anexo VII.)
-?: Assinatura do Termo de Concessão de Bolsa (O cronograma do procedimento será informado oportunamente, após a publicação do resultado final. A assinatura é eletrônica via E-Docs/Acesso Cidadão.)</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>As bolsas e o auxílio-instalação serão pagas em reais (BRL) conforme conversão a ser realizada através do Conversor de Moedas do Banco Central do Brasil. Todo o custeio do curso, incluindo anuidades e taxas de matrícula, moradia, passagens, visto, transporte, acomodação, realização da pesquisa e outras despesas, é de responsabilidade exclusiva do beneficiário. Os aprovados podem ser elegíveis a se candidatar a descontos de 15% a 100% nas anuidades e taxas de matrícula de universidades conveniadas, e financiamento para custeio do curso no exterior, oferecidos pelo Instituto Trajetórias. A aprovação no processo seletivo não garante autorização automática de afastamento remunerado, que é um ato discricionário e condicionado a processo próprio e autorização do Governador. O curso de mestrado deve se enquadrar em áreas como transformação digital, políticas de inovação, sustentabilidade, desenvolvimento econômico regional, saúde pública, educação pública ou planejamento governamental. As universidades de excelência são aquelas entre os 100 primeiros colocados nos rankings QS World University Rankings ou Times Higher Education World University Rankings (edições de 2026). Há vedações específicas para participação, incluindo servidores em cargo em comissão, com licenças sem vencimentos nos últimos 2 anos, ou que não concluíram cursos anteriores. O beneficiário deve retornar ao Brasil e permanecer a serviço do Estado do Espírito Santo pelo prazo correspondente ao período de licenciamento, aplicando o conhecimento adquirido. O reconhecimento (revalidação) do título de mestrado obtido no exterior é de competência exclusiva do beneficiário e deve ocorrer em até 1 (um) ano após a conclusão do curso.</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_SERVIDORES_ES_22.05.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_SEGER_No_14_2026_-_PROGRAMA_TALENTOS_GLOBAIS_ESPÍRITO_SANTO_-_MESTRADO_INTERNACIONAL_SERVIDORES_PÚBLICOS_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Formação Científica</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES/SECTI Nº 15/2026 - PROGRAMA TALENTOS GLOBAIS ESPÍRITO SANTO - MESTRADO INTERNACIONAL PÚBLICO GERAL 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa selecionar até 10 candidatos para cursos presenciais de mestrado stricto sensu em instituições estrangeiras de excelência, no âmbito do Programa Talentos Globais Espírito Santo – Mestrado Internacional. O programa busca estimular a mobilidade acadêmica internacional, apoiar a formação de recursos humanos altamente qualificados para o desenvolvimento do Estado e promover o retorno e aplicação do conhecimento adquirido no Brasil.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Candidatos brasileiros, com graduação completa e diploma reconhecido no Brasil, residentes no Estado do Espírito Santo, que tenham iniciado processo de candidatura ou possuam carta de aceite/admissão em programa presencial de mestrado em universidade estrangeira de excelência nas áreas do conhecimento destacadas no edital.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>US$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>US$ 30.000,00 a US$ 50.000,00</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>bolsas.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-25 a 2026-06-23: Submissão de candidatura (Prazo de submissão vence às 17h59min do dia 23/06/2026. Suporte e informações aos candidatos de 08h até às 18h (horário oficial de Brasília/DF).)
-2026-07-01 a 2026-07-07: Interposição de recurso administrativo (Prazo de 05 (cinco) dias úteis após a divulgação do resultado preliminar. Interposto via formulário específico no Sistema E-Flow.)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>O edital prevê duas etapas de seleção: Habilitação e Análise de Mérito, conduzidas por um Comitê de Avaliação. As universidades estrangeiras de excelência são aquelas entre as 100 primeiras colocadas nos rankings QS World University Rankings ou Times Higher Education World University Rankings (edições de 2026). O custeio total do curso, incluindo anuidades, taxas, moradia, passagens e visto, é de responsabilidade exclusiva do beneficiário. Os aprovados podem ser elegíveis a descontos de 15% a 100% nas anuidades/taxas de universidades conveniadas e financiamento para custeio do curso, oferecidos pelo Instituto Trajetórias. O cronograma para a assinatura do Termo de Concessão de Bolsa será informado após a publicação do resultado final. O beneficiário se compromete a residir e atuar no Brasil pelo mesmo período de vigência da bolsa, aplicando o conhecimento adquirido em atividades de ensino, pesquisa, inovação, extensão, gestão pública ou iniciativas de impacto social e econômico no Estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Talentos_Globais_Secti_22.05.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_SECTI_No_15_2026_-_PROGRAMA_TALENTOS_GLOBAIS_ESPÍRITO_SANTO_-_MESTRADO_INTERNACIONAL_PÚBLICO_GERAL_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 308.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 12.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
-?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 800.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -931,70 +718,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Coordenadores de projetos vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, com graduação e experiência em projetos de extensão (mínimo 3 anos) ou titulação mínima de mestre, currículo Lattes atualizado, adimplentes com a Fapes, brasileiros/estrangeiros com visto permanente e residentes no ES ou municípios limítrofes.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 60.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))
 2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)
@@ -1006,66 +793,66 @@
 ?: Envio do Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Suplentes) (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
 2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
@@ -1074,66 +861,66 @@
 2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1147,70 +934,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
@@ -1233,70 +1020,70 @@
 2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1306,70 +1093,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 24/06/2026</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 250.000,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1381,199 +1168,199 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-27 08:35
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -961,25 +969,32 @@
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 27/06/2026</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica." → "Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica."
+Público-alvo: "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba." → "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba."
+Submissão (removida): Abertura de empresa e atualização documental (1ª chamada) — 2026-10-27 a 2026-11-03
+Submissão (removida): Abertura de empresa e atualização documental (2ª chamada) — 2027-04-27 a 2027-05-03</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica.</t>
+          <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
+          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -999,30 +1014,20 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
-2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
-2026-07-31 a 2026-08-06: Prazo para recursos administrativos da habilitação (1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2026-10-02 a 2026-10-08: Prazo para recursos administrativos da avaliação de mérito (1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h (horário de Brasília) via SIGFAPES)
-2026-10-27 a 2026-11-03: Período de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2026-10-27 a 2026-11-03: Abertura de empresa e atualização documental (1ª chamada) (Para propostas aprovadas sem empresas constituídas, até as 17h00min)
-2026-10-27 a 2026-11-03: Atualização documental no SIGFAPES (1ª chamada) (Envio de documentos pessoais, até as 17h00min)
-2026-10-27 a 2026-11-03: Assinatura do Termo de Outorga e Projeto Aprovado (1ª chamada) (Eletronicamente via E-docs, até as 17h00min)
-2026-11-03: Envio do e-Flow (Formulário nº 25) e disponibilização de documentos no SIGFAPES (1ª chamada) (Até as 17h00min)
-2026-11-04: Período de contratação de suplentes (1ª chamada) (Se aplicável, até as 17h00min)
-2027-01-08 a 2027-01-14: Prazo para recursos administrativos da habilitação (2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2027-03-19 a 2027-03-25: Prazo para recursos administrativos da avaliação de mérito (2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2027-04-27 a 2027-05-03: Período de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
-2027-04-27 a 2027-05-03: Abertura de empresa e atualização documental (2ª chamada) (Para propostas aprovadas sem empresas constituídas, até as 17h00min)
-2027-04-27 a 2027-05-03: Atualização documental no SIGFAPES (2ª chamada) (Envio de documentos pessoais, até as 17h00min)
-2027-04-27 a 2027-05-03: Assinatura do Termo de Outorga e Projeto Aprovado (2ª chamada) (Eletronicamente via E-docs, até as 17h00min)
-2027-05-03: Envio do e-Flow (Formulário nº 25) e disponibilização de documentos no SIGFAPES (2ª chamada) (Até as 17h00min)
-2027-05-04: Período de contratação de suplentes (2ª chamada) (Se aplicável, até as 17h00min)</t>
+          <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
+2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
+?: Prazo para submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+?: Prazo para submissão de recursos administrativos (mérito - 1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)
+?: Processo de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
+?: Prazo para submissão de recursos administrativos (habilitação - 2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+?: Prazo para submissão de recursos administrativos (mérito - 2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
+?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital, sendo responsabilidade do proponente acompanhar as atualizações no site da FAPES. O edital poderá ser suspenso, revogado ou anulado por interesse público ou exigência legal, sem direito a indenização. O proponente deve manter seus dados cadastrais atualizados no SIGFAPES. A FAPES não exigirá direitos de participação e propriedade intelectual sobre as pesquisas e projetos, mas deverá ser notificada em caso de registro de propriedade intelectual. Os participantes concordam em ceder direitos de imagem para divulgação das ações da FAPES.</t>
+          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-06-28 08:37
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -969,9 +961,9 @@
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 27/06/2026</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -979,14 +971,7 @@
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Este edital da FAPES visa fomentar o empreendedorismo inovador no Espírito Santo, apoiando projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores. Destina-se a doutores que buscam transformar ideias inovadoras em empreendimentos sustentáveis, promovendo a transferência de conhecimento e tecnologia para o mercado e impulsionando a criação ou fortalecimento de micro e pequenas empresas de base tecnológica." → "Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica."
-Público-alvo: "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, interessados em transformar conhecimento científico em soluções inovadoras, criar novos negócios e fortalecer o ecossistema de inovação capixaba." → "Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba."
-Submissão (removida): Abertura de empresa e atualização documental (1ª chamada) — 2026-10-27 a 2026-11-03
-Submissão (removida): Abertura de empresa e atualização documental (2ª chamada) — 2027-04-27 a 2027-05-03</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-01 09:05
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)</t>
+          <t>2026-10-01: Início da vigência dos projetos contratados (No 1º dia útil do mês subsequente à data de assinatura do Termo de Outorga)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)</t>
+          <t>2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)</t>
+          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-03 09:58
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -531,7 +539,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28 a 2026-07-02: Prazo para dúvidas e informações (Até 2 dias úteis antecedentes ao término da submissão das propostas.)</t>
+          <t>2026-07-06: Submissão das propostas (Até as 17h59.)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -742,38 +750,42 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 12/2026 - EXTENSÃO TECNOLÓGICA</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-01: Início da vigência dos projetos contratados (No 1º dia útil do mês subsequente à data de assinatura do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 03/07/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado."
+Público-alvo: "Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024." → "Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital."
+Contato: "editais.extensao@fapes.es.gov.br" → "editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br"
+Submissão (nova): Submissão de propostas — ? a 2026-07-02
+Submissão (removida): Submissão de propostas — ? a 2026-06-30</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão tecnológica em diversas áreas temáticas, coordenados por profissionais de Instituições de Ensino Superior, Pesquisa ou Tecnologia (IES/P/T) no Espírito Santo. O objetivo é promover o envolvimento e a formação de estudantes para o desenvolvimento econômico e social, visando a inclusão social e produtiva nas diferentes microrregiões do estado.</t>
+          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Coordenadores de projetos vinculados a Instituições de Ensino Superior, de Pesquisa ou de Tecnologia (IES/P/T) no Espírito Santo, com graduação e experiência em projetos de extensão (mínimo 3 anos) ou titulação mínima de mestre, currículo Lattes atualizado, adimplentes com a Fapes, brasileiros/estrangeiros com visto permanente e residentes no ES ou municípios limítrofes.</t>
+          <t>Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
+          <t>R$ 5.000.000,00</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>R$ 60.000,00</t>
+          <t>R$ 80.000,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -783,37 +795,37 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até o quinto dia útil que anteceder a data final de submissão das propostas (2026-06-30))
-2026-06-30: Data limite para submissão das propostas (até as 17h59, via Sigfapes)
-?: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
-?: Prazo para submissão de recursos administrativos (Avaliação de Mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
-?: Assinatura do Termo de Outorga e do Projeto Aprovado (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)
-2026-10-01: Início da vigência dos projetos contratados (No 1º dia útil do mês subsequente à data de assinatura do Termo de Outorga)
-?: Contratação de suplentes (se aplicável) (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)
-?: Envio do Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Suplentes) (Os prazos de contratação serão divulgados junto com o resultado final homologado pelo CCAF. Até as 17h00.)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="n"/>
+          <t>2026-07-02: Submissão de propostas (até as 17h59 via Sigfapes)
+?: Interposição de recursos (habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
+?: Interposição de recursos (análise de mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
+?: Início do processo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>O edital oferece pontuação adicional para propostas apresentadas por pessoas com deficiência (PcD), negras, quilombolas, indígenas, trans ou travestis. O prazo de execução dos projetos é de 24 meses. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F por pelo menos 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Serão apoiados 6 projetos por microrregião, com recursos remanescentes distribuídos entre os projetos mais bem classificados, independentemente da microrregião. Propostas que indicarem microrregião coincidente com a instituição de vínculo do proponente concorrerão nos blocos das respectivas microrregiões, enquanto propostas para microrregião distinta concorrerão na ampla concorrência.</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Extensão%20Tecnológica%20-%2012-2026%20-%20Assinado.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>extensao/EDITAL_FAPES_No_12_2026_-_EXTENSÃO_TECNOLÓGICA.pdf</t>
+          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -821,106 +833,34 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)</t>
-        </is>
-      </c>
+      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado.</t>
+          <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024.</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>R$ 5.000.000,00</t>
+          <t>R$ 40.000.000,00</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>R$ 80.000,00</t>
+          <t>R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-23: Prazo para impugnação do edital (Até 5 dias úteis antes da data limite de submissão das propostas)
-2026-06-30: Submissão de propostas (Até as 17h59 via SigFapes)
-2026-08-01 a 2026-08-07: Prazo para submissão de recursos administrativos (Habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
-2026-10-05 a 2026-10-09: Prazo para submissão de recursos administrativos (Análise de Mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
-2026-10-29 a 2026-11-05: Início da contratação e envio de documentos (Até 5 dias úteis da publicação do resultado homologado para o início do processo de contratação. Inclui assinatura do Termo de Outorga e envio do Registro da Lista de Checagem de Documentação (e-Flow) até as 17h00.)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução dos projetos é de 24 meses. É obrigatória a previsão de pelo menos um bolsista EXT-E ou EXT-F por um período mínimo de 22 meses. As propostas devem ser submetidas para apenas uma das 10 microrregiões listadas no edital. Proponentes que declararem pertencimento a grupos de ações afirmativas (PcD, negra, quilombola, indígena, trans ou travesti) podem receber pontuação adicional. Propostas com nota final inferior a 70 pontos serão desclassificadas. É exigida a elaboração de um vídeo apresentando os resultados do projeto. É indispensável a menção explícita e destacada ao apoio da Fapes em todas as divulgações do trabalho.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -934,70 +874,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
@@ -1010,19 +950,99 @@
 ?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 03/07/2026</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável." → "Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões."
+Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br"
+Submissão (nova): Envio da primeira proposta — 2026-05-21 a 2026-07-03
+Submissão (removida): Envio da primeira proposta (Fase 1) — 2026-05-21 a 2026-06-30</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.500.000,00</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 30.000,00</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
+?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
+2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)
+2026-09-21 a 2026-09-30: Apresentação do pitch
+?: Prazo para recurso administrativo (Fase 2) (Até 5 dias úteis após divulgação do resultado preliminar)
+?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
+          <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente ou membros da equipe deverão participar de, no mínimo, 80% das oficinas e mentorias em cada fase, sob pena de desclassificação. Propostas com nota final inferior a 70,0 pontos serão desclassificadas em ambas as fases. A Fapes somente considerará despesas/gastos realizados a partir do início da vigência do Termo de Outorga. O não atendimento ao prazo de entrega da documentação completa ou o descumprimento dos requisitos para contratação resultará na perda do direito à contratação.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
+          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1054,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
+          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1044,109 +1064,36 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)</t>
+          <t>2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável.</t>
+          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
+          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>R$ 4.500.000,00</t>
+          <t>R$ 9.800.000,00</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 250.000,00</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21 a 2026-06-30: Envio da primeira proposta (Fase 1) (até as 17h59)
-?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
-2026-09-14 a 2026-09-22: Envio da segunda proposta (Fase 2) (até as 17h59)
-2026-09-21 a 2026-09-30: Apresentação do pitch (A partir de 21/09/2026)
-?: Prazo para recurso administrativo (Fase 2) (Até 5 dias úteis após divulgação do resultado preliminar)
-?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>O edital será executado em duas fases. Na Fase 1, serão selecionadas 80 propostas de cada microrregião. Na Fase 2, serão selecionadas 25 propostas ou mais por microrregião. O valor total do edital de R$ 4.500.000,00 será distribuído entre as 6 microrregiões, com até R$ 750.000,00 para cada, visando financiar 25 projetos ou mais por microrregião. A participação em no mínimo 80% das oficinas e mentorias é obrigatória para o proponente ou membros da equipe, sob pena de desclassificação. Proponentes podem submeter mais de uma proposta na Fase 1, mas apenas a de maior nota avançará para a Fase 2. Propostas com nota final inferior a 70,0 serão desclassificadas. A Fapes pode alterar as datas e prazos do cronograma.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 9.800.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 250.000,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1158,19 +1105,79 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1189,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1192,18 +1199,18 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -1215,22 +1222,22 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1249,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1250,107 +1257,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
       <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 25.000,00 por ano de projeto</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-04 09:07
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -753,21 +745,13 @@
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 03/07/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do estado." → "Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado."
-Público-alvo: "Pesquisadores com titulação mínima de mestre, experiência comprovada em projetos de extensão nos últimos 3 anos, e vínculo empregatício, estatutário, temporário ou voluntário com Instituições de Ensino Superior ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo. O proponente não deve ter sido contratado no Edital Fapes nº 04/2025 nem solicitado prorrogação de projeto do Edital FAPES nº 02/2024." → "Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital."
-Contato: "editais.extensao@fapes.es.gov.br" → "editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br"
-Submissão (nova): Submissão de propostas — ? a 2026-07-02
-Submissão (removida): Submissão de propostas — ? a 2026-06-30</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado.</t>
@@ -977,24 +961,17 @@
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 03/07/2026</t>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana, no Espírito Santo. Ele oferece apoio técnico e financeiro para soluções inovadoras com potencial de se tornarem negócios ou startups, incentivando a criação de novos negócios de base tecnológica e fortalecendo os ecossistemas locais de inovação para o desenvolvimento sustentável." → "Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões."
-Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br"
-Submissão (nova): Envio da primeira proposta — 2026-05-21 a 2026-07-03
-Submissão (removida): Envio da primeira proposta (Fase 1) — 2026-05-21 a 2026-06-30</t>
-        </is>
-      </c>
+          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-07 10:23
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -531,7 +547,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06: Submissão das propostas (Até as 17h59.)</t>
+          <t>2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -1106,55 +1122,51 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 07/07/2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1178,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1176,18 +1188,18 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -1199,22 +1211,22 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-07-10: Submissao de propostas (Propostas completas, incluindo todos os documentos solicitados no Item nº 6.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Os pesquisadores elegíveis devem registrar sua expressão de interesse no portal online https://sistema.confap.org.br/ e preencher os itens listados. Após o registro e verificação de elegibilidade, terão acesso à lista de projetos ERC-financiados que podem hospedar pesquisadores brasileiros. Os pesquisadores devem contatar o Pesquisador Principal do ERC para acordar a colaboração e definir um Plano de Trabalho. As FAPs participantes fornecerão apoio para despesas de viagem e outros apoios complementares, cujas modalidades devem ser consultadas junto às agências. Os pesquisadores continuarão a receber seus salários/bolsas de acordo com os termos institucionais. Mais informações sobre 'ERC teams open to the world' estão disponíveis em https://erc.europa.eu/managing-your-project/set-and-develop-your-team. O edital é apoiado pelas seguintes FAPs: Fundação Araucária - Paraná, FACEPE - Pernambuco, FAPDF - Distrito Federal, FAPEAL - Alagoas, FAPEAM - Amazonas, FAPEAP - Amapá, FAPEG - Goiás, FAPERGS - Rio Grande do Sul, FAPES - Espírito Santo, FAPESB - Bahia, FAPESC - Santa Catarina, FAPESP - São Paulo, FAPESPA - Pará, FAPERR - Roraima.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1226,55 +1238,134 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 07/07/2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos." → "Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas."
+Público-alvo: "Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros." → "Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES."
+Valor total: "-" → "US$ 18.000,00"
+Valor por proposta: "-" → "US$ 6.000,00"
+Contato: "internacional.confap@gmail.com" → "internacional.confap@gmail.com, global@fapes.es.gov.br"
+Submissão (nova): Submissão de propostas (CONFAP) — ? a 2026-08-10
+Submissão (removida): Submissao de propostas — ? a 2026-07-10</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-08 09:23
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -39,11 +39,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +54,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -68,9 +63,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -438,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -606,116 +598,429 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.500.000,00</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>US$ 2.700,00</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
+2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
+2026-02-06 a 2026-03-09: Período de submissão (1ª Chamada) (eventos com início entre 01/05/2026 a 31/07/2026, até as 17h59)
+2026-03-07: Prazo para envio de dúvidas (1ª Chamada) (até 2 dias antes do prazo final de submissão da 1ª Chamada)
+2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 1ª Chamada)
+2026-03-17 a 2026-04-24: Período de submissão (2ª Chamada) (eventos com início entre 01/08/2026 a 31/12/2026)
+2026-04-22: Prazo para envio de dúvidas (2ª Chamada) (até 2 dias antes do prazo final de submissão da 2ª Chamada)
+2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)
+2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)
+2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)
+2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.500.000,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
+2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
+2026-03-07: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 1ª chamada)
+2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
+2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Eventos com início entre 01/08/2026 a 31/12/2026)
+2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 2ª chamada)
+2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
+2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)
+2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)
+2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
+?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 10.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
+2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
+2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada) (Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/05/2026 a 31/07/2026.)
+2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)
+2026-04-22: Prazo final para envio de dúvidas (2ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada) (Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-08-13: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas da última chamada.)
+2026-08-18: Prazo final para envio de dúvidas (3ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 2.000.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>US$ 2.600,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
+2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
+2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada) (Até 2 dias antes do prazo final de submissão.)
+2026-03-17 a 2026-04-24: Submissão de propostas (2ª Chamada) (Para visitas com início entre 01/08/2026 a 31/12/2026.)
+2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
+2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada) (Até 2 dias antes do prazo final de submissão.)
+2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
+2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)
+2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)
+2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
 ?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -734,66 +1039,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Submissão de propostas (até as 17h59 via Sigfapes)
 ?: Interposição de recursos (habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -801,66 +1106,66 @@
 ?: Início do processo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital oferece pontuação adicional para propostas apresentadas por pessoas com deficiência (PcD), negras, quilombolas, indígenas, trans ou travestis. O prazo de execução dos projetos é de 24 meses. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F por pelo menos 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Serão apoiados 6 projetos por microrregião, com recursos remanescentes distribuídos entre os projetos mais bem classificados, independentemente da microrregião. Propostas que indicarem microrregião coincidente com a instituição de vínculo do proponente concorrerão nos blocos das respectivas microrregiões, enquanto propostas para microrregião distinta concorrerão na ampla concorrência.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -874,70 +1179,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
@@ -950,70 +1255,70 @@
 ?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1023,70 +1328,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente ou membros da equipe deverão participar de, no mínimo, 80% das oficinas e mentorias em cada fase, sob pena de desclassificação. Propostas com nota final inferior a 70,0 pontos serão desclassificadas em ambas as fases. A Fapes somente considerará despesas/gastos realizados a partir do início da vigência do Termo de Outorga. O não atendimento ao prazo de entrega da documentação completa ou o descumprimento dos requisitos para contratação resultará na perda do direito à contratação.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 250.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1098,274 +1403,332 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 08/07/2026</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 07/07/2026</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 07/07/2026</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O edital convida pesquisadores do Brasil a buscar colaborações de pesquisa com Pesquisadores Principais já apoiados por bolsas do Conselho Europeu de Pesquisa (ERC) financiadas pela UE. O objetivo é proporcionar oportunidades de pesquisa na Europa para pesquisadores brasileiros ativos, promovendo intercâmbios científicos e o desenvolvimento de projetos colaborativos." → "Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas."
-Público-alvo: "Pesquisadores ativos do Brasil, com título de PhD, que estejam desenvolvendo atividades de pesquisa em universidades, institutos ou centros de pesquisa brasileiros." → "Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES."
-Valor total: "-" → "US$ 18.000,00"
-Valor por proposta: "-" → "US$ 6.000,00"
-Contato: "internacional.confap@gmail.com" → "internacional.confap@gmail.com, global@fapes.es.gov.br"
-Submissão (nova): Submissão de propostas (CONFAP) — ? a 2026-08-10
-Submissão (removida): Submissao de propostas — ? a 2026-07-10</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>US$ 18.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>US$ 6.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
 2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-09 10:51
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -754,28 +754,28 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO CIENTÍFICO</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 09/07/2026</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)</t>
+          <t>2026-06-19 a 2026-07-19: Período de contratação (2ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de estágio técnico-científico. O estágio pode ser em laboratório ou centro de pesquisa, desenvolvimento ou inovação (PD&amp;I), no país ou no exterior. O objetivo é aprimorar/desenvolver técnicas e processos, além de adquirir conhecimentos específicos vinculados a projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, localizadas no estado do Espírito Santo.</t>
+          <t>Selecionar propostas para concessão de auxílio financeiro para realização de estágio técnico-científico em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de alunos de pós-graduação e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P pública ou privada, localizada no estado do Espírito Santo. Alunos regularmente matriculados em curso de Mestrado ou Doutorado de IES/P localizada no Espírito Santo e recomendado pela CAPES.</t>
+          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -783,11 +783,7 @@
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>R$ 10.000,00</t>
-        </is>
-      </c>
+      <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
@@ -795,24 +791,24 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada) (Para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
-2026-03-10: Prazo final para envio de dúvidas (1ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada) (Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-03-31 a 2026-04-30: Período de Contratação (1ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/05/2026 a 31/07/2026.)
-2026-04-22: Prazo final para envio de dúvidas (2ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-06-19 a 2026-07-19: Período de Contratação (2ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada) (Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-08-13: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas da última chamada.)
-2026-08-18: Prazo final para envio de dúvidas (3ª Chamada) (Até 2 dias antes do prazo final de submissão. Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar. Para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-10-26 a 2026-11-25: Período de Contratação (3ª Chamada) (Até 30 dias após a publicação do resultado final homologado. Para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
+          <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão da 1ª Chamada.)
+2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
+2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada, até 2 dias antes do prazo final de submissão.)
+2026-03-19 a 2026-03-26: Prazo para interposição de recursos (1ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)
+2026-03-31 a 2026-04-30: Período de contratação (1ª Chamada, até 30 dias após a publicação do resultado final homologado.)
+2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada para estágios com início entre 01/08/2026 a 31/12/2026.)
+2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada, até 2 dias antes do prazo final de submissão.)
+2026-05-22 a 2026-05-29: Prazo para interposição de recursos (2ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)
+2026-06-19 a 2026-07-19: Período de contratação (2ª Chamada, até 30 dias após a publicação do resultado final homologado.)
+2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada para estágios com início entre 04/01/2027 a 30/04/2027.)
+2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada, até 2 dias antes do prazo final de submissão.)
+2026-10-02 a 2026-10-09: Prazo para interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)
+2026-10-26 a 2026-11-25: Período de contratação (3ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas nas plataformas. Cada proponente pode apresentar apenas uma proposta por chamada. Não é permitida a contratação concomitante de projeto de estágio técnico-científico e visita técnico-científica para o mesmo período/chamada. O coordenador pode solicitar o adiamento da data de início do estágio por até 30 dias após a contratação, mediante justificativa. É obrigatório mencionar o apoio da Fapes em todas as publicações ou divulgações relacionadas ao projeto.</t>
+          <t>O edital prevê auxílios financeiros para estágios técnico-científicos com valores que variam de R$ 4.000,00 a R$ 10.000,00 para estágios no Brasil (30 a 90 dias) e de US$ 1.400,00 a US$ 6.500,00 para estágios no exterior (30 a 90 dias), dependendo da duração e da região. Os recursos totais são distribuídos em três chamadas, com R$ 668.000,00 para a 1ª chamada e R$ 666.000,00 para a 2ª e 3ª chamadas, divididos igualmente entre as categorias pesquisador e aluno. A Fapes pode alterar datas e prazos do cronograma. Proponentes só podem submeter uma proposta por chamada e não podem ser contratados concomitantemente para estágio técnico-científico e visita técnico-científica no mesmo período. Saldo de recursos não utilizados em uma chamada pode ser aplicado em chamadas subsequentes.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -822,7 +818,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO_CIENTÍFICO.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
@@ -1430,9 +1426,9 @@
           <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 08/07/2026</t>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-10 10:12
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -757,9 +749,9 @@
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 09/07/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-14 09:13
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -516,120 +516,51 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Formação Científica</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 09/2026 - BOLSAS DE ESTÁGIO DOUTORADO SANDUÍCHE</t>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)</t>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Apoiar alunos de doutorado regularmente matriculados em programas de pós-graduação do Espírito Santo para a realização de estágio de pesquisa no exterior. O objetivo é proporcionar aprofundamento teórico, coleta e/ou tratamento de dados, ou desenvolvimento parcial da tese, visando ao intercâmbio científico e ao aprimoramento da qualificação acadêmica, com a concessão de bolsa na modalidade Doutorado Sanduíche.</t>
+          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Alunos de doutorado regularmente matriculados em Programas de Pós-graduação stricto sensu, recomendados pela CAPES e vinculados a instituições de ensino superior e/ou pesquisa (IES/P) públicas ou privadas no Espírito Santo. Os proponentes devem ser brasileiros ou estrangeiros com autorização de residência, residentes no Espírito Santo, sem título de doutor, com currículo Lattes atualizado, cursando entre o 13º e o 42º mês do doutorado (com pelo menos seis meses restantes para a conclusão após o estágio no exterior), com proficiência na língua da instituição de destino, e com anuência do orientador, supervisor no exterior, e coordenador do PPG. Não devem ter realizado mobilidade acadêmica no exterior com auxílio da Fapes nos últimos 12 meses, nem ter sido contemplados com bolsa de Doutorado Sanduíche da Fapes, Capes ou CNPq anteriormente, e devem estar adimplentes junto à Fapes.</t>
+          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="n"/>
+          <t>R$ 2.500.000,00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>US$ 2.700,00</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>bolsas.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-28 a 2026-06-29: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão das propostas.)
-2026-04-28 a 2026-07-02: Prazo para dúvidas e informações (Até 2 dias úteis antecedentes ao término da submissão das propostas.)
-2026-07-06: Submissão das propostas (Até as 17h59.)
-2026-07-28 a 2026-08-03: Prazo para recurso (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação.)
-2026-10-09 a 2026-10-16: Prazo para recurso (classificação) (Até 5 dias úteis após a divulgação do resultado preliminar de classificação.)
-2026-11-01: Contratação dos projetos (Inclui a assinatura eletrônica do Termo de Outorga e o envio de documentos pessoais, com datas a serem divulgadas no resultado homologado.)</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>A duração do estágio de doutorado sanduíche é de, no mínimo, 6 e, no máximo, 12 meses. Os valores das bolsas mensais variam de US$ 1.100,00 a US$ 1.800,00, dependendo do país de destino. O auxílio instalação é equivalente a uma mensalidade da bolsa. O auxílio seguro-saúde é limitado a US$ 90,00 por mês de bolsa, e o auxílio deslocamento é limitado a R$ 12.000,00. A conversão da moeda estrangeira (dólar) ocorre pelo câmbio oficial na data de aprovação do Resultado de Classificação. Taxas administrativas, acadêmicas (tuition &amp; fees), de bancada (bench fees) e adicional dependente não são cobertas. Não é permitida a alteração da instituição de destino ou do supervisor após a submissão da proposta. O prazo de vigência do instrumento de contratação é de 16 meses, improrrogáveis, e o proponente deve realizar o deslocamento dentro desse período. As atividades devem ser realizadas presencialmente na instituição de destino. Para o pagamento integral da mensalidade, o bolsista deve ter executado as atividades por no mínimo 16 dias no mês. O beneficiário tem 16 meses a partir do início da vigência do Termo de Outorga para iniciar e finalizar a bolsa. A existência de inadimplência do proponente com a Fapes ou com as Fazendas Federal, Estadual e Municipal e a Justiça Trabalhista constitui fator impeditivo para contratação. Para a assinatura eletrônica do Termo de Outorga, o proponente e o gestor institucional da IES/P devem ter cadastro ativo no portal 'Acesso Cidadão'.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL%20FAPES%20N°%2009.2026%20-%20BDS.pdf</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>formacao_cientifica/EDITAL_FAPES_No_09_2026_-_BOLSAS_DE_ESTÁGIO_DOUTORADO_SANDUÍCHE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.500.000,00</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>US$ 2.700,00</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -644,70 +575,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -722,66 +653,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-07-19: Período de contratação (2ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para realização de estágio técnico-científico em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de alunos de pós-graduação e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão da 1ª Chamada.)
 2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -798,70 +729,70 @@
 2026-10-26 a 2026-11-25: Período de contratação (3ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O edital prevê auxílios financeiros para estágios técnico-científicos com valores que variam de R$ 4.000,00 a R$ 10.000,00 para estágios no Brasil (30 a 90 dias) e de US$ 1.400,00 a US$ 6.500,00 para estágios no exterior (30 a 90 dias), dependendo da duração e da região. Os recursos totais são distribuídos em três chamadas, com R$ 668.000,00 para a 1ª chamada e R$ 666.000,00 para a 2ª e 3ª chamadas, divididos igualmente entre as categorias pesquisador e aluno. A Fapes pode alterar datas e prazos do cronograma. Proponentes só podem submeter uma proposta por chamada e não podem ser contratados concomitantemente para estágio técnico-científico e visita técnico-científica no mesmo período. Saldo de recursos não utilizados em uma chamada pode ser aplicado em chamadas subsequentes.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -875,19 +806,89 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
+          <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -899,7 +900,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -909,28 +910,28 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
+          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
+          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>R$ 308.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R$ 12.000,00</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -939,76 +940,6 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
-?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 800.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1027,66 +958,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Submissão de propostas (até as 17h59 via Sigfapes)
 ?: Interposição de recursos (habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1094,66 +1025,66 @@
 ?: Início do processo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O edital oferece pontuação adicional para propostas apresentadas por pessoas com deficiência (PcD), negras, quilombolas, indígenas, trans ou travestis. O prazo de execução dos projetos é de 24 meses. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F por pelo menos 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Serão apoiados 6 projetos por microrregião, com recursos remanescentes distribuídos entre os projetos mais bem classificados, independentemente da microrregião. Propostas que indicarem microrregião coincidente com a instituição de vínculo do proponente concorrerão nos blocos das respectivas microrregiões, enquanto propostas para microrregião distinta concorrerão na ampla concorrência.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
 ?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
@@ -1167,70 +1098,70 @@
 ?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
@@ -1243,70 +1174,70 @@
 ?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1316,70 +1247,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente ou membros da equipe deverão participar de, no mínimo, 80% das oficinas e mentorias em cada fase, sob pena de desclassificação. Propostas com nota final inferior a 70,0 pontos serão desclassificadas em ambas as fases. A Fapes somente considerará despesas/gastos realizados a partir do início da vigência do Termo de Outorga. O não atendimento ao prazo de entrega da documentação completa ou o descumprimento dos requisitos para contratação resultará na perda do direito à contratação.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 250.000,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1391,19 +1322,87 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1414,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1423,32 +1422,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1456,22 +1443,22 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1470,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1491,43 +1478,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1530,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1549,45 +1540,54 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1607,116 +1607,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
-        </is>
-      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-16 09:23
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1661,81 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 16/07/2026</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
+2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
+2026-12-16 a 2026-12-25: Período para interposição de recursos (Resultados Etapa 1) (Janela de 10 dias para recursos)
+2027-01-31: Solicitações (e aprovação) de mudanças entre as etapas 1 e 2
+2027-02-15: Prazo final para submissão de propostas completas (até as 15:00 CET)
+2027-03-06 a 2027-03-15: Período para interposição de recursos (Elegibilidade Etapa 2) (Janela de 10 dias para recursos)
+2027-05-16 a 2027-05-25: Período para interposição de recursos (Resultados Etapa 2) (Janela de 10 dias para recursos)
+2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-17 09:10
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1672,9 +1664,9 @@
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 16/07/2026</t>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-23 09:26
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -833,25 +841,30 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 23/07/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições (Categorias Projetos e Destaque (até 17h59))</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Ele visa valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer profissionais apoiados pela Fapes, e ampliar a divulgação da ciência e inovação no estado."
+Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas e projetos fomentados pela Fundação."</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado.</t>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Ele visa valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer profissionais apoiados pela Fapes, e ampliar a divulgação da ciência e inovação no estado.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas e projetos fomentados pela Fundação.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -871,14 +884,15 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições – Categorias Projetos e Destaque (até as 17h59)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até as 17h59)
-?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
+          <t>2026-06-22 a 2026-07-24: Envio das inscrições (Categorias Projetos e Destaque (até 17h59))
+2026-06-22 a 2026-09-15: Envio das inscrições (Categoria Jornalismo (até 17h59))
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)
+?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias após a publicação do resultado final no DIO-ES)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>É permitida apenas uma inscrição por pessoa neste edital, sendo considerada válida a última enviada dentro do prazo. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. O comparecimento do premiado à cerimônia de premiação é obrigatório, ou deve ser indicado formalmente um representante. A matéria jornalística da Categoria Jornalismo deve ter sido veiculada entre 01/09/2025 e 15/09/2026.</t>
+          <t>Servidores da Fapes e membros do Conselho Científico-Administrativo da Fapes (CCAF), ativos ou que tenham atuado na Fundação no ano de publicação do edital e nos 3 (três) anos anteriores, bem como seus cônjuges, companheiros e parentes até o segundo grau, não podem participar. É permitida apenas uma inscrição por pessoa. Em caso de múltiplas inscrições, apenas a última enviada dentro do prazo será considerada válida. A premiação tem caráter honorífico e eventual, não configurando vínculo empregatício. As 3 (três) propostas/matérias com as maiores notas em cada subcategoria (anteriormente 5) seguem para votação final (Comitê de Especialistas para Projetos e Destaque, e votação popular para Jornalismo).</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-24 09:20
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -843,28 +843,28 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Atualizado - e-mail enviado em 23/07/2026</t>
+          <t>Atualizado - e-mail enviado em 24/07/2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições (Categorias Projetos e Destaque (até 17h59))</t>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. A iniciativa visa valorizar a relevância, o impacto e a aplicabilidade da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes e ampliar a divulgação e popularização da ciência no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Ele visa valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer profissionais apoiados pela Fapes, e ampliar a divulgação da ciência e inovação no estado."
-Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Servidores da Fapes, membros do CCAF (ativos ou que atuaram na Fundação no ano de publicação do edital e nos 3 anos anteriores), e seus cônjuges, companheiros e parentes até o segundo grau não podem participar." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas e projetos fomentados pela Fundação."</t>
+          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Ele visa valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer profissionais apoiados pela Fapes, e ampliar a divulgação da ciência e inovação no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado."
+Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas e projetos fomentados pela Fundação." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados."</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Ele visa valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer profissionais apoiados pela Fapes, e ampliar a divulgação da ciência e inovação no estado.</t>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas e projetos fomentados pela Fundação.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -884,15 +884,14 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-07-24: Envio das inscrições (Categorias Projetos e Destaque (até 17h59))
-2026-06-22 a 2026-09-15: Envio das inscrições (Categoria Jornalismo (até 17h59))
-?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)
-?: Solicitação de pagamento da premiação (Prazo máximo de 90 (noventa) dias após a publicação do resultado final no DIO-ES)</t>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Servidores da Fapes e membros do Conselho Científico-Administrativo da Fapes (CCAF), ativos ou que tenham atuado na Fundação no ano de publicação do edital e nos 3 (três) anos anteriores, bem como seus cônjuges, companheiros e parentes até o segundo grau, não podem participar. É permitida apenas uma inscrição por pessoa. Em caso de múltiplas inscrições, apenas a última enviada dentro do prazo será considerada válida. A premiação tem caráter honorífico e eventual, não configurando vínculo empregatício. As 3 (três) propostas/matérias com as maiores notas em cada subcategoria (anteriormente 5) seguem para votação final (Comitê de Especialistas para Projetos e Destaque, e votação popular para Jornalismo).</t>
+          <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-07-25 09:03
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -841,9 +833,9 @@
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 24/07/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -851,12 +843,7 @@
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Ele visa valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer profissionais apoiados pela Fapes, e ampliar a divulgação da ciência e inovação no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado."
-Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também podem participar profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas e projetos fomentados pela Fundação." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados."</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-01 09:05
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -516,51 +532,190 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 01/08/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+          <t>2026-09-02: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, tecnologia e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>R$ 8.887.500,00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>R$ 10.000,00</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
+2026-09-09: Submissão de propostas (Até as 17h59, via Sistema de Gestão da Fapes)
+?: Prazo para interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
+?: Prazo para interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2027-02-09: Contratação dos projetos selecionados</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Somente as cinco bolsas de Iniciação Científica Júnior (ICJr) são obrigatórias para implementação; as demais modalidades de bolsas (BCO, BTU e ICT) são opcionais. Cada coordenador deve apresentar apenas uma proposta, sendo considerada a última enviada em caso de múltiplas submissões. A Fapes pode alterar datas e prazos do cronograma por necessidade institucional ou reabrir prazos em caso de falhas comprovadas nos sistemas.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/PIC_JR_2027%20-.pdf</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_No_19_2026_-_PIC_JR_2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Formação Científica</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 01/08/2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos de pesquisa que visem contribuir para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil, por meio da concessão de bolsas para estágios de pós-doutorado sênior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica e ampliar a cooperação acadêmica nacional e internacional, em instituições de excelência no país ou no exterior.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores com vínculo formal (mínimo de 20h semanais) em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas, sediadas no estado do Espírito Santo, que sejam docentes permanentes de Programa de Pós-Graduação (PPG) stricto sensu e que atendam aos requisitos de tempo de titulação de doutor (Faixas A, B ou C).</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>R$ 6.000.000,00</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)
+?: Interposição de recursos administrativos (habilitação) (5 dias úteis após a publicação do resultado preliminar de habilitação)
+?: Interposição de recursos administrativos (classificação) (5 dias úteis após a publicação do resultado preliminar de classificação)
+2027-01-18: Contratação das propostas (A partir de)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 16 meses, improrrogáveis, exceto em caso de Advento de Prole. Cada proponente deve apresentar apenas uma proposta, sendo a última enviada considerada. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. As atividades devem ser realizadas presencialmente na Instituição de Destino, sem pesquisa à distância. Não é permitida a alteração da Instituição de Destino ou do Supervisor após a submissão da proposta. O valor mensal da bolsa de POSDOC varia de acordo com o nível da bolsa e localidade, sendo fixado na Tabela de Valores de Bolsas e Auxílios da Fapes, podendo ser alterado por norma regulamentadora. Os itens financiáveis incluem bolsa mensal (6 a 10 meses), auxílio instalação (equivalente a uma bolsa POSDOC), seguro saúde (limitado a R$ 550,00/mês para exterior) e auxílio deslocamento (limitado a R$ 2.500,00 no país e R$ 12.000,00 no exterior), todos por reembolso, exceto a bolsa mensal e auxílio instalação que podem ser antecipados. A concessão de adaptações, tecnologias assistivas ou outros recursos de acessibilidade é avaliada segundo critérios de viabilidade e razoabilidade, desde que solicitadas em até 10 dias do término de submissão das propostas. O estágio de pós-doutorado deve ter duração mínima de 6 meses e máxima de 10 meses. O proponente deve ser o bolsista POSDOC.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/POSDOC_Sênior%20-.pdf</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_No_20_2026_-_BOLSAS_DE_PÓS-DOUTORADO_SÊNIOR.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -575,70 +730,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -653,66 +808,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada, até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para realização de estágio técnico-científico em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de alunos de pós-graduação e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão da 1ª Chamada.)
 2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -729,70 +884,70 @@
 2026-10-26 a 2026-11-25: Período de contratação (3ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O edital prevê auxílios financeiros para estágios técnico-científicos com valores que variam de R$ 4.000,00 a R$ 10.000,00 para estágios no Brasil (30 a 90 dias) e de US$ 1.400,00 a US$ 6.500,00 para estágios no exterior (30 a 90 dias), dependendo da duração e da região. Os recursos totais são distribuídos em três chamadas, com R$ 668.000,00 para a 1ª chamada e R$ 666.000,00 para a 2ª e 3ª chamadas, divididos igualmente entre as categorias pesquisador e aluno. A Fapes pode alterar datas e prazos do cronograma. Proponentes só podem submeter uma proposta por chamada e não podem ser contratados concomitantemente para estágio técnico-científico e visita técnico-científica no mesmo período. Saldo de recursos não utilizados em uma chamada pode ser aplicado em chamadas subsequentes.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -806,140 +961,140 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
 ?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -958,66 +1113,66 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 5.000.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 80.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-07-02: Submissão de propostas (até as 17h59 via Sigfapes)
 ?: Interposição de recursos (habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
@@ -1025,143 +1180,151 @@
 ?: Início do processo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital oferece pontuação adicional para propostas apresentadas por pessoas com deficiência (PcD), negras, quilombolas, indígenas, trans ou travestis. O prazo de execução dos projetos é de 24 meses. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F por pelo menos 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Serão apoiados 6 projetos por microrregião, com recursos remanescentes distribuídos entre os projetos mais bem classificados, independentemente da microrregião. Propostas que indicarem microrregião coincidente com a instituição de vínculo do proponente concorrerão nos blocos das respectivas microrregiões, enquanto propostas para microrregião distinta concorrerão na ampla concorrência.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 01/08/2026</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES)." → "O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa."
+Público-alvo: "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas." → "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais."
+Valor por proposta: "R$ 3.000.000,00" → "Entre R$ 500.000,00 e R$ 3.000.000,00"
+Contato: "duvidas.inovacao@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
+Submissão (nova): Submissão das propostas no SIGFAPES — 2026-08-01 a ?</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 40.000.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
+2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
+?: Prazo de submissão dos recursos administrativos (TRL e Mérito) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
+?: Prazo de submissão dos recursos administrativos (Visita Técnica) (05 (cinco) dias úteis a partir da publicação do resultado preliminar da visita técnica.)
+?: Submissão das documentações para contratação (Até 30 (trinta) dias a partir da publicação do resultado homologado do julgamento de mérito.)
+?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES).</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>?: Impugnação do edital (Até 5 dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo (se houver ciclo definido))
-?: Submissão de propostas (Fluxo contínuo, via SIGFAPES)
-?: Interposição de recursos administrativos da habilitação (05 dias úteis a partir da publicação do resultado preliminar)
-?: Interposição de recursos administrativos da avaliação de TRL e mérito (05 dias úteis a partir da publicação do resultado preliminar)
-?: Interposição de recursos administrativos das visitas técnicas (05 dias úteis a partir da publicação do resultado preliminar da visita técnica)
-?: Submissão de documentação para contratação (Até 30 dias a partir da publicação do resultado homologado do julgamento de mérito)
-?: Informar dados da conta bancária (Até 30 dias após a publicação do Termo de Outorga)
-?: Prestação de contas parcial (1ª) (Até 30 dias após o 8º mês de vigência do Termo de Outorga)
-?: Prestação de contas parcial (2ª) (Até 30 dias após o 16º mês de vigência do Termo de Outorga)
-?: Prestação de contas final (Até 30 dias após o fim do prazo de vigência do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>As resoluções e formulários estão disponíveis no site da FAPES (www.fapes.es.gov.br/resolucoes) e no Sistema SIGFAPES (www.sigfapes.es.gov.br). Empresas proponentes não podem ter sido contratadas nos Editais FAPES nº 07/2024, nº 10/2025 e nº 06/2026. Não é permitido que empresas beneficiadas possuam em seu quadro societário estagiários, funcionários, servidores, colaboradores, dirigentes ou profissionais com vínculo empregatício com a FAPES, incluindo cônjuges, companheiros ou parentes até o segundo grau. As atividades do projeto devem ser realizadas no Espírito Santo, exceto certificação, homologação e testes. É permitida a submissão de apenas uma proposta por empresa. A contratação de bolsistas (DTI, BIPI, AT) é opcional e seus recursos são descontados do valor da subvenção econômica. Não é permitida a contratação de bolsistas com vínculo empregatício com a FAPES ou parentes até o segundo grau.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
@@ -1174,70 +1337,70 @@
 ?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1247,70 +1410,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente ou membros da equipe deverão participar de, no mínimo, 80% das oficinas e mentorias em cada fase, sob pena de desclassificação. Propostas com nota final inferior a 70,0 pontos serão desclassificadas em ambas as fases. A Fapes somente considerará despesas/gastos realizados a partir do início da vigência do Termo de Outorga. O não atendimento ao prazo de entrega da documentação completa ou o descumprimento dos requisitos para contratação resultará na perda do direito à contratação.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>R$ 250.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1322,143 +1485,19 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1509,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1480,45 +1519,53 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1577,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1538,169 +1585,285 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>US$ 18.000,00</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>US$ 6.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
 2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1712,17 +1875,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-02 09:03
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,22 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,18 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -540,9 +524,9 @@
           <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 01/08/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -612,9 +596,9 @@
           <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 01/08/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1207,25 +1191,17 @@
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 01/08/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Promover um significativo aumento da competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação. Os projetos devem ser desenvolvidos por empresas do Espírito Santo em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas, públicas ou privadas, e apresentar aderência aos setores econômicos do Plano de Desenvolvimento de Longo Prazo (ES 500 Anos) ou ao Plano Estadual de Ciência, Tecnologia e Inovação do Espírito Santo (PCTI-ES)." → "O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa."
-Público-alvo: "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, em colaboração com Instituições de Ciência e Tecnologia (ICT) ou Instituições de Ensino Superior (IES) capixabas." → "Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais."
-Valor por proposta: "R$ 3.000.000,00" → "Entre R$ 500.000,00 e R$ 3.000.000,00"
-Contato: "duvidas.inovacao@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br"
-Submissão (nova): Submissão das propostas no SIGFAPES — 2026-08-01 a ?</t>
-        </is>
-      </c>
+          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-04 08:45
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1116,12 +1116,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 16/2026 - UNIVERSAL DE EXTENSÃO</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1129,105 +1129,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Apoiar financeiramente projetos de extensão em diversas áreas temáticas, coordenados por profissionais vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) no Espírito Santo. O objetivo é contribuir para a redução de desigualdades ou vulnerabilidades sociais, promovendo o desenvolvimento socioambiental e/ou econômico nas microrregiões do Estado.</t>
+          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores com titulação mínima de mestre, experiência em projetos de extensão nos últimos 3 anos, vínculo empregatício ou termo de adesão a trabalho voluntário com Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, e que atendam aos demais critérios de elegibilidade do edital.</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>R$ 5.000.000,00</t>
+          <t>R$ 40.000.000,00</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>R$ 80.000,00</t>
+          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, nupex@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-02: Submissão de propostas (até as 17h59 via Sigfapes)
-?: Interposição de recursos (habilitação) (05 dias úteis a partir da publicação do resultado preliminar da habilitação)
-?: Interposição de recursos (análise de mérito) (05 dias úteis a partir da publicação do resultado preliminar do mérito)
-?: Início do processo de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>O edital oferece pontuação adicional para propostas apresentadas por pessoas com deficiência (PcD), negras, quilombolas, indígenas, trans ou travestis. O prazo de execução dos projetos é de 24 meses. É obrigatória a permanência de no mínimo 1 bolsista EXT-E ou EXT-F por pelo menos 22 meses. As propostas devem ser submetidas para desenvolvimento em apenas uma das 10 microrregiões listadas no Quadro 2 do edital. Serão apoiados 6 projetos por microrregião, com recursos remanescentes distribuídos entre os projetos mais bem classificados, independentemente da microrregião. Propostas que indicarem microrregião coincidente com a instituição de vínculo do proponente concorrerão nos blocos das respectivas microrregiões, enquanto propostas para microrregião distinta concorrerão na ampla concorrência.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Universal%20Extensão%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>extensao/EDITAL_FAPES_No_16_2026_-_UNIVERSAL_DE_EXTENSÃO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1237,70 +1170,70 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 10.662.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 355.400,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
 2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
@@ -1313,70 +1246,70 @@
 ?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 30.000,00</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
 ?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
@@ -1386,70 +1319,70 @@
 ?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente ou membros da equipe deverão participar de, no mínimo, 80% das oficinas e mentorias em cada fase, sob pena de desclassificação. Propostas com nota final inferior a 70,0 pontos serão desclassificadas em ambas as fases. A Fapes somente considerará despesas/gastos realizados a partir do início da vigência do Termo de Outorga. O não atendimento ao prazo de entrega da documentação completa ou o descumprimento dos requisitos para contratação resultará na perda do direito à contratação.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 250.000,00</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1461,19 +1394,87 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1486,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1493,32 +1494,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1526,22 +1515,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1542,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1561,43 +1550,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1602,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1619,45 +1612,54 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1671,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1677,56 +1679,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
-        </is>
-      </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1733,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1746,100 +1741,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
+          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>€ 25.000,00 por ano de projeto</t>
+          <t>EUR 100.000,00</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1851,17 +1784,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-05 08:44
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1039,46 +1047,123 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
+          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 500.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>US$ 1.500,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
+2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
+2026-03-04 a 2026-04-09: Submissão de propostas (Até as 17:59h. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
+2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
+?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
+?: Contratação e assinatura do Termo de Outorga (Até 30 dias após a publicação do resultado final homologado. Período específico de assinatura será definido após a homologação.)
+?: Prazo para informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga)
+?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1097,70 +1182,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1170,95 +1255,19 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 10/2026 - DR. EMPREENDEDOR CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Fomentar projetos de pesquisa e desenvolvimento de produtos (bens e serviços) ou processos inovadores, conduzidos por doutores apoiados por Instituições de Ensino Superior ou Pesquisa (IES/P) ou Instituições Científicas, Tecnológicas e de Inovação (ICTs), públicas ou privadas, sediadas no Espírito Santo. O objetivo é transformar ideias inovadoras em empreendimentos potencialmente sustentáveis, promovendo a transferência de conhecimento e tecnologias para o mercado, impulsionando a criação ou o fortalecimento de micro e pequenas empresas (MPEs) de base tecnológica.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Doutores empreendedores, sem vínculo empregatício, que atuem no Estado do Espírito Santo, com ou sem empresa previamente constituída, de qualquer área de conhecimento, interessados em transformar conhecimento científico em soluções inovadoras, promover a criação de novos negócios e fortalecer o ecossistema de inovação capixaba.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 10.662.000,00</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>R$ 355.400,00</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>?: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento do prazo de submissão da 1ª chamada)
-2026-05-04 a 2026-07-07: Período de submissão de propostas (1ª chamada) (Até as 17:59h, via Sigfapes)
-?: Prazo para submissão de recursos administrativos (habilitação - 1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-?: Prazo para submissão de recursos administrativos (mérito - 1ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-2026-10-14 a 2026-12-15: Período de submissão de propostas (2ª chamada) (Até as 17:59h, via Sigfapes)
-?: Processo de contratação (1ª chamada) (Até 5 dias úteis da publicação do resultado homologado)
-?: Prazo para submissão de recursos administrativos (habilitação - 2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-?: Prazo para submissão de recursos administrativos (mérito - 2ª chamada) (5 dias úteis a partir da publicação do resultado preliminar)
-?: Processo de contratação (2ª chamada) (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>As datas do cronograma podem ser alteradas de acordo com o andamento do Edital. É de responsabilidade do proponente acompanhar as atualizações do Edital publicadas no site da FAPES (https://fapes.es.gov.br/) e consequentes alterações no cronograma. Inclusão de item referente à ciência do Núcleo de Inovação Tecnológica (NIT), quando for aplicável. Alteração do item 7.3 C) para que a verificação de vínculo empregatício seja realizada na fase de contratação do projeto. Inclusão da exigência de apresentação da Declaração de Ciência do NIT no ato da contratação, quando aplicável (item 12.6). Inclusão de item referente à definição de responsabilidades quanto ao registro ou depósito de pedido de proteção intelectual (item 19.2). O Anexo III (Declaração de Apoio da Instituição Copartícipe) agora permite que o documento seja assinado por autoridade com competência formalmente delegada. Inclusão do Anexo IX (Modelo de Declaração de Ciência do Núcleo de Inovação Tecnológica - NIT).</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_102026_DR._EMPREENDEDOR_CAPIXABA_-_CORRIGIDO.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_No_10_2026_-_DR._EMPREENDEDOR_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1279,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES N° 11/2026 – PROGRAMA GÊNESIS</t>
+          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1280,109 +1289,36 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)</t>
+          <t>2026-10-02 a 2026-10-09: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa estimular o empreendedorismo e a inovação nas microrregiões Caparaó, Centro-Oeste, Central Sul, Noroeste, Rio Doce e Sudoeste Serrana. O objetivo é oferecer apoio técnico e financeiro a soluções inovadoras com alto potencial de mercado, que possam se transformar em novos negócios ou startups, contribuindo para o desenvolvimento sustentável das regiões.</t>
+          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pessoas físicas com 18 anos ou mais que morem, estudem ou trabalhem em uma das seis microrregiões contempladas pelo edital (Caparaó, Centro-Oeste, Central-Sul, Noroeste, Rio Doce e Sudoeste Serrana) e que necessitem de apoio técnico e financeiro para desenvolver suas ideias.</t>
+          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>R$ 4.500.000,00</t>
+          <t>R$ 9.800.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R$ 30.000,00</t>
+          <t>R$ 250.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-21 a 2026-07-03: Envio da primeira proposta (até as 17h59)
-?: Prazo para recurso administrativo (Fase 1) (Até 5 dias úteis após divulgação do resultado preliminar)
-2026-09-14 a 2026-09-22: Envio da segunda proposta após a 1ª oficina e capacitação (até as 17h59)
-2026-09-21 a 2026-09-30: Apresentação do pitch
-?: Prazo para recurso administrativo (Fase 2) (Até 5 dias úteis após divulgação do resultado preliminar)
-?: Período de contratação (Até 5 dias úteis da publicação do resultado homologado)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo reabrir o prazo para recebimento de propostas em casos de força maior ou falhas comprovadas. O proponente ou membros da equipe deverão participar de, no mínimo, 80% das oficinas e mentorias em cada fase, sob pena de desclassificação. Propostas com nota final inferior a 70,0 pontos serão desclassificadas em ambas as fases. A Fapes somente considerará despesas/gastos realizados a partir do início da vigência do Termo de Outorga. O não atendimento ao prazo de entrega da documentação completa ou o descumprimento dos requisitos para contratação resultará na perda do direito à contratação.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Programa%20Gênesis%202026%20-%20Assinado.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_N°_11_2026_–_PROGRAMA_GÊNESIS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 9.800.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 250.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
 2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
@@ -1394,19 +1330,87 @@
 ?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
         </is>
       </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 05/08/2026</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-06 09:58
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -1282,25 +1282,33 @@
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 06/08/2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 a 2026-10-09: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>2026-06-22 a 2026-08-11: Submissão das propostas no SIGFAPES (Até as 17h59.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável." → "Selecionar e apoiar, através de subvenção econômica, startups capixabas que busquem celebrar parcerias estratégicas com outras startups (nacionais ou internacionais) para a evolução de produtos, serviços ou modelos de negócio. O edital visa a expansão de mercado, inovação, aprimoramento de competências, posicionamento de marca, acesso a financiamentos e impacto socioambiental sustentável."
+Público-alvo: "Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos." → "Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo."
+Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, (27) 3636-1862, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br"
+Submissão (nova): Submissão das propostas no SIGFAPES — 2026-06-22 a 2026-08-11
+Submissão (removida): Submissão das propostas — 2026-06-22 a 2026-08-04</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável.</t>
+          <t>Selecionar e apoiar, através de subvenção econômica, startups capixabas que busquem celebrar parcerias estratégicas com outras startups (nacionais ou internacionais) para a evolução de produtos, serviços ou modelos de negócio. O edital visa a expansão de mercado, inovação, aprimoramento de competências, posicionamento de marca, acesso a financiamentos e impacto socioambiental sustentável.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos.</t>
+          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1315,24 +1323,24 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, (27) 3636-1862, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-08-04: Submissão das propostas (Até às 17h59, via SIGFAPES)
-2026-07-28: Prazo para impugnação do edital (Até 5 (cinco) dias úteis antes da data final de submissão das propostas.)
-2026-10-02 a 2026-10-09: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)
-?: Constituição de empresa e atualização documental no SIGFAPES (Proponentes aprovados) (Para proponentes aprovados sem empresa constituída. Período a ser definido pela FAPES após homologação do resultado.)
-?: Assinatura do Termo de Outorga e Projeto Aprovado (Proponentes aprovados) (Até às 17h. Período a ser definido pela FAPES após homologação do resultado.)
-?: Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Até às 17h. Período a ser definido pela FAPES após homologação do resultado. Envio via e-Flow Formulário nº 26.)
-2026-12-01 a 2026-12-31: Informar dados da conta bancária aberta (Prazo de 30 dias a partir do início da vigência do Termo de Outorga.)
-?: Período de contratação das propostas suplentes (Até às 17h. Período a ser definido pela FAPES, se aplicável.)</t>
+          <t>2026-06-22 a 2026-08-11: Submissão das propostas no SIGFAPES (Até as 17h59.)
+?: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)
+?: Disponibilização de documentos para contratação (para projetos aprovados) (Até as 17h. Coordenador(a) deverá disponibilizar documentos atualizados e válidos no SIGFAPES. Datas são placeholders (XX.XX.20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
+?: Abertura de empresa e atualização documental (para propostas aprovadas sem empresas constituídas) (Até as 17h. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
+?: Assinatura do Termo de Outorga e do Projeto Aprovado (Até as 17h. Assinatura eletrônica via E-DOCS. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
+?: Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Até as 17h. Envio do e-Flow Formulário nº 26. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
+?: Informar dados da conta bancária à Fapes (Prazo de 30 (trinta) dias a partir do início da vigência do Termo de Outorga e publicação da contratação no DIO-ES.)
+?: Período de contratação das propostas suplentes (Até as 17h, se aplicável. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração. É responsabilidade do coordenador da parceria acompanhar as atualizações do Edital. O valor máximo por proposta é R$ 250.000,00, mas varia por modalidade (R$ 120.000,00 para Modalidade I, R$ 150.000,00 para Modalidade II, R$ 250.000,00 para Modalidade III). Se o número de propostas previstas não for alcançado, os recursos remanescentes serão redirecionados para propostas suplentes. A startup classificada deverá depositar 5% do valor contratado como contrapartida financeira. A startup proponente e a parceira não podem ser caracterizadas como holding. Cada proponente pode submeter até 2 propostas, desde que em modalidades e com parceiros diferentes. Em caso de múltiplas submissões para a mesma faixa, apenas a última será considerada. É vedada a submissão de propostas com as mesmas startups alternando papéis de proponente e parceira. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. A contratação está condicionada à comprovação de adimplência fiscal e previdenciária do coordenador e da empresa. Para critérios de contratação, as empresas deverão estar localizadas obrigatoriamente na microrregião do Caparaó do Espírito Santo, sendo este endereço verificado pelo cartão de CNPJ, na etapa de Assinatura do Termo de Outorga.</t>
+          <t>As datas do cronograma são passíveis de alteração de acordo com o andamento do Edital. É de responsabilidade do coordenador da parceria acompanhar as atualizações do Edital publicadas no site da FAPES e consequentes alterações no cronograma. Se o número de propostas previstas para contratação nas modalidades I, II ou III não for alcançado, os recursos financeiros remanescentes serão redirecionados para a contratação das propostas suplentes nas modalidades I, II e III respectivamente, respeitando a ordem de classificação. A startup proponente e a startup parceira não poderão ser caracterizadas como holding, nem possuir participação acionária ou societária majoritária de uma das startups na outra, ou participação de um dos sócios em ambas que configure controle societário, influência dominante ou dependência societária. É vedada a submissão de propostas contendo as mesmas startups participantes com alternância das funções de proponente e parceira entre propostas distintas. Caso seja identificada essa situação, ambas as propostas serão inabilitadas. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Critérios de desempate para propostas com pontuação final igual: 1. Detalhamento dos objetivos da parceria; 2. Experiência da startup proponente; 3. Detalhamento das entregas; 4. Benefícios e resultados esperados; 5. Apresentação das propostas; 6. Justificativa para parceria; 7. Riscos, restrições e viabilidade técnica; 8. Características das empresas; 9. Proposta submetida no Sistema SIGFAPES com mais antecedência. A adimplência do coordenador(a) ou da empresa com a Fapes, Fazendas Federal, Estadual e Municipal e Justiça Trabalhista é fator impeditivo para contratação. A apresentação de comprovante de pagamento ou parcelamento do débito NÃO será aceito pela Fapes; é necessário apresentar Certidão Negativa ou Certidão Positiva com efeito de Negativa. Constitui fator impeditivo à liberação das parcelas, a qualquer tempo, a existência de inadimplência, de natureza financeira ou técnica, da Empresa Beneficiária com a FAPES e com as esferas municipal, estadual e federal, além da Justiça Trabalhista e do FGTS. A startup proponente será a principal responsável pelas entregas pactuadas na parceria, devendo as startups parceiras participarem efetivamente da execução do projeto. A análise da prestação de contas técnica e financeira final dos projetos deverá ser concluída pela Fapes no prazo de até um ano, a contar da data de sua entrega, prorrogável por igual período, mediante justificativa. Qualquer cidadão poderá requerer, fundamentadamente, a impugnação deste edital, por meio do Formulário de Impugnação de Edital em até 5 (cinco) dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo no SIGFAPES. Não será permitido pela FAPES que a empresa proponente outorgada, utilizando o recurso da subvenção econômica ou contrapartida, contrate a empresa parceira para: realização de serviços de terceiros, aquisição de bens de capital, aquisição de materiais de consumo, entre outros.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1357,9 +1365,9 @@
           <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 05/08/2026</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-07 08:45
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -663,51 +663,122 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Pesquisa</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 07/08/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+          <t>2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos visa apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. Seu objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, bem como consolidar grupos de referência em áreas do conhecimento e setores estratégicos do estado.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores doutores, além do coordenador, com representação da Instituição Executora, outras IES/P capixabas, IES/P de fora do estado ou do País, e um pesquisador vinculado a órgão ou instituição pública estadual.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000.000,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.200.000,00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 a 2026-09-14: Envio da proposta e documentos (via SigFapes, até as 17h59)
+2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
+2026-09-25 a 2026-10-01: Prazo para recorrer (habilitação) (5 dias úteis após o resultado preliminar da habilitação)
+2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após o resultado preliminar de análise de mérito)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional. Cada coordenador pode apresentar apenas uma proposta, sendo a última enviada considerada válida em caso de múltiplas submissões. A etapa de habilitação é eliminatória. Serão classificadas apenas as propostas com nota final igual ou superior a 70,0 pontos. Em caso de empate na nota final, o desempate será pela maior nota nos critérios de avaliação (item 3.2.1) na ordem apresentada, e persistindo o empate, pela proposta submetida primeiro. A proposta aprovada não poderá ser alterada no momento da contratação. O projeto aprovado não será contratado se o coordenador não cumprir as condições, apresentar informações falsas ou não atender aos requisitos, resultando na convocação de suplentes. A Fapes não reivindicará direitos de participação na propriedade intelectual sobre as pesquisas e projetos apoiados. É obrigatória a menção clara e destacada do apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>US$ 2.700,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
 2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
@@ -722,70 +793,70 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 2.500.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
 2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
@@ -800,66 +871,66 @@
 ?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada, até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para realização de estágio técnico-científico em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de alunos de pós-graduação e apoiar os Programas de Pós-graduação do estado.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão da 1ª Chamada.)
 2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
@@ -876,70 +947,70 @@
 2026-10-26 a 2026-11-25: Período de contratação (3ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O edital prevê auxílios financeiros para estágios técnico-científicos com valores que variam de R$ 4.000,00 a R$ 10.000,00 para estágios no Brasil (30 a 90 dias) e de US$ 1.400,00 a US$ 6.500,00 para estágios no exterior (30 a 90 dias), dependendo da duração e da região. Os recursos totais são distribuídos em três chamadas, com R$ 668.000,00 para a 1ª chamada e R$ 666.000,00 para a 2ª e 3ª chamadas, divididos igualmente entre as categorias pesquisador e aluno. A Fapes pode alterar datas e prazos do cronograma. Proponentes só podem submeter uma proposta por chamada e não podem ser contratados concomitantemente para estágio técnico-científico e visita técnico-científica no mesmo período. Saldo de recursos não utilizados em uma chamada pode ser aplicado em chamadas subsequentes.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 2.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 2.600,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
 2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
@@ -953,140 +1024,140 @@
 2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
 ?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -1100,70 +1171,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
 2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
@@ -1182,70 +1253,70 @@
 ?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1255,78 +1326,70 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 06/08/2026</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-11: Submissão das propostas no SIGFAPES (Até as 17h59.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Selecionar e apoiar, através de subvenção econômica (recursos não reembolsáveis), startups capixabas que busquem celebrar parcerias estratégicas com outras startups (do Espírito Santo, nacionais ou internacionais). O objetivo é impulsionar a expansão de mercado, inovação tecnológica, aprimoramento de produtos/serviços, acesso a novos canais de distribuição, atração de talentos, posicionamento de marca e mercado, acesso a financiamento e impacto socioambiental sustentável." → "Selecionar e apoiar, através de subvenção econômica, startups capixabas que busquem celebrar parcerias estratégicas com outras startups (nacionais ou internacionais) para a evolução de produtos, serviços ou modelos de negócio. O edital visa a expansão de mercado, inovação, aprimoramento de competências, posicionamento de marca, acesso a financiamentos e impacto socioambiental sustentável."
-Público-alvo: "Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo, com CNPJ constituído há no mínimo 1 ano e no máximo 10 anos." → "Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo."
-Contato: "duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br" → "duvidas.inovacao@fapes.es.gov.br, (27) 3636-1862, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br"
-Submissão (nova): Submissão das propostas no SIGFAPES — 2026-06-22 a 2026-08-11
-Submissão (removida): Submissão das propostas — 2026-06-22 a 2026-08-04</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Selecionar e apoiar, através de subvenção econômica, startups capixabas que busquem celebrar parcerias estratégicas com outras startups (nacionais ou internacionais) para a evolução de produtos, serviços ou modelos de negócio. O edital visa a expansão de mercado, inovação, aprimoramento de competências, posicionamento de marca, acesso a financiamentos e impacto socioambiental sustentável.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 9.800.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 250.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, (27) 3636-1862, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-11: Submissão das propostas no SIGFAPES (Até as 17h59.)
 ?: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)
@@ -1338,87 +1401,19 @@
 ?: Período de contratação das propostas suplentes (Até as 17h, se aplicável. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital.)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>As datas do cronograma são passíveis de alteração de acordo com o andamento do Edital. É de responsabilidade do coordenador da parceria acompanhar as atualizações do Edital publicadas no site da FAPES e consequentes alterações no cronograma. Se o número de propostas previstas para contratação nas modalidades I, II ou III não for alcançado, os recursos financeiros remanescentes serão redirecionados para a contratação das propostas suplentes nas modalidades I, II e III respectivamente, respeitando a ordem de classificação. A startup proponente e a startup parceira não poderão ser caracterizadas como holding, nem possuir participação acionária ou societária majoritária de uma das startups na outra, ou participação de um dos sócios em ambas que configure controle societário, influência dominante ou dependência societária. É vedada a submissão de propostas contendo as mesmas startups participantes com alternância das funções de proponente e parceira entre propostas distintas. Caso seja identificada essa situação, ambas as propostas serão inabilitadas. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Critérios de desempate para propostas com pontuação final igual: 1. Detalhamento dos objetivos da parceria; 2. Experiência da startup proponente; 3. Detalhamento das entregas; 4. Benefícios e resultados esperados; 5. Apresentação das propostas; 6. Justificativa para parceria; 7. Riscos, restrições e viabilidade técnica; 8. Características das empresas; 9. Proposta submetida no Sistema SIGFAPES com mais antecedência. A adimplência do coordenador(a) ou da empresa com a Fapes, Fazendas Federal, Estadual e Municipal e Justiça Trabalhista é fator impeditivo para contratação. A apresentação de comprovante de pagamento ou parcelamento do débito NÃO será aceito pela Fapes; é necessário apresentar Certidão Negativa ou Certidão Positiva com efeito de Negativa. Constitui fator impeditivo à liberação das parcelas, a qualquer tempo, a existência de inadimplência, de natureza financeira ou técnica, da Empresa Beneficiária com a FAPES e com as esferas municipal, estadual e federal, além da Justiça Trabalhista e do FGTS. A startup proponente será a principal responsável pelas entregas pactuadas na parceria, devendo as startups parceiras participarem efetivamente da execução do projeto. A análise da prestação de contas técnica e financeira final dos projetos deverá ser concluída pela Fapes no prazo de até um ano, a contar da data de sua entrega, prorrogável por igual período, mediante justificativa. Qualquer cidadão poderá requerer, fundamentadamente, a impugnação deste edital, por meio do Formulário de Impugnação de Edital em até 5 (cinco) dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo no SIGFAPES. Não será permitido pela FAPES que a empresa proponente outorgada, utilizando o recurso da subvenção econômica ou contrapartida, contrate a empresa parceira para: realização de serviços de terceiros, aquisição de bens de capital, aquisição de materiais de consumo, entre outros.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1425,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1440,53 +1435,53 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1493,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1506,20 +1501,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1527,22 +1534,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1561,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1562,47 +1569,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1617,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1624,167 +1627,227 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>US$ 18.000,00</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>US$ 6.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
 2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1796,17 +1859,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-08 08:28
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -671,9 +663,9 @@
           <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 07/08/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-11 08:44
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -1677,11 +1677,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)</t>
-        </is>
-      </c>
+      <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-12 08:45
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1337,12 +1337,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Chamadas Internacionais</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 18/2026 - PARCERIAS ENTRE STARTUPS</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1352,60 +1352,53 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-08-11: Submissão das propostas no SIGFAPES (Até as 17h59.)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Selecionar e apoiar, através de subvenção econômica, startups capixabas que busquem celebrar parcerias estratégicas com outras startups (nacionais ou internacionais) para a evolução de produtos, serviços ou modelos de negócio. O edital visa a expansão de mercado, inovação, aprimoramento de competências, posicionamento de marca, acesso a financiamentos e impacto socioambiental sustentável.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Startups (pessoas jurídicas) com faturamento bruto anual de até R$ 16.000.000,00, sediadas no Espírito Santo.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>R$ 9.800.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 250.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, (27) 3636-1862, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br, geinov@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-08-11: Submissão das propostas no SIGFAPES (Até as 17h59.)
-?: Prazo de submissão dos recursos administrativos (05 (cinco) dias úteis a partir da publicação do resultado preliminar da habilitação.)
-?: Disponibilização de documentos para contratação (para projetos aprovados) (Até as 17h. Coordenador(a) deverá disponibilizar documentos atualizados e válidos no SIGFAPES. Datas são placeholders (XX.XX.20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
-?: Abertura de empresa e atualização documental (para propostas aprovadas sem empresas constituídas) (Até as 17h. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
-?: Assinatura do Termo de Outorga e do Projeto Aprovado (Até as 17h. Assinatura eletrônica via E-DOCS. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
-?: Registro da Lista de Checagem de Documentação de Contratação em CT&amp;I (Até as 17h. Envio do e-Flow Formulário nº 26. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital, ocorrendo após a homologação e antes do início da vigência.)
-?: Informar dados da conta bancária à Fapes (Prazo de 30 (trinta) dias a partir do início da vigência do Termo de Outorga e publicação da contratação no DIO-ES.)
-?: Período de contratação das propostas suplentes (Até as 17h, se aplicável. Datas são placeholders (DE XX/XX/20XX a XX/XX/20XX) no edital.)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>As datas do cronograma são passíveis de alteração de acordo com o andamento do Edital. É de responsabilidade do coordenador da parceria acompanhar as atualizações do Edital publicadas no site da FAPES e consequentes alterações no cronograma. Se o número de propostas previstas para contratação nas modalidades I, II ou III não for alcançado, os recursos financeiros remanescentes serão redirecionados para a contratação das propostas suplentes nas modalidades I, II e III respectivamente, respeitando a ordem de classificação. A startup proponente e a startup parceira não poderão ser caracterizadas como holding, nem possuir participação acionária ou societária majoritária de uma das startups na outra, ou participação de um dos sócios em ambas que configure controle societário, influência dominante ou dependência societária. É vedada a submissão de propostas contendo as mesmas startups participantes com alternância das funções de proponente e parceira entre propostas distintas. Caso seja identificada essa situação, ambas as propostas serão inabilitadas. Propostas com Nota Final inferior a 70 pontos serão desclassificadas. Critérios de desempate para propostas com pontuação final igual: 1. Detalhamento dos objetivos da parceria; 2. Experiência da startup proponente; 3. Detalhamento das entregas; 4. Benefícios e resultados esperados; 5. Apresentação das propostas; 6. Justificativa para parceria; 7. Riscos, restrições e viabilidade técnica; 8. Características das empresas; 9. Proposta submetida no Sistema SIGFAPES com mais antecedência. A adimplência do coordenador(a) ou da empresa com a Fapes, Fazendas Federal, Estadual e Municipal e Justiça Trabalhista é fator impeditivo para contratação. A apresentação de comprovante de pagamento ou parcelamento do débito NÃO será aceito pela Fapes; é necessário apresentar Certidão Negativa ou Certidão Positiva com efeito de Negativa. Constitui fator impeditivo à liberação das parcelas, a qualquer tempo, a existência de inadimplência, de natureza financeira ou técnica, da Empresa Beneficiária com a FAPES e com as esferas municipal, estadual e federal, além da Justiça Trabalhista e do FGTS. A startup proponente será a principal responsável pelas entregas pactuadas na parceria, devendo as startups parceiras participarem efetivamente da execução do projeto. A análise da prestação de contas técnica e financeira final dos projetos deverá ser concluída pela Fapes no prazo de até um ano, a contar da data de sua entrega, prorrogável por igual período, mediante justificativa. Qualquer cidadão poderá requerer, fundamentadamente, a impugnação deste edital, por meio do Formulário de Impugnação de Edital em até 5 (cinco) dias úteis antes da data final fixada para submissão das propostas do primeiro Ciclo no SIGFAPES. Não será permitido pela FAPES que a empresa proponente outorgada, utilizando o recurso da subvenção econômica ou contrapartida, contrate a empresa parceira para: realização de serviços de terceiros, aquisição de bens de capital, aquisição de materiais de consumo, entre outros.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_18-2026_-_PARCERIAS_ENTRE_STARTUPS%20(1).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_18_2026_-_PARCERIAS_ENTRE_STARTUPS.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1410,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1427,53 +1420,53 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1478,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1493,32 +1486,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1526,22 +1507,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1534,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1561,43 +1542,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1594,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1617,47 +1602,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1659,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1681,161 +1671,96 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1847,17 +1772,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-19 08:24
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)</t>
+          <t>2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)</t>
+          <t>2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -897,7 +897,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada, até 2 dias antes do prazo final de submissão.)</t>
+          <t>2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)</t>
+          <t>2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-20 08:26
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1182,12 +1182,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1197,118 +1197,36 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)</t>
+          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade.</t>
+          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>R$ 800.000,00</t>
+          <t>R$ 40.000.000,00</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>US$ 1.500,00</t>
+          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-18: Prazo para impugnação do Edital (Até 5 dias úteis antes do encerramento do prazo de submissão da primeira chamada.)
-2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59)
-?: Interposição de recursos - 1ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-04-30: Contratação / Assinatura do TO e envio de documentos - 1ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59)
-?: Interposição de recursos - 2ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-07-30: Contratação / Assinatura do TO e envio de documentos - 2ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59)
-?: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-10-30: Contratação / Assinatura do TO e envio de documentos - 3ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59)
-?: Interposição de recursos - 4ª Chamada (5 dias úteis após a publicação do resultado preliminar)
-2026-12-30: Contratação / Assinatura do TO e envio de documentos - 4ª Chamada (Até 30 dias após a publicação do resultado final homologado.)
-?: Informar dados da conta bancária (Até 30 dias a partir do início da vigência do TO (publicação no DIO-ES).)
-?: Prestação de contas (Até 30 dias após o término de vigência do Termo de Outorga.)</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. Cada coordenador pode apresentar apenas uma proposta a este edital, sendo considerada a última enviada em caso de múltiplas submissões. O apoio financeiro é exclusivo para pagamento de taxa de publicação de artigos técnico-científicos. Se houver saldo de recursos financeiros não utilizados em uma chamada, o valor poderá ser aplicado na chamada subsequente. É obrigatório mencionar o apoio da Fapes de forma clara e visível em todas as publicações ou divulgações relacionadas ao projeto.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1318,19 +1236,87 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1328,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1352,53 +1338,53 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1396,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1418,32 +1404,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1451,22 +1425,22 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1452,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1486,43 +1460,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1512,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1542,47 +1520,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1577,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1606,48 +1589,45 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1639,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1667,100 +1647,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
+          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>€ 25.000,00 por ano de projeto</t>
+          <t>EUR 100.000,00</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1772,17 +1690,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-21 08:26
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -741,7 +741,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)</t>
+          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)</t>
+          <t>2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -897,7 +897,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada para estágios com início entre 04/01/2027 a 30/04/2027.)</t>
+          <t>2026-10-02 a 2026-10-09: Prazo para interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -973,7 +973,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)</t>
+          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-22 08:19
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -731,38 +731,38 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 02/2026 - PARTICIPAÇÃO EM EVENTOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
+          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>O objetivo geral deste edital é selecionar e apoiar financeiramente pesquisadores e alunos para participação em eventos técnico-científicos de curta duração. Visa divulgar os resultados de projetos de pesquisa, desenvolvimento e inovação (P, D&amp;I) desenvolvidos em instituições de ensino superior e/ou pesquisa, públicas ou privadas, localizadas no Estado do Espírito Santo.</t>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores e alunos de pós-graduação vinculados a Instituição de Ensino e/ou Pesquisa (IES/P), pública ou privada, localizada no estado do Espírito Santo.</t>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.500.000,00</t>
+          <t>R$ 308.000,00</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>US$ 2.700,00</t>
+          <t>R$ 12.000,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -772,32 +772,24 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>2026-02-27: Prazo para solicitação de atendimento especializado (até 10 dias antes do prazo final de submissão da 1ª Chamada)
-2026-03-02: Prazo para impugnação do edital (até 5 dias úteis antes do prazo final de submissão da 1ª Chamada)
-2026-02-06 a 2026-03-09: Período de submissão (1ª Chamada) (eventos com início entre 01/05/2026 a 31/07/2026, até as 17h59)
-2026-03-07: Prazo para envio de dúvidas (1ª Chamada) (até 2 dias antes do prazo final de submissão da 1ª Chamada)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 1ª Chamada)
-2026-03-17 a 2026-04-24: Período de submissão (2ª Chamada) (eventos com início entre 01/08/2026 a 31/12/2026)
-2026-04-22: Prazo para envio de dúvidas (2ª Chamada) (até 2 dias antes do prazo final de submissão da 2ª Chamada)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 2ª Chamada)
-2026-07-01 a 2026-08-20: Período de submissão (3ª Chamada) (eventos com início entre 04/01/2027 a 30/04/2027)
-2026-08-18: Prazo para envio de dúvidas (3ª Chamada) (até 2 dias antes do prazo final de submissão da 3ª Chamada)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar da 3ª Chamada)</t>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
+2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>O valor total do edital será distribuído em três chamadas. O valor por proposta é fixo e varia conforme o local do evento: R$ 1.800,00 para eventos no Brasil (exceto Espírito Santo), US$ 1.400,00 para América Central ou América do Sul, US$ 2.300,00 para América do Norte e US$ 2.700,00 para outros continentes. A Fapes pode alterar as datas e prazos do cronograma. Cada proponente pode apresentar apenas uma proposta por chamada. O prazo para informar dados bancários é de até 30 dias corridos após o início da vigência do Termo de Outorga. O prazo para envio da prestação de contas é de até 30 dias após o término da vigência do Termo de Outorga. A contratação das propostas aprovadas ocorrerá em até 30 dias após a publicação do resultado final homologado. O envio do comprovante de aceite do trabalho é condicional para o repasse do recurso e deve ser feito até 15 dias antes do evento.</t>
+          <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_02-2026-Participação_Evento_Técnico_Científico.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_02_2026_-_PARTICIPAÇÃO_EM_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -809,7 +801,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 03/2026 - ORGANIZAÇÃO DE EVENTOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -819,337 +811,36 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)</t>
+          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa selecionar propostas para conceder apoio financeiro a pesquisadores de nível superior. O objetivo é fomentar a organização de eventos técnico-científicos de curta duração, como congressos, simpósios e seminários, a serem realizados no Espírito Santo.</t>
+          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de nível superior vinculados a Instituição de Ensino Superior e/ou Pesquisa (IES/P), pública ou privada sem fins lucrativos, localizada no estado do Espírito Santo.</t>
+          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>R$ 2.500.000,00</t>
+          <t>R$ 500.000,00</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Varia de R$ 10.000,00 a R$ 35.000,00</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
+          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-02: Prazo para impugnação do edital (Até 5 dias úteis antes do prazo final de submissão da 1ª chamada)
-2026-02-06 a 2026-03-09: 1ª Chamada - Período de submissão de propostas (Eventos com início entre 01/05/2026 a 31/07/2026, até 17h59)
-2026-03-07: 1ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 1ª chamada)
-2026-03-20 a 2026-03-26: 1ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-2026-03-17 a 2026-04-24: 2ª Chamada - Período de submissão de propostas (Eventos com início entre 01/08/2026 a 31/12/2026)
-2026-04-22: 2ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 2ª chamada)
-2026-05-23 a 2026-05-29: 2ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-2026-07-01 a 2026-08-20: 3ª Chamada - Período de submissão de propostas (Eventos com início entre 04/01/2027 a 30/04/2027)
-2026-08-18: 3ª Chamada - Prazo para envio de dúvidas (Até 2 dias antes do prazo final de submissão da 3ª chamada)
-2026-10-03 a 2026-10-09: 3ª Chamada - Prazo para interposição de recursos (5 dias úteis após a publicação do resultado preliminar)
-?: Contratação das propostas aprovadas (Até 30 dias após a publicação do resultado final homologado para cada chamada. As datas exatas serão publicadas posteriormente.)</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>O valor do auxílio financeiro é fixo e varia de acordo com o nível do evento: R$ 10.000,00 para Estadual/Regional, R$ 20.000,00 para Nacional e R$ 35.000,00 para Internacional. A Fapes pode alterar as datas e os prazos do cronograma por necessidade ou decisão institucional. Cada proponente pode apresentar apenas uma proposta por chamada. Caso envie mais de uma, será considerada apenas a última enviada. O proponente que já tiver sido contratado neste edital não poderá submeter nova proposta. O evento deve ter duração máxima de 15 dias, consecutivos ou não, e ser chancelado por entidade/sociedade conforme o nível do evento (nacional ou internacional). Os recursos financeiros estão distribuídos por chamada e nível de evento, com possibilidade de remanejamento de saldos não utilizados entre níveis e chamadas subsequentes. É obrigatório mencionar o apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto. A data de início do apoio poderá ser adiada, após a contratação, em até 12 meses, mediante justificativa.</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_03_2026_Organização_Eventos_Técnico-Científicos.pdf</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_03_2026_-_ORGANIZAÇÃO_DE_EVENTOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 04/2026 - ESTÁGIO TÉCNICO-CIENTÍFICO</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-02 a 2026-10-09: Prazo para interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para realização de estágio técnico-científico em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, adquirir conhecimentos específicos para projetos de PD&amp;I no Espírito Santo, estimular o intercâmbio de conhecimentos, a formação de alunos de pós-graduação e apoiar os Programas de Pós-graduação do estado.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas localizadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P localizadas no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-05: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de submissão da 1ª Chamada.)
-2026-02-09 a 2026-03-12: Período de submissão de propostas (1ª Chamada para estágios com início entre 01/05/2026 a 31/07/2026, até as 17h59.)
-2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada, até 2 dias antes do prazo final de submissão.)
-2026-03-19 a 2026-03-26: Prazo para interposição de recursos (1ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)
-2026-03-31 a 2026-04-30: Período de contratação (1ª Chamada, até 30 dias após a publicação do resultado final homologado.)
-2026-03-17 a 2026-04-24: Período de submissão de propostas (2ª Chamada para estágios com início entre 01/08/2026 a 31/12/2026.)
-2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada, até 2 dias antes do prazo final de submissão.)
-2026-05-22 a 2026-05-29: Prazo para interposição de recursos (2ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)
-2026-06-19 a 2026-07-19: Período de contratação (2ª Chamada, até 30 dias após a publicação do resultado final homologado.)
-2026-07-01 a 2026-08-20: Período de submissão de propostas (3ª Chamada para estágios com início entre 04/01/2027 a 30/04/2027.)
-2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada, até 2 dias antes do prazo final de submissão.)
-2026-10-02 a 2026-10-09: Prazo para interposição de recursos (3ª Chamada, 5 dias úteis após a publicação do resultado preliminar.)
-2026-10-26 a 2026-11-25: Período de contratação (3ª Chamada, até 30 dias após a publicação do resultado final homologado.)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>O edital prevê auxílios financeiros para estágios técnico-científicos com valores que variam de R$ 4.000,00 a R$ 10.000,00 para estágios no Brasil (30 a 90 dias) e de US$ 1.400,00 a US$ 6.500,00 para estágios no exterior (30 a 90 dias), dependendo da duração e da região. Os recursos totais são distribuídos em três chamadas, com R$ 668.000,00 para a 1ª chamada e R$ 666.000,00 para a 2ª e 3ª chamadas, divididos igualmente entre as categorias pesquisador e aluno. A Fapes pode alterar datas e prazos do cronograma. Proponentes só podem submeter uma proposta por chamada e não podem ser contratados concomitantemente para estágio técnico-científico e visita técnico-científica no mesmo período. Saldo de recursos não utilizados em uma chamada pode ser aplicado em chamadas subsequentes.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_04_2026_-_Estágio_Técnico_Cientifico.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_04_2026_-_ESTÁGIO_TÉCNICO-CIENTÍFICO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 05/2026 - VISITA TÉCNICO-CIENTÍFICA</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Selecionar propostas para concessão de auxílio financeiro para a realização de visitas técnico-científicas em laboratórios ou centros de pesquisa, desenvolvimento ou inovação (PD&amp;I), no Brasil ou no exterior. O objetivo é aprimorar técnicas, processos e adquirir conhecimentos específicos para projetos de PD&amp;I desenvolvidos em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores com título de doutor ou mestre, com vínculo ativo celetista ou estatutário em IES/P públicas ou privadas no Espírito Santo; e alunos regularmente matriculados em cursos de Mestrado ou Doutorado de IES/P no Espírito Santo, reconhecidos pela CAPES, CNE e/ou MEC.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 2.000.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>US$ 2.600,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2026-02-09 a 2026-03-12: Submissão de propostas (1ª Chamada) (Até as 17h59. Para visitas com início entre 01/05/2026 a 31/07/2026.)
-2026-03-05: Prazo final para impugnação do edital (Até o quinto dia útil que anteceder o prazo final de submissão da 1ª Chamada.)
-2026-03-10: Prazo para envio de dúvidas sobre o edital (1ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-03-17 a 2026-04-24: Submissão de propostas (2ª Chamada) (Para visitas com início entre 01/08/2026 a 31/12/2026.)
-2026-03-26: Prazo para interposição de recursos (1ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
-2026-04-22: Prazo para envio de dúvidas sobre o edital (2ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-05-29: Prazo para interposição de recursos (2ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)
-2026-07-01 a 2026-08-20: Submissão de propostas (3ª Chamada) (Para visitas com início entre 04/01/2027 a 30/04/2027.)
-2026-08-18: Prazo para envio de dúvidas sobre o edital (3ª Chamada) (Até 2 dias antes do prazo final de submissão.)
-2026-10-09: Prazo para interposição de recursos (3ª Chamada) (5 dias úteis após a publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade institucional, podendo reabrir prazos em casos de força maior ou falhas de sistema, com publicidade das alterações. Cada proponente pode submeter apenas uma proposta por chamada; em caso de múltiplas submissões, apenas a última será considerada. Proponentes já contratados neste edital não poderão submeter nova proposta. Após a contratação, o beneficiário pode solicitar adiamento da data de início da visita por até 30 dias, mediante justificativa e autorização. Não será permitida a alteração da instituição de destino da visita técnico-científica após a contratação.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2005_2026%20-%20Visita%20Técnico%20Cientifica%20(1).pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_05_2026_-_VISITA_TÉCNICO-CIENTÍFICA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 308.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 12.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
-?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -1163,70 +854,70 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1236,19 +927,271 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1203,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1268,55 +1211,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
+      <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>US$ 18.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>US$ 6.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1268,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1336,55 +1276,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1330,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1404,281 +1338,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1690,17 +1381,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-28 18:23
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -655,51 +671,121 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Pesquisa</t>
+          <t>Formação Científica</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 28/08/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
+          <t>2026-10-01: Submissão das propostas (até as 17h59)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, focando em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. Seu propósito é criar condições para que o doutor desenvolva uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores que atuem como coordenadores de projetos, sem vínculo empregatício, com título de doutor obtido há no máximo 10 anos, residentes no Espírito Santo, e vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 31.803.200,00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>R$ 400.000,00</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>bolsas.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01: Submissão das propostas (até as 17h59)
+?: Prazo para recurso (seleção) (Até 5 dias úteis após a divulgação do resultado preliminar)
+2027-01-04: Contratação dos projetos</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>As datas e os períodos estabelecidos no cronograma são passíveis de alteração. Cada coordenador deve apresentar apenas uma proposta, caso contrário, ambas serão indeferidas. A convocação de suplentes pode ocorrer em casos de desistência, não contratação ou ampliação de recursos, com validade de 24 meses após o resultado final. O edital pode ser revogado ou anulado por interesse público ou exigência legal, sem gerar direito a indenização.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2022.2026%20-%20PROFIX-CB.pdf</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>formacao_cientifica/EDITAL_FAPES_CNPq_CAPES_No_22_2026_-_PROGRAMA_DE_APOIO_À_FIXAÇÃO_DE_DOUTORES_NO_BRASIL_(PROFIX-CB).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisa</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos visa apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. Seu objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, bem como consolidar grupos de referência em áreas do conhecimento e setores estratégicos do estado.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores doutores, além do coordenador, com representação da Instituição Executora, outras IES/P capixabas, IES/P de fora do estado ou do País, e um pesquisador vinculado a órgão ou instituição pública estadual.</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000.000,00</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>R$ 1.200.000,00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>2026-08-07 a 2026-09-14: Envio da proposta e documentos (via SigFapes, até as 17h59)
 2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
@@ -707,140 +793,212 @@
 2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após o resultado preliminar de análise de mérito)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional. Cada coordenador pode apresentar apenas uma proposta, sendo a última enviada considerada válida em caso de múltiplas submissões. A etapa de habilitação é eliminatória. Serão classificadas apenas as propostas com nota final igual ou superior a 70,0 pontos. Em caso de empate na nota final, o desempate será pela maior nota nos critérios de avaliação (item 3.2.1) na ordem apresentada, e persistindo o empate, pela proposta submetida primeiro. A proposta aprovada não poderá ser alterada no momento da contratação. O projeto aprovado não será contratado se o coordenador não cumprir as condições, apresentar informações falsas ou não atender aos requisitos, resultando na convocação de suplentes. A Fapes não reivindicará direitos de participação na propriedade intelectual sobre as pesquisas e projetos apoiados. É obrigatória a menção clara e destacada do apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto.</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos.pdf</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisa</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 28/08/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>O Edital Fapes n° 24/2026 (PPP-ES) tem como objetivo apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira. Ele visa promover o acesso a recursos para o desenvolvimento de seus primeiros projetos, fortalecer a infraestrutura de pesquisa e apoiar a formação e consolidação de novos grupos de pesquisa no Estado do Espírito Santo. Os projetos devem estar vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, localizadas no Espírito Santo, e contemplar as 8 grandes áreas do conhecimento do CNPq, com duração de até 24 meses.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores em início de carreira, com título obtido a partir de 28/08/2018, que possuam vínculo estatutário ou celetista por tempo indeterminado com uma Instituição de Ensino Superior e/ou de Pesquisa (IES/P) pública ou privada localizada no Espírito Santo, residam no Espírito Santo ou em município limítrofe, e que não tenham atuado como coordenador de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq (com exceções específicas).</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.000.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 180.000,00</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
+2026-08-29 a 2026-09-30: Envio da proposta e documentos (até as 17h59, via SigFapes)
+?: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+?: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2026-12-10: Envio de documentos para contratação (O coordenador receberá informações com prazo e documentação necessária via SigFapes.)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Projetos aprovados terão duração máxima de 24 meses e devem estar enquadrados em uma das 8 grandes áreas do conhecimento do CNPq. A Fapes reserva-se o direito de alterar as datas e prazos do cronograma por necessidade administrativa ou decisão institucional. É fundamental que o coordenador mantenha seus dados cadastrais atualizados no sistema SigFapes para garantir o recebimento das comunicações oficiais. A proposta aprovada não poderá ser alterada no momento da contratação, e a ausência da documentação ética e legal exigida impedirá a contratação do projeto.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
 2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
 ?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 500.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
 2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
@@ -854,70 +1012,158 @@
 ?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 28/08/2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31 a 2026-08-29: Informar dados bancários - 2ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade." → "O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica."</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 800.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>US$ 1.500,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
+2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
+2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59.)
+2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59.)
+2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)
+2026-03-06 a 2026-03-13: Interposição de recursos - 1ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-04-01 a 2026-04-30: Contratação e atualização documental - 1ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-05-01 a 2026-05-30: Informar dados bancários - 1ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
+2026-06-05 a 2026-06-12: Interposição de recursos - 2ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-07-01 a 2026-07-30: Contratação e atualização documental - 2ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-07-31 a 2026-08-29: Informar dados bancários - 2ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
+2026-09-04 a 2026-09-12: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-10-01 a 2026-10-30: Contratação e atualização documental - 3ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-10-31 a 2026-11-29: Informar dados bancários - 3ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
+2026-11-05 a 2026-11-12: Interposição de recursos - 4ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-12-01 a 2026-12-30: Contratação e atualização documental - 4ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -927,211 +1173,19 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1197,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1153,45 +1207,53 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1265,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1211,52 +1273,55 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>US$ 18.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1333,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1280,96 +1345,277 @@
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA ERC-CONFAP 2026</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1381,17 +1627,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-29 12:30
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -39,11 +39,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +54,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -68,9 +63,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -438,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -679,9 +671,9 @@
           <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 28/08/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -820,9 +812,9 @@
           <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 28/08/2026</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1039,9 +1031,9 @@
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 28/08/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1049,11 +1041,7 @@
           <t>2026-07-31 a 2026-08-29: Informar dados bancários - 2ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O objetivo geral deste edital é incentivar a publicação científica e tecnológica no Espírito Santo por meio da concessão de auxílio financeiro para publicação de artigos técnico-científicos. O edital visa apoiar artigos que apresentem resultados de pesquisa desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado, valorizando a produção técnico-científica e ampliando sua visibilidade." → "O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica."</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
@@ -1192,68 +1180,71 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 29/08/2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam fomentar o empreendedorismo inovador. O apoio logístico, gerencial e tecnológico destina-se a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O objetivo é ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Organizações ou instituições incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 4.500.000,00</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 252.000,00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
+2026-08-25 a 2026-09-24: Submissão de propostas (Até as 17h59, via SigFapes)
+?: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
+2026-11-04: Contratação dos projetos selecionados</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: R$ 252.000,00 para Nível Avançado, R$ 192.000,00 para Nível Intermediário e R$ 132.000,00 para Nível Básico. O projeto terá prazo de vigência de 24 meses. É obrigatório destinar no mínimo 20% do valor total dos recursos financeiros solicitados para bolsas. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar as datas do cronograma por necessidade institucional.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1256,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1275,53 +1266,53 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1324,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1341,20 +1332,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1362,22 +1365,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1392,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1397,47 +1400,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1448,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1457,52 +1456,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1514,7 +1508,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1526,96 +1520,161 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1627,17 +1686,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-08-30 12:12
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1038,7 +1030,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31 a 2026-08-29: Informar dados bancários - 2ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
+          <t>2026-09-04 a 2026-09-12: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1188,9 +1180,9 @@
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 29/08/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-01 12:24
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1015,12 +1015,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Difusão do Conhecimento</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1030,120 +1030,36 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04 a 2026-09-12: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar.)</t>
+          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
+          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
+          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>R$ 800.000,00</t>
+          <t>R$ 40.000.000,00</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>US$ 1.500,00</t>
+          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
-2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
-2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59.)
-2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59.)
-2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)
-2026-03-06 a 2026-03-13: Interposição de recursos - 1ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
-2026-04-01 a 2026-04-30: Contratação e atualização documental - 1ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
-2026-05-01 a 2026-05-30: Informar dados bancários - 1ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
-2026-06-05 a 2026-06-12: Interposição de recursos - 2ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
-2026-07-01 a 2026-07-30: Contratação e atualização documental - 2ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
-2026-07-31 a 2026-08-29: Informar dados bancários - 2ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
-2026-09-04 a 2026-09-12: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
-2026-10-01 a 2026-10-30: Contratação e atualização documental - 3ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
-2026-10-31 a 2026-11-29: Informar dados bancários - 3ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
-2026-11-05 a 2026-11-12: Interposição de recursos - 4ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
-2026-12-01 a 2026-12-30: Contratação e atualização documental - 4ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
-2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 40.000.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1153,70 +1069,70 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam fomentar o empreendedorismo inovador. O apoio logístico, gerencial e tecnológico destina-se a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O objetivo é ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Organizações ou instituições incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
 2026-08-25 a 2026-09-24: Submissão de propostas (Até as 17h59, via SigFapes)
@@ -1224,19 +1140,87 @@
 2026-11-04: Contratação dos projetos selecionados</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: R$ 252.000,00 para Nível Avançado, R$ 192.000,00 para Nível Intermediário e R$ 132.000,00 para Nível Básico. O projeto terá prazo de vigência de 24 meses. É obrigatório destinar no mínimo 20% do valor total dos recursos financeiros solicitados para bolsas. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar as datas do cronograma por necessidade institucional.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: R$ 252.000,00 para Nível Avançado, R$ 192.000,00 para Nível Intermediário e R$ 132.000,00 para Nível Básico. O projeto terá prazo de vigência de 24 meses. É obrigatório destinar no mínimo 20% do valor total dos recursos financeiros solicitados para bolsas. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar as datas do cronograma por necessidade institucional.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1232,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1258,53 +1242,53 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1300,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1324,32 +1308,20 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>R$ 150.000,00</t>
-        </is>
-      </c>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1357,22 +1329,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1356,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1392,43 +1364,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1416,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1448,47 +1424,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1481,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1512,48 +1493,45 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1543,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1573,100 +1551,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
+          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
+          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>€ 25.000,00 por ano de projeto</t>
+          <t>EUR 100.000,00</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1678,17 +1594,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-04 11:53
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +59,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -524,25 +540,31 @@
           <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09: Submissão de propostas (Até as 17h59, via Sistema de Gestão da Fapes)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>2026-09-21: Envio da proposta e documentos (até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, tecnologia e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores." → "Selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, desenvolvimento tecnológico e inovação. O programa visa incentivar a participação ativa dos estudantes em pesquisa, promover a popularização da ciência, estimular parcerias entre IES/P e escolas públicas, e contribuir para a formação acadêmica e profissional dos estudantes, com foco na inclusão social e cidadania em comunidades vulneráveis."
+Público-alvo: "Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo." → "Pesquisadores (mínimo mestre, brasileiro ou estrangeiro com residência indeterminada, residente no ES, com vínculo estatutário ou celetista por tempo indeterminado a uma IES/P do ES, sem afastamento e sem parentesco com diretor/tutor da escola parceira) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, que submeterão propostas em parceria com escolas públicas de Educação Básica do Estado do Espírito Santo."
+Submissão (removida): Submissão de propostas — ? a 2026-09-09</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, tecnologia e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores.</t>
+          <t>Selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, desenvolvimento tecnológico e inovação. O programa visa incentivar a participação ativa dos estudantes em pesquisa, promover a popularização da ciência, estimular parcerias entre IES/P e escolas públicas, e contribuir para a formação acadêmica e profissional dos estudantes, com foco na inclusão social e cidadania em comunidades vulneráveis.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo.</t>
+          <t>Pesquisadores (mínimo mestre, brasileiro ou estrangeiro com residência indeterminada, residente no ES, com vínculo estatutário ou celetista por tempo indeterminado a uma IES/P do ES, sem afastamento e sem parentesco com diretor/tutor da escola parceira) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, que submeterão propostas em parceria com escolas públicas de Educação Básica do Estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -562,16 +584,15 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
-2026-09-09: Submissão de propostas (Até as 17h59, via Sistema de Gestão da Fapes)
-?: Prazo para interposição de recursos (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
-?: Prazo para interposição de recursos (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
-2027-02-09: Contratação dos projetos selecionados</t>
+          <t>2026-09-21: Envio da proposta e documentos (até as 17h59)
+2026-10-14: Prazo para recorrer (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
+2027-01-12: Prazo para recorrer (mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2027-02-09: Contratação dos projetos selecionados (A partir de)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Somente as cinco bolsas de Iniciação Científica Júnior (ICJr) são obrigatórias para implementação; as demais modalidades de bolsas (BCO, BTU e ICT) são opcionais. Cada coordenador deve apresentar apenas uma proposta, sendo considerada a última enviada em caso de múltiplas submissões. A Fapes pode alterar datas e prazos do cronograma por necessidade institucional ou reabrir prazos em caso de falhas comprovadas nos sistemas.</t>
+          <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo também reabrir o prazo para recebimento de propostas em casos de força maior ou de falhas comprovadas nas plataformas e sistemas da Fundação.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -596,25 +617,30 @@
           <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>2026-07-31 a 2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "Apoiar projetos de pesquisa que visem contribuir para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil, por meio da concessão de bolsas para estágios de pós-doutorado sênior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica e ampliar a cooperação acadêmica nacional e internacional, em instituições de excelência no país ou no exterior." → "A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior, visando o aprimoramento da qualificação de pesquisadores, ao fortalecimento das atividades de pesquisa científica e tecnológica e à ampliação da cooperação acadêmica nacional e internacional."
+Público-alvo: "Pesquisadores doutores com vínculo formal (mínimo de 20h semanais) em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas, sediadas no estado do Espírito Santo, que sejam docentes permanentes de Programa de Pós-Graduação (PPG) stricto sensu e que atendam aos requisitos de tempo de titulação de doutor (Faixas A, B ou C)." → "Pesquisador com título de doutor, vinculado a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que seja docente permanente de Programa de Pós-Graduação (PPG) stricto sensu de IES/P localizada no Espírito Santo, recomendado pela Capes e, em funcionamento, com as atividades letivas regulares e discentes matriculados."</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos de pesquisa que visem contribuir para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil, por meio da concessão de bolsas para estágios de pós-doutorado sênior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica e ampliar a cooperação acadêmica nacional e internacional, em instituições de excelência no país ou no exterior.</t>
+          <t>A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior, visando o aprimoramento da qualificação de pesquisadores, ao fortalecimento das atividades de pesquisa científica e tecnológica e à ampliação da cooperação acadêmica nacional e internacional.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores com vínculo formal (mínimo de 20h semanais) em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas, sediadas no estado do Espírito Santo, que sejam docentes permanentes de Programa de Pós-Graduação (PPG) stricto sensu e que atendam aos requisitos de tempo de titulação de doutor (Faixas A, B ou C).</t>
+          <t>Pesquisador com título de doutor, vinculado a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que seja docente permanente de Programa de Pós-Graduação (PPG) stricto sensu de IES/P localizada no Espírito Santo, recomendado pela Capes e, em funcionamento, com as atividades letivas regulares e discentes matriculados.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -630,15 +656,16 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes)
-?: Interposição de recursos administrativos (habilitação) (5 dias úteis após a publicação do resultado preliminar de habilitação)
-?: Interposição de recursos administrativos (classificação) (5 dias úteis após a publicação do resultado preliminar de classificação)
-2027-01-18: Contratação das propostas (A partir de)</t>
+          <t>2026-07-31 a 2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)
+2026-09-24: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes.)
+2026-10-10 a 2026-10-14: Prazo para recurso administrativo (habilitação) (5 dias após a publicação do resultado preliminar.)
+2026-12-22 a 2026-12-26: Prazo para recurso administrativo (classificação) (5 dias após a publicação do resultado preliminar.)
+2027-01-18: Contratação das propostas (A partir desta data, com assinatura eletrônica do Termo de Outorga.)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>O prazo de execução do projeto é de 16 meses, improrrogáveis, exceto em caso de Advento de Prole. Cada proponente deve apresentar apenas uma proposta, sendo a última enviada considerada. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. As atividades devem ser realizadas presencialmente na Instituição de Destino, sem pesquisa à distância. Não é permitida a alteração da Instituição de Destino ou do Supervisor após a submissão da proposta. O valor mensal da bolsa de POSDOC varia de acordo com o nível da bolsa e localidade, sendo fixado na Tabela de Valores de Bolsas e Auxílios da Fapes, podendo ser alterado por norma regulamentadora. Os itens financiáveis incluem bolsa mensal (6 a 10 meses), auxílio instalação (equivalente a uma bolsa POSDOC), seguro saúde (limitado a R$ 550,00/mês para exterior) e auxílio deslocamento (limitado a R$ 2.500,00 no país e R$ 12.000,00 no exterior), todos por reembolso, exceto a bolsa mensal e auxílio instalação que podem ser antecipados. A concessão de adaptações, tecnologias assistivas ou outros recursos de acessibilidade é avaliada segundo critérios de viabilidade e razoabilidade, desde que solicitadas em até 10 dias do término de submissão das propostas. O estágio de pós-doutorado deve ter duração mínima de 6 meses e máxima de 10 meses. O proponente deve ser o bolsista POSDOC.</t>
+          <t>Cada Proponente deve apresentar apenas uma proposta. Caso envie mais de uma, apenas a última enviada será considerada. As bolsas não contemplam pesquisa à distância, exigindo atividades presenciais na Instituição de Destino durante toda a vigência da bolsa. O prazo de execução do projeto é de 16 meses, improrrogáveis, exceto em caso de Advento de Prole. Os itens financiáveis incluem bolsa POSDOC mensal (6 a 10 meses), auxílio instalação (equivalente a uma bolsa POSDOC) e auxílio deslocamento (limitado a R$ 2.500,00 para o país ou R$ 12.000,00 para o exterior), além de seguro saúde para o exterior (limitado a R$ 550,00/mês de bolsa). O valor mensal da bolsa POSDOC varia conforme a localidade e é fixado na Tabela de Valores de Bolsas e Auxílios da Fapes.</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -663,25 +690,30 @@
           <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01: Submissão das propostas (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>2026-10-01: Submissão das propostas (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, focando em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. Seu propósito é criar condições para que o doutor desenvolva uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação no Espírito Santo." → "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que doutores estabeleçam e desenvolvam uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas de Ciência, Tecnologia e Inovação (CT&amp;I) do Espírito Santo."
+Público-alvo: "Pesquisadores doutores que atuem como coordenadores de projetos, sem vínculo empregatício, com título de doutor obtido há no máximo 10 anos, residentes no Espírito Santo, e vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq." → "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo."</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, focando em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. Seu propósito é criar condições para que o doutor desenvolva uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação no Espírito Santo.</t>
+          <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que doutores estabeleçam e desenvolvam uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas de Ciência, Tecnologia e Inovação (CT&amp;I) do Espírito Santo.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores que atuem como coordenadores de projetos, sem vínculo empregatício, com título de doutor obtido há no máximo 10 anos, residentes no Espírito Santo, e vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq.</t>
+          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -701,14 +733,14 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01: Submissão das propostas (até as 17h59)
+          <t>2026-10-01: Submissão das propostas (Até as 17h59)
 ?: Prazo para recurso (seleção) (Até 5 dias úteis após a divulgação do resultado preliminar)
-2027-01-04: Contratação dos projetos</t>
+2027-01-04: Contratação dos projetos (A partir de)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>As datas e os períodos estabelecidos no cronograma são passíveis de alteração. Cada coordenador deve apresentar apenas uma proposta, caso contrário, ambas serão indeferidas. A convocação de suplentes pode ocorrer em casos de desistência, não contratação ou ampliação de recursos, com validade de 24 meses após o resultado final. O edital pode ser revogado ou anulado por interesse público ou exigência legal, sem gerar direito a indenização.</t>
+          <t>É permitida a participação do mesmo coordenador em Chamadas Públicas PROFIX-CB promovidas por diferentes Fundações de Amparo à Pesquisa. Entretanto, é vedada sua contratação pela Fapes caso tenha sido contratado no âmbito do Programa PROFIX-CB por Fundação de Amparo à Pesquisa de qualquer outra Unidade da Federação ou do Distrito Federal. Constatada, a qualquer tempo, a contratação do coordenador por outra Fundação de Amparo à Pesquisa no âmbito do Programa PROFIX-CB, sua proposta é eliminada desta Chamada e, caso a concessão pela Fapes já tenha sido implementada, é cancelada, sem prejuízo da comunicação ao CNPq, à Capes e à respectiva Fundação de Amparo à Pesquisa para adoção das providências cabíveis.</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -1015,51 +1047,127 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Extensão</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
+          <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>O edital visa incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCC) com foco em inovação, empreendedorismo e aplicabilidade prática. Serão concedidas Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para propostas que apresentem soluções inovadoras e empreendedoras, com impacto econômico, social e/ou ambiental no Espírito Santo, alinhadas aos ODS da ONU (especialmente 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Podem submeter propostas professores orientadores com vínculo estatutário ou celetista por tempo indeterminado a IES reconhecidas pelo MEC e localizadas no Espírito Santo, que não estejam afastados da IES, estejam adimplentes com a FAPES, residam no ES ou municípios limítrofes, e possuam currículo Lattes atualizado. Cada proponente deve submeter entre 3 e 5 propostas, cada uma vinculada a um único aluno. Se os alunos orientados estiverem vinculados a outra IES, o proponente deve apresentar declaração de autorização de ambas as IES. Os alunos orientados devem ser estudantes regulares de graduação em IES localizadas no Espírito Santo, com desempenho acadêmico igual ou superior a 7.0, adimplentes com a FAPES, com o proponente como professor orientador durante todo o período da bolsa, residência no ES ou municípios limítrofes, e cadastrados no Sigfapes. As IES devem ser públicas ou privadas, localizadas no ES, e prestar anuência às propostas.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.600.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 11.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até as 17h59)
+?: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
+?: Prazo de contratação (Primeira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)
+2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)
+?: Prazo para interposição de recursos administrativos (Segunda Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
+?: Prazo de contratação (Segunda Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)
+2027-02-02 a 2027-03-30: Período de submissão das propostas (Terceira Chamada) (Até as 17h59)
+?: Prazo para interposição de recursos administrativos (Terceira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
+?: Prazo de contratação (Terceira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O edital aceita todos os formatos de TCC definido pelas DCNs, como monografia, dissertação, projeto experimental, relatório técnico ou científico, artigo, plano de negócios e outros. As propostas concorrerão com as demais de suas respectivas microrregiões. Serão apoiados no máximo 20 projetos de TCC por microrregião na primeira chamada, e até 10 projetos de TCC por microrregião nas segunda e terceira chamadas. Recursos financeiros remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Propostas com Nota Final (NF) inferior a 70 pontos serão desclassificadas. Em caso de empate na NF, serão utilizados os critérios de avaliação 1, 2, 3, 4 e 5, nesta ordem, para desempate. Persistindo o empate, será selecionada a proposta submetida primeiro. Não é permitido o acúmulo de bolsas FAPES com outras bolsas, exceto as do Programa Nossa Bolsa, Programa Universidade para Todos (Prouni) e Bolsas de Extensão (Ext-E e Ext-F). O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes (https://fapes.es.gov.br/valores-de-bolsas-e-auxilios) na data de publicação deste edital. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. O orientador receberá até dois auxílios para orientação de TCC: o primeiro após a contratação e o segundo quando pelo menos um aluno orientado apresentar a Ata de Defesa do TCC. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1069,158 +1177,95 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Inovação</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam fomentar o empreendedorismo inovador. O apoio logístico, gerencial e tecnológico destina-se a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O objetivo é ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Organizações ou instituições incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 4.500.000,00</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>R$ 252.000,00</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas)
-2026-08-25 a 2026-09-24: Submissão de propostas (Até as 17h59, via SigFapes)
-?: Interposição de recursos (Até 5 dias úteis após a divulgação do resultado preliminar)
-2026-11-04: Contratação dos projetos selecionados</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>O valor por proposta varia conforme o nível de maturidade da incubadora: R$ 252.000,00 para Nível Avançado, R$ 192.000,00 para Nível Intermediário e R$ 132.000,00 para Nível Básico. O projeto terá prazo de vigência de 24 meses. É obrigatório destinar no mínimo 20% do valor total dos recursos financeiros solicitados para bolsas. Propostas com nota final inferior a 70 pontos serão desclassificadas. A Fapes pode alterar as datas do cronograma por necessidade institucional.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Chamadas Internacionais</t>
+          <t>Inovação</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
+          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 04/09/2026</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam fomentar o empreendedorismo inovador. O apoio logístico, gerencial e tecnológico destina-se a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O objetivo é ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado." → "Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo."
+Público-alvo: "Organizações ou instituições incubadoras, sem fins lucrativos, sediadas no Espírito Santo." → "Incubadoras, sem fins lucrativos, sediadas no Espírito Santo."
+Submissão (removida): Submissão de propostas — 2026-08-25 a 2026-09-24</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 4.500.000,00</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>R$ 252.000,00</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
+2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>Os valores por proposta variam conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é baseada nas seguintes pontuações: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos) e Nível Básico (60 a 75 pontos). Os recursos financeiros remanescentes serão redirecionados para propostas suplentes nos níveis de maturidade I, II e III, nesta ordem, respeitando a classificação. O projeto terá prazo de vigência de 24 meses, sem prorrogação. Mínimo de 20% do valor total solicitado deve ser destinado a bolsas. Parte dos recursos de custeio deve ser destinada à associação à Anprotec. Serão permitidas exclusivamente bolsas na modalidade BPIG, níveis II a X, por no máximo 24 meses.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1277,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1242,53 +1287,53 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1345,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1308,20 +1353,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1329,22 +1386,22 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1413,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1364,47 +1421,43 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1469,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1424,52 +1477,47 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1529,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1493,96 +1541,161 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1594,17 +1707,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-05 10:42
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -39,11 +39,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +54,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -68,9 +63,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -542,7 +534,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+          <t>Atualizado - e-mail enviado em 05/09/2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -552,19 +544,19 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: "O Programa de Iniciação Científica Júnior (PICJr) visa apoiar financeiramente projetos de pesquisa desenvolvidos em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, tecnologia e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores." → "Selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, desenvolvimento tecnológico e inovação. O programa visa incentivar a participação ativa dos estudantes em pesquisa, promover a popularização da ciência, estimular parcerias entre IES/P e escolas públicas, e contribuir para a formação acadêmica e profissional dos estudantes, com foco na inclusão social e cidadania em comunidades vulneráveis."
-Público-alvo: "Pesquisadores (mínimo mestre) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo." → "Pesquisadores (mínimo mestre, brasileiro ou estrangeiro com residência indeterminada, residente no ES, com vínculo estatutário ou celetista por tempo indeterminado a uma IES/P do ES, sem afastamento e sem parentesco com diretor/tutor da escola parceira) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, que submeterão propostas em parceria com escolas públicas de Educação Básica do Estado do Espírito Santo."
-Submissão (removida): Submissão de propostas — ? a 2026-09-09</t>
+          <t>Objetivo: "Selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, desenvolvimento tecnológico e inovação. O programa visa incentivar a participação ativa dos estudantes em pesquisa, promover a popularização da ciência, estimular parcerias entre IES/P e escolas públicas, e contribuir para a formação acadêmica e profissional dos estudantes, com foco na inclusão social e cidadania em comunidades vulneráveis." → "O Programa de Iniciação Científica Júnior (PICJr) da Fapes visa apoiar financeiramente projetos de pesquisa em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, desenvolvimento tecnológico e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores."
+Público-alvo: "Pesquisadores (mínimo mestre, brasileiro ou estrangeiro com residência indeterminada, residente no ES, com vínculo estatutário ou celetista por tempo indeterminado a uma IES/P do ES, sem afastamento e sem parentesco com diretor/tutor da escola parceira) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, que submeterão propostas em parceria com escolas públicas de Educação Básica do Estado do Espírito Santo." → "Pesquisadores com titulação mínima de mestre, brasileiros ou estrangeiros com autorização de residência por prazo indeterminado, vinculados por tempo indeterminado a uma IES/P localizada no Espírito Santo. Os pesquisadores devem estar regularizados junto à Fapes e ter cadastro atualizado na Plataforma Lattes. O programa também envolve professores tutores de escolas parceiras e estudantes da Rede Pública de Educação Básica do Espírito Santo."
+Valor por proposta: "R$ 10.000,00" → "-"</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, desenvolvimento tecnológico e inovação. O programa visa incentivar a participação ativa dos estudantes em pesquisa, promover a popularização da ciência, estimular parcerias entre IES/P e escolas públicas, e contribuir para a formação acadêmica e profissional dos estudantes, com foco na inclusão social e cidadania em comunidades vulneráveis.</t>
+          <t>O Programa de Iniciação Científica Júnior (PICJr) da Fapes visa apoiar financeiramente projetos de pesquisa em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, desenvolvimento tecnológico e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores (mínimo mestre, brasileiro ou estrangeiro com residência indeterminada, residente no ES, com vínculo estatutário ou celetista por tempo indeterminado a uma IES/P do ES, sem afastamento e sem parentesco com diretor/tutor da escola parceira) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, que submeterão propostas em parceria com escolas públicas de Educação Básica do Estado do Espírito Santo.</t>
+          <t>Pesquisadores com titulação mínima de mestre, brasileiros ou estrangeiros com autorização de residência por prazo indeterminado, vinculados por tempo indeterminado a uma IES/P localizada no Espírito Santo. Os pesquisadores devem estar regularizados junto à Fapes e ter cadastro atualizado na Plataforma Lattes. O programa também envolve professores tutores de escolas parceiras e estudantes da Rede Pública de Educação Básica do Espírito Santo.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -572,11 +564,7 @@
           <t>R$ 8.887.500,00</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>R$ 10.000,00</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>bolsas.duvidas@fapes.es.gov.br</t>
@@ -585,19 +573,19 @@
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>2026-09-21: Envio da proposta e documentos (até as 17h59)
-2026-10-14: Prazo para recorrer (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
-2027-01-12: Prazo para recorrer (mérito) (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
-2027-02-09: Contratação dos projetos selecionados (A partir de)</t>
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação)
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2027-02-09: Contratação dos projetos selecionados</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>A Fapes pode alterar as datas e os prazos definidos no cronograma por necessidade ou decisão institucional, podendo também reabrir o prazo para recebimento de propostas em casos de força maior ou de falhas comprovadas nas plataformas e sistemas da Fundação.</t>
+          <t>O edital prevê um auxílio financeiro fixo de R$ 10.000,00 para o coordenador de cada projeto contratado, destinado ao desenvolvimento da pesquisa. Além disso, são concedidas bolsas de estudo, sendo cinco bolsas de Iniciação Científica Júnior (ICJr) obrigatórias para a implementação do projeto, e bolsas de Coordenador (BCO), Tutor (BTU) e Iniciação Científica e Tecnológica (ICT) opcionais, conforme as necessidades do projeto. Os valores mensais das bolsas são definidos em tabela específica da Fapes. As propostas devem ser inéditas para a Fapes, e a fundação pode alterar datas e prazos do cronograma por necessidade institucional ou falhas sistêmicas. A etapa de habilitação é eliminatória.</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/PIC_JR_2027%20-.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Ed.%2019.2026%20PIC%20JR%202027%20-%201ª%20Alteração%20-%20Publicada.pdf</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -617,9 +605,9 @@
           <t>EDITAL FAPES Nº 20/2026 - BOLSAS DE PÓS-DOUTORADO SÊNIOR</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -627,12 +615,7 @@
           <t>2026-07-31 a 2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Apoiar projetos de pesquisa que visem contribuir para o desenvolvimento científico e tecnológico no Espírito Santo e do Brasil, por meio da concessão de bolsas para estágios de pós-doutorado sênior. O objetivo é aprimorar a qualificação de pesquisadores, fortalecer as atividades de pesquisa científica e tecnológica e ampliar a cooperação acadêmica nacional e internacional, em instituições de excelência no país ou no exterior." → "A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior, visando o aprimoramento da qualificação de pesquisadores, ao fortalecimento das atividades de pesquisa científica e tecnológica e à ampliação da cooperação acadêmica nacional e internacional."
-Público-alvo: "Pesquisadores doutores com vínculo formal (mínimo de 20h semanais) em Instituições de Ensino e/ou Pesquisa (IES/P) públicas ou privadas, sediadas no estado do Espírito Santo, que sejam docentes permanentes de Programa de Pós-Graduação (PPG) stricto sensu e que atendam aos requisitos de tempo de titulação de doutor (Faixas A, B ou C)." → "Pesquisador com título de doutor, vinculado a Instituições de Ensino e/ou Pesquisa (IES/P), públicas ou privadas, sediadas no estado do Espírito Santo, que seja docente permanente de Programa de Pós-Graduação (PPG) stricto sensu de IES/P localizada no Espírito Santo, recomendado pela Capes e, em funcionamento, com as atividades letivas regulares e discentes matriculados."</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>A presente chamada pública tem por objetivo selecionar propostas para concessão de bolsas de pós-doutorado sênior, a serem realizadas em instituições de excelência, no país ou no exterior, visando o aprimoramento da qualificação de pesquisadores, ao fortalecimento das atividades de pesquisa científica e tecnológica e à ampliação da cooperação acadêmica nacional e internacional.</t>
@@ -690,9 +673,9 @@
           <t>EDITAL FAPES/CNPq/CAPES Nº 22/2026 - PROGRAMA DE APOIO À FIXAÇÃO DE DOUTORES NO BRASIL (PROFIX-CB)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -700,12 +683,7 @@
           <t>2026-10-01: Submissão das propostas (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país, focando em áreas estratégicas para o desenvolvimento científico, tecnológico e de inovação. Seu propósito é criar condições para que o doutor desenvolva uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação no Espírito Santo." → "O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que doutores estabeleçam e desenvolvam uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas de Ciência, Tecnologia e Inovação (CT&amp;I) do Espírito Santo."
-Público-alvo: "Pesquisadores doutores que atuem como coordenadores de projetos, sem vínculo empregatício, com título de doutor obtido há no máximo 10 anos, residentes no Espírito Santo, e vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo, com registro ativo no Diretório de Instituições do CNPq." → "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) públicas ou privadas localizadas no Espírito Santo."</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>O Programa de Apoio à Fixação de Doutores no Brasil – Conhecimento Brasil (PROFIX-CB) é uma iniciativa do CNPq, CAPES e FAPs para atrair, inserir e fixar pesquisadores doutores em instituições de pesquisa, universidades e centros de inovação no país. Seu propósito é criar condições para que doutores estabeleçam e desenvolvam uma trajetória científica de médio prazo, contribuindo para a formação de recursos humanos, fortalecimento de programas de pós-graduação, consolidação de grupos de pesquisa e geração de conhecimento e inovação, especialmente em áreas estratégicas de Ciência, Tecnologia e Inovação (CT&amp;I) do Espírito Santo.</t>
@@ -1055,9 +1033,9 @@
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 04/09/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1204,9 +1182,9 @@
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 04/09/2026</t>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1214,13 +1192,7 @@
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O edital visa apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, que buscam fomentar o empreendedorismo inovador. O apoio logístico, gerencial e tecnológico destina-se a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O objetivo é ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, promovendo a capacitação de novos empreendedores e o desenvolvimento socioeconômico do estado." → "Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo."
-Público-alvo: "Organizações ou instituições incubadoras, sem fins lucrativos, sediadas no Espírito Santo." → "Incubadoras, sem fins lucrativos, sediadas no Espírito Santo."
-Submissão (removida): Submissão de propostas — 2026-08-25 a 2026-09-24</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
@@ -1477,11 +1449,7 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-06 10:57
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -532,9 +524,9 @@
           <t>EDITAL FAPES Nº 19/2026 - PIC JR 2027</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 05/09/2026</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -542,13 +534,7 @@
           <t>2026-09-21: Envio da proposta e documentos (até as 17h59)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "Selecionar projetos que despertem nos estudantes da Rede Pública de Educação Básica do Espírito Santo o interesse pela ciência, desenvolvimento tecnológico e inovação. O programa visa incentivar a participação ativa dos estudantes em pesquisa, promover a popularização da ciência, estimular parcerias entre IES/P e escolas públicas, e contribuir para a formação acadêmica e profissional dos estudantes, com foco na inclusão social e cidadania em comunidades vulneráveis." → "O Programa de Iniciação Científica Júnior (PICJr) da Fapes visa apoiar financeiramente projetos de pesquisa em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, desenvolvimento tecnológico e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores."
-Público-alvo: "Pesquisadores (mínimo mestre, brasileiro ou estrangeiro com residência indeterminada, residente no ES, com vínculo estatutário ou celetista por tempo indeterminado a uma IES/P do ES, sem afastamento e sem parentesco com diretor/tutor da escola parceira) vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo, que submeterão propostas em parceria com escolas públicas de Educação Básica do Estado do Espírito Santo." → "Pesquisadores com titulação mínima de mestre, brasileiros ou estrangeiros com autorização de residência por prazo indeterminado, vinculados por tempo indeterminado a uma IES/P localizada no Espírito Santo. Os pesquisadores devem estar regularizados junto à Fapes e ter cadastro atualizado na Plataforma Lattes. O programa também envolve professores tutores de escolas parceiras e estudantes da Rede Pública de Educação Básica do Espírito Santo."
-Valor por proposta: "R$ 10.000,00" → "-"</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>O Programa de Iniciação Científica Júnior (PICJr) da Fapes visa apoiar financeiramente projetos de pesquisa em parceria entre escolas públicas de Educação Básica e Instituições de Ensino Superior e/ou de Pesquisa (IES/P) do Espírito Santo. O objetivo geral é despertar nos estudantes da Rede Pública de Educação Básica o interesse pela ciência, desenvolvimento tecnológico e inovação, aproximando-os de práticas científicas sob orientação de pesquisadores e professores tutores.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-09 12:03
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1011,51 +1011,135 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Extensão</t>
+          <t>Difusão do Conhecimento</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)</t>
+          <t>2026-09-04 a 2026-09-12: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar.)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 800.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>US$ 1.500,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
+2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
+2026-03-19 a 2026-05-25: Submissão de propostas - 2ª Chamada (Até as 17h59.)
+2026-06-19 a 2026-08-25: Submissão de propostas - 3ª Chamada (Até as 17h59.)
+2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)
+2026-03-06 a 2026-03-13: Interposição de recursos - 1ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-04-01 a 2026-04-30: Contratação e atualização documental - 1ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-05-01 a 2026-05-30: Informar dados bancários - 1ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
+2026-06-05 a 2026-06-12: Interposição de recursos - 2ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-07-01 a 2026-07-30: Contratação e atualização documental - 2ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-07-31 a 2026-08-29: Informar dados bancários - 2ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
+2026-09-04 a 2026-09-12: Interposição de recursos - 3ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-10-01 a 2026-10-30: Contratação e atualização documental - 3ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-10-31 a 2026-11-29: Informar dados bancários - 3ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)
+2026-11-05 a 2026-11-12: Interposição de recursos - 4ª Chamada (5 dias úteis após a publicação do resultado preliminar.)
+2026-12-01 a 2026-12-30: Contratação e atualização documental - 4ª Chamada (Assinatura do Termo de Outorga. Prazo de até 30 dias após a publicação do resultado final homologado.)
+2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Extensão</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O edital visa incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCC) com foco em inovação, empreendedorismo e aplicabilidade prática. Serão concedidas Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para propostas que apresentem soluções inovadoras e empreendedoras, com impacto econômico, social e/ou ambiental no Espírito Santo, alinhadas aos ODS da ONU (especialmente 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Podem submeter propostas professores orientadores com vínculo estatutário ou celetista por tempo indeterminado a IES reconhecidas pelo MEC e localizadas no Espírito Santo, que não estejam afastados da IES, estejam adimplentes com a FAPES, residam no ES ou municípios limítrofes, e possuam currículo Lattes atualizado. Cada proponente deve submeter entre 3 e 5 propostas, cada uma vinculada a um único aluno. Se os alunos orientados estiverem vinculados a outra IES, o proponente deve apresentar declaração de autorização de ambas as IES. Os alunos orientados devem ser estudantes regulares de graduação em IES localizadas no Espírito Santo, com desempenho acadêmico igual ou superior a 7.0, adimplentes com a FAPES, com o proponente como professor orientador durante todo o período da bolsa, residência no ES ou municípios limítrofes, e cadastrados no Sigfapes. As IES devem ser públicas ou privadas, localizadas no ES, e prestar anuência às propostas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até as 17h59)
 ?: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
@@ -1068,70 +1152,70 @@
 ?: Prazo de contratação (Terceira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital aceita todos os formatos de TCC definido pelas DCNs, como monografia, dissertação, projeto experimental, relatório técnico ou científico, artigo, plano de negócios e outros. As propostas concorrerão com as demais de suas respectivas microrregiões. Serão apoiados no máximo 20 projetos de TCC por microrregião na primeira chamada, e até 10 projetos de TCC por microrregião nas segunda e terceira chamadas. Recursos financeiros remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Propostas com Nota Final (NF) inferior a 70 pontos serão desclassificadas. Em caso de empate na NF, serão utilizados os critérios de avaliação 1, 2, 3, 4 e 5, nesta ordem, para desempate. Persistindo o empate, será selecionada a proposta submetida primeiro. Não é permitido o acúmulo de bolsas FAPES com outras bolsas, exceto as do Programa Nossa Bolsa, Programa Universidade para Todos (Prouni) e Bolsas de Extensão (Ext-E e Ext-F). O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes (https://fapes.es.gov.br/valores-de-bolsas-e-auxilios) na data de publicação deste edital. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. O orientador receberá até dois auxílios para orientação de TCC: o primeiro após a contratação e o segundo quando pelo menos um aluno orientado apresentar a Ata de Defesa do TCC. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1141,157 +1225,89 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)
 ?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os valores por proposta variam conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é baseada nas seguintes pontuações: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos) e Nível Básico (60 a 75 pontos). Os recursos financeiros remanescentes serão redirecionados para propostas suplentes nos níveis de maturidade I, II e III, nesta ordem, respeitando a classificação. O projeto terá prazo de vigência de 24 meses, sem prorrogação. Mínimo de 20% do valor total solicitado deve ser destinado a bolsas. Parte dos recursos de custeio deve ser destinada à associação à Anprotec. Serão permitidas exclusivamente bolsas na modalidade BPIG, níveis II a X, por no máximo 24 meses.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1319,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1313,53 +1329,53 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1387,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1379,20 +1395,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1400,22 +1428,22 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>20